<commit_message>
qa_test: rename Reference Answer, add APAI-Chat Answer column, dark teal headers, clear Validated
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2CBD856-7C14-44B5-9253-4E99573D9CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54751AB4-C440-4F4C-A5DC-7BDF272A032E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="277">
   <si>
     <t>ID</t>
   </si>
@@ -59,9 +59,6 @@
     <t>Difficulty</t>
   </si>
   <si>
-    <t>Reference Answer</t>
-  </si>
-  <si>
     <t>Validated</t>
   </si>
   <si>
@@ -86,9 +83,6 @@
     <t>The variable is $page.rlindex. Under the attributes of the Text Mark, change default 'Text Mark' to $page.rlindex.</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>AP-IMP-002</t>
   </si>
   <si>
@@ -873,6 +867,12 @@
   </si>
   <si>
     <t>Press {: Flip the current view horizontally.</t>
+  </si>
+  <si>
+    <t>Reference Answer (Expected Answer)</t>
+  </si>
+  <si>
+    <t>APAI-Chat Answer</t>
   </si>
 </sst>
 </file>
@@ -905,13 +905,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC47244"/>
+        <fgColor rgb="FFF1E6DC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF1E6DC"/>
+        <fgColor rgb="FF1F6B75"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -930,8 +930,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1266,7 +1266,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2DD8A55-FC28-4FDC-803C-713C907C6695}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
@@ -1275,153 +1275,148 @@
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="164.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="D3" t="s">
         <v>15</v>
       </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" t="s">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="D4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="B5" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="C5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
         <v>23</v>
       </c>
-      <c r="C5" t="s">
+      <c r="F5" t="s">
         <v>24</v>
       </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F5" t="s">
+      <c r="B6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="D6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="2"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1430,7 +1425,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07129D57-73FC-44EA-91A3-D051877B6598}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
@@ -1439,128 +1434,124 @@
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="108.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
         <v>35</v>
       </c>
-      <c r="B3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="B4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="G3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="E4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
         <v>41</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="D5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" t="s">
         <v>42</v>
-      </c>
-      <c r="B5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" t="s">
-        <v>40</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
-        <v>44</v>
-      </c>
-      <c r="G5" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1570,7 +1561,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB492513-0CEA-4027-8146-2D0121182802}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -1579,153 +1570,148 @@
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="83" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>47</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="B3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
         <v>49</v>
       </c>
-      <c r="B3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="B4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="D4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
         <v>54</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" t="s">
         <v>55</v>
       </c>
-      <c r="B5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" t="s">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="B6" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="G5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="D6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="2"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1734,7 +1720,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED61EE79-1B75-41E6-BD8B-15990556690E}">
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
@@ -1743,1397 +1729,1285 @@
     <col min="4" max="4" width="17.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="196.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>64</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="B3" t="s">
         <v>65</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="C3" t="s">
         <v>66</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
         <v>67</v>
       </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="B4" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="G3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="D4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>71</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="B5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" t="s">
         <v>72</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="B5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C5" t="s">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="B6" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="G5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="D6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>77</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="2" t="s">
+      <c r="B7" t="s">
         <v>78</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="C7" t="s">
         <v>79</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
         <v>80</v>
       </c>
-      <c r="C7" t="s">
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="B8" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="G7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="D8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>85</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="2" t="s">
+      <c r="B9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9" t="s">
         <v>86</v>
       </c>
-      <c r="G8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="D9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" t="s">
         <v>87</v>
       </c>
-      <c r="B9" t="s">
-        <v>84</v>
-      </c>
-      <c r="C9" t="s">
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="D9" t="s">
-        <v>17</v>
-      </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="B10" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="G9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="C10" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="D10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>92</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="B11" t="s">
+        <v>89</v>
+      </c>
+      <c r="C11" t="s">
         <v>93</v>
       </c>
-      <c r="G10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="D11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" t="s">
         <v>94</v>
       </c>
-      <c r="B11" t="s">
-        <v>91</v>
-      </c>
-      <c r="C11" t="s">
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D11" t="s">
-        <v>17</v>
-      </c>
-      <c r="E11" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="B12" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="G11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="D12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>98</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F12" s="2" t="s">
+      <c r="B13" t="s">
+        <v>89</v>
+      </c>
+      <c r="C13" t="s">
         <v>99</v>
       </c>
-      <c r="G12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="D13" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" t="s">
         <v>100</v>
       </c>
-      <c r="B13" t="s">
-        <v>91</v>
-      </c>
-      <c r="C13" t="s">
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
-        <v>25</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="B14" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="G13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="C14" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="D14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>105</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" s="2" t="s">
+      <c r="B15" t="s">
+        <v>102</v>
+      </c>
+      <c r="C15" t="s">
         <v>106</v>
       </c>
-      <c r="G14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H14" s="2"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="D15" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" t="s">
         <v>107</v>
       </c>
-      <c r="B15" t="s">
-        <v>104</v>
-      </c>
-      <c r="C15" t="s">
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="D15" t="s">
-        <v>17</v>
-      </c>
-      <c r="E15" t="s">
-        <v>12</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="B16" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="G15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+      <c r="D16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C16" s="2" t="s">
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>111</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F16" s="2" t="s">
+      <c r="B17" t="s">
         <v>112</v>
       </c>
-      <c r="G16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H16" s="2"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="C17" t="s">
         <v>113</v>
       </c>
-      <c r="B17" t="s">
+      <c r="D17" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" t="s">
         <v>114</v>
       </c>
-      <c r="C17" t="s">
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" t="s">
-        <v>12</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="B18" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="G17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+      <c r="D18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C18" s="2" t="s">
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>118</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F18" s="2" t="s">
+      <c r="B19" t="s">
         <v>119</v>
       </c>
-      <c r="G18" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H18" s="2"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="C19" t="s">
         <v>120</v>
       </c>
-      <c r="B19" t="s">
+      <c r="D19" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" t="s">
         <v>121</v>
       </c>
-      <c r="C19" t="s">
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D19" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" t="s">
-        <v>12</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="B20" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="G19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
+      <c r="C20" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="D20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>126</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F20" s="2" t="s">
+      <c r="B21" t="s">
+        <v>123</v>
+      </c>
+      <c r="C21" t="s">
         <v>127</v>
       </c>
-      <c r="G20" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H20" s="2"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="D21" t="s">
         <v>128</v>
       </c>
-      <c r="B21" t="s">
-        <v>125</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="E21" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21" t="s">
         <v>129</v>
       </c>
-      <c r="D21" t="s">
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E21" t="s">
-        <v>25</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="B22" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="G21" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
+      <c r="D22" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C22" s="2" t="s">
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>133</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F22" s="2" t="s">
+      <c r="B23" t="s">
         <v>134</v>
       </c>
-      <c r="G22" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="C23" t="s">
         <v>135</v>
       </c>
-      <c r="B23" t="s">
+      <c r="D23" t="s">
         <v>136</v>
       </c>
-      <c r="C23" t="s">
+      <c r="E23" t="s">
+        <v>23</v>
+      </c>
+      <c r="F23" t="s">
         <v>137</v>
       </c>
-      <c r="D23" t="s">
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="E23" t="s">
-        <v>25</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="B24" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="G23" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
+      <c r="C24" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="D24" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>142</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F24" s="2" t="s">
+      <c r="B25" t="s">
         <v>143</v>
       </c>
-      <c r="G24" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H24" s="2"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="C25" t="s">
         <v>144</v>
       </c>
-      <c r="B25" t="s">
+      <c r="D25" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" t="s">
+        <v>23</v>
+      </c>
+      <c r="F25" t="s">
         <v>145</v>
       </c>
-      <c r="C25" t="s">
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D25" t="s">
-        <v>11</v>
-      </c>
-      <c r="E25" t="s">
-        <v>25</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="B26" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="G25" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
+      <c r="C26" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="D26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
         <v>150</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F26" s="2" t="s">
+      <c r="B27" t="s">
         <v>151</v>
       </c>
-      <c r="G26" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H26" s="2"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+      <c r="C27" t="s">
         <v>152</v>
       </c>
-      <c r="B27" t="s">
+      <c r="D27" t="s">
+        <v>128</v>
+      </c>
+      <c r="E27" t="s">
+        <v>23</v>
+      </c>
+      <c r="F27" t="s">
         <v>153</v>
       </c>
-      <c r="C27" t="s">
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="D27" t="s">
-        <v>130</v>
-      </c>
-      <c r="E27" t="s">
-        <v>25</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="B28" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="G27" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
+      <c r="C28" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="D28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
         <v>158</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F28" s="2" t="s">
+      <c r="B29" t="s">
         <v>159</v>
       </c>
-      <c r="G28" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H28" s="2"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+      <c r="C29" t="s">
         <v>160</v>
       </c>
-      <c r="B29" t="s">
+      <c r="D29" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" t="s">
         <v>161</v>
       </c>
-      <c r="C29" t="s">
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="D29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E29" t="s">
-        <v>12</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="B30" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="G29" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A30" s="2" t="s">
+      <c r="C30" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="D30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
         <v>166</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F30" s="2" t="s">
+      <c r="B31" t="s">
+        <v>159</v>
+      </c>
+      <c r="C31" t="s">
         <v>167</v>
       </c>
-      <c r="G30" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H30" s="2"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
+      <c r="D31" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" t="s">
+        <v>23</v>
+      </c>
+      <c r="F31" t="s">
         <v>168</v>
       </c>
-      <c r="B31" t="s">
-        <v>161</v>
-      </c>
-      <c r="C31" t="s">
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="D31" t="s">
-        <v>11</v>
-      </c>
-      <c r="E31" t="s">
-        <v>25</v>
-      </c>
-      <c r="F31" t="s">
+      <c r="B32" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="G31" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
+      <c r="C32" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="D32" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F32" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
         <v>173</v>
       </c>
-      <c r="D32" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F32" s="2" t="s">
+      <c r="B33" t="s">
         <v>174</v>
       </c>
-      <c r="G32" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H32" s="2"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
+      <c r="C33" t="s">
         <v>175</v>
       </c>
-      <c r="B33" t="s">
+      <c r="D33" t="s">
+        <v>10</v>
+      </c>
+      <c r="E33" t="s">
         <v>176</v>
       </c>
-      <c r="C33" t="s">
+      <c r="F33" t="s">
         <v>177</v>
       </c>
-      <c r="D33" t="s">
-        <v>11</v>
-      </c>
-      <c r="E33" t="s">
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="F33" t="s">
+      <c r="B34" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="G33" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
+      <c r="C34" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="D34" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
         <v>182</v>
       </c>
-      <c r="D34" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F34" s="2" t="s">
+      <c r="B35" t="s">
         <v>183</v>
       </c>
-      <c r="G34" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H34" s="2"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
+      <c r="C35" t="s">
         <v>184</v>
       </c>
-      <c r="B35" t="s">
+      <c r="D35" t="s">
+        <v>10</v>
+      </c>
+      <c r="E35" t="s">
+        <v>23</v>
+      </c>
+      <c r="F35" t="s">
         <v>185</v>
       </c>
-      <c r="C35" t="s">
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="D35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E35" t="s">
-        <v>25</v>
-      </c>
-      <c r="F35" t="s">
+      <c r="B36" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G35" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36" s="2" t="s">
+      <c r="D36" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F36" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="C36" s="2" t="s">
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
         <v>189</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F36" s="2" t="s">
+      <c r="B37" t="s">
         <v>190</v>
       </c>
-      <c r="G36" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H36" s="2"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
+      <c r="C37" t="s">
         <v>191</v>
       </c>
-      <c r="B37" t="s">
+      <c r="D37" t="s">
+        <v>15</v>
+      </c>
+      <c r="E37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F37" t="s">
         <v>192</v>
       </c>
-      <c r="C37" t="s">
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="D37" t="s">
-        <v>17</v>
-      </c>
-      <c r="E37" t="s">
-        <v>12</v>
-      </c>
-      <c r="F37" t="s">
+      <c r="B38" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="G37" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
+      <c r="C38" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="D38" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F38" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
         <v>197</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F38" s="2" t="s">
+      <c r="B39" t="s">
         <v>198</v>
       </c>
-      <c r="G38" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H38" s="2"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
+      <c r="C39" t="s">
         <v>199</v>
       </c>
-      <c r="B39" t="s">
+      <c r="D39" t="s">
+        <v>10</v>
+      </c>
+      <c r="E39" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" t="s">
         <v>200</v>
       </c>
-      <c r="C39" t="s">
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="D39" t="s">
-        <v>11</v>
-      </c>
-      <c r="E39" t="s">
-        <v>12</v>
-      </c>
-      <c r="F39" t="s">
+      <c r="B40" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="G39" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A40" s="2" t="s">
+      <c r="C40" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="D40" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
         <v>205</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F40" s="2" t="s">
+      <c r="B41" t="s">
         <v>206</v>
       </c>
-      <c r="G40" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H40" s="2"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
+      <c r="C41" t="s">
         <v>207</v>
       </c>
-      <c r="B41" t="s">
+      <c r="D41" t="s">
+        <v>10</v>
+      </c>
+      <c r="E41" t="s">
+        <v>23</v>
+      </c>
+      <c r="F41" t="s">
         <v>208</v>
       </c>
-      <c r="C41" t="s">
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="D41" t="s">
-        <v>11</v>
-      </c>
-      <c r="E41" t="s">
-        <v>25</v>
-      </c>
-      <c r="F41" t="s">
+      <c r="B42" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="G41" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A42" s="2" t="s">
+      <c r="C42" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="D42" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="G42" s="1"/>
+      <c r="H42" s="1"/>
+      <c r="I42" s="1"/>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
         <v>213</v>
       </c>
-      <c r="D42" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F42" s="2" t="s">
+      <c r="B43" t="s">
+        <v>210</v>
+      </c>
+      <c r="C43" t="s">
         <v>214</v>
       </c>
-      <c r="G42" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H42" s="2"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
+      <c r="D43" t="s">
+        <v>10</v>
+      </c>
+      <c r="E43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F43" t="s">
         <v>215</v>
       </c>
-      <c r="B43" t="s">
-        <v>212</v>
-      </c>
-      <c r="C43" t="s">
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="D43" t="s">
-        <v>11</v>
-      </c>
-      <c r="E43" t="s">
-        <v>25</v>
-      </c>
-      <c r="F43" t="s">
+      <c r="B44" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="G43" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A44" s="2" t="s">
+      <c r="C44" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="D44" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="G44" s="1"/>
+      <c r="H44" s="1"/>
+      <c r="I44" s="1"/>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
         <v>220</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F44" s="2" t="s">
+      <c r="B45" t="s">
         <v>221</v>
       </c>
-      <c r="G44" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H44" s="2"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
+      <c r="C45" t="s">
         <v>222</v>
       </c>
-      <c r="B45" t="s">
+      <c r="D45" t="s">
+        <v>128</v>
+      </c>
+      <c r="E45" t="s">
+        <v>11</v>
+      </c>
+      <c r="F45" t="s">
         <v>223</v>
       </c>
-      <c r="C45" t="s">
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="D45" t="s">
-        <v>130</v>
-      </c>
-      <c r="E45" t="s">
-        <v>12</v>
-      </c>
-      <c r="F45" t="s">
+      <c r="B46" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C46" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="G45" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
+      <c r="D46" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="C46" s="2" t="s">
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+      <c r="I46" s="1"/>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
         <v>227</v>
       </c>
-      <c r="D46" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F46" s="2" t="s">
+      <c r="B47" t="s">
         <v>228</v>
       </c>
-      <c r="G46" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H46" s="2"/>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
+      <c r="C47" t="s">
         <v>229</v>
       </c>
-      <c r="B47" t="s">
+      <c r="D47" t="s">
+        <v>136</v>
+      </c>
+      <c r="E47" t="s">
+        <v>176</v>
+      </c>
+      <c r="F47" t="s">
         <v>230</v>
       </c>
-      <c r="C47" t="s">
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="D47" t="s">
-        <v>138</v>
-      </c>
-      <c r="E47" t="s">
-        <v>178</v>
-      </c>
-      <c r="F47" t="s">
+      <c r="B48" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="G47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A48" s="2" t="s">
+      <c r="C48" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="D48" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F48" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+      <c r="I48" s="1"/>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
         <v>235</v>
       </c>
-      <c r="D48" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="F48" s="2" t="s">
+      <c r="B49" t="s">
+        <v>232</v>
+      </c>
+      <c r="C49" t="s">
         <v>236</v>
       </c>
-      <c r="G48" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H48" s="2"/>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
+      <c r="D49" t="s">
+        <v>10</v>
+      </c>
+      <c r="E49" t="s">
+        <v>23</v>
+      </c>
+      <c r="F49" t="s">
         <v>237</v>
       </c>
-      <c r="B49" t="s">
-        <v>234</v>
-      </c>
-      <c r="C49" t="s">
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="D49" t="s">
-        <v>11</v>
-      </c>
-      <c r="E49" t="s">
-        <v>25</v>
-      </c>
-      <c r="F49" t="s">
+      <c r="B50" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="G49" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A50" s="2" t="s">
+      <c r="C50" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="D50" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F50" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="C50" s="2" t="s">
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+      <c r="I50" s="1"/>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
         <v>242</v>
       </c>
-      <c r="D50" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F50" s="2" t="s">
+      <c r="B51" t="s">
         <v>243</v>
       </c>
-      <c r="G50" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H50" s="2"/>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
+      <c r="C51" t="s">
         <v>244</v>
       </c>
-      <c r="B51" t="s">
+      <c r="D51" t="s">
+        <v>15</v>
+      </c>
+      <c r="E51" t="s">
+        <v>11</v>
+      </c>
+      <c r="F51" t="s">
         <v>245</v>
       </c>
-      <c r="C51" t="s">
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="D51" t="s">
-        <v>17</v>
-      </c>
-      <c r="E51" t="s">
-        <v>12</v>
-      </c>
-      <c r="F51" t="s">
+      <c r="B52" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="G51" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A52" s="2" t="s">
+      <c r="C52" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="D52" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F52" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="C52" s="2" t="s">
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+      <c r="I52" s="1"/>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
         <v>250</v>
       </c>
-      <c r="D52" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F52" s="2" t="s">
+      <c r="B53" t="s">
+        <v>247</v>
+      </c>
+      <c r="C53" t="s">
         <v>251</v>
       </c>
-      <c r="G52" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H52" s="2"/>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
+      <c r="D53" t="s">
+        <v>10</v>
+      </c>
+      <c r="E53" t="s">
+        <v>23</v>
+      </c>
+      <c r="F53" t="s">
         <v>252</v>
       </c>
-      <c r="B53" t="s">
-        <v>249</v>
-      </c>
-      <c r="C53" t="s">
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A54" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="D53" t="s">
-        <v>11</v>
-      </c>
-      <c r="E53" t="s">
-        <v>25</v>
-      </c>
-      <c r="F53" t="s">
+      <c r="B54" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="G53" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A54" s="2" t="s">
+      <c r="C54" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="D54" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F54" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="G54" s="1"/>
+      <c r="H54" s="1"/>
+      <c r="I54" s="1"/>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
         <v>257</v>
       </c>
-      <c r="D54" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F54" s="2" t="s">
+      <c r="B55" t="s">
         <v>258</v>
       </c>
-      <c r="G54" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H54" s="2"/>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
+      <c r="C55" t="s">
         <v>259</v>
       </c>
-      <c r="B55" t="s">
+      <c r="D55" t="s">
+        <v>10</v>
+      </c>
+      <c r="E55" t="s">
+        <v>23</v>
+      </c>
+      <c r="F55" t="s">
         <v>260</v>
       </c>
-      <c r="C55" t="s">
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="D55" t="s">
-        <v>11</v>
-      </c>
-      <c r="E55" t="s">
-        <v>25</v>
-      </c>
-      <c r="F55" t="s">
+      <c r="B56" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="G55" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A56" s="2" t="s">
+      <c r="C56" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="D56" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="C56" s="2" t="s">
+      <c r="G56" s="1"/>
+      <c r="H56" s="1"/>
+      <c r="I56" s="1"/>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
         <v>265</v>
       </c>
-      <c r="D56" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F56" s="2" t="s">
+      <c r="B57" t="s">
+        <v>262</v>
+      </c>
+      <c r="C57" t="s">
         <v>266</v>
       </c>
-      <c r="G56" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H56" s="2"/>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
+      <c r="D57" t="s">
+        <v>10</v>
+      </c>
+      <c r="E57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F57" t="s">
         <v>267</v>
       </c>
-      <c r="B57" t="s">
-        <v>264</v>
-      </c>
-      <c r="C57" t="s">
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A58" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="D57" t="s">
-        <v>11</v>
-      </c>
-      <c r="E57" t="s">
-        <v>12</v>
-      </c>
-      <c r="F57" t="s">
+      <c r="B58" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="G57" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A58" s="2" t="s">
+      <c r="C58" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="D58" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F58" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="C58" s="2" t="s">
+      <c r="G58" s="1"/>
+      <c r="H58" s="1"/>
+      <c r="I58" s="1"/>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
         <v>272</v>
       </c>
-      <c r="D58" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F58" s="2" t="s">
+      <c r="B59" t="s">
+        <v>269</v>
+      </c>
+      <c r="C59" t="s">
         <v>273</v>
       </c>
-      <c r="G58" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H58" s="2"/>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
+      <c r="D59" t="s">
+        <v>38</v>
+      </c>
+      <c r="E59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F59" t="s">
         <v>274</v>
-      </c>
-      <c r="B59" t="s">
-        <v>271</v>
-      </c>
-      <c r="C59" t="s">
-        <v>275</v>
-      </c>
-      <c r="D59" t="s">
-        <v>40</v>
-      </c>
-      <c r="E59" t="s">
-        <v>12</v>
-      </c>
-      <c r="F59" t="s">
-        <v>276</v>
-      </c>
-      <c r="G59" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
qa_test: reorder Validated columns, fill source Validated=Yes, new styling with teal header + light gray stripes
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54751AB4-C440-4F4C-A5DC-7BDF272A032E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CEEC262-F0E9-4A0D-8979-7C5D3889DC0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="278">
   <si>
     <t>ID</t>
   </si>
@@ -873,6 +873,9 @@
   </si>
   <si>
     <t>APAI-Chat Answer</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -905,18 +908,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF1E6DC"/>
+        <fgColor rgb="FF1F6B75"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F6B75"/>
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -924,14 +927,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1266,7 +1285,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2DD8A55-FC28-4FDC-803C-713C907C6695}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
@@ -1275,148 +1294,173 @@
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="164.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="D2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="G2" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="E3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="G3" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="E4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="G4" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="G5" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="1" t="s">
+      <c r="D6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
+      <c r="G6" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1425,7 +1469,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07129D57-73FC-44EA-91A3-D051877B6598}">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
@@ -1434,125 +1478,147 @@
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="108.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="D2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="G2" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="3" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="G3" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="G4" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="E5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>42</v>
       </c>
+      <c r="G5" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1561,7 +1627,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB492513-0CEA-4027-8146-2D0121182802}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -1570,148 +1636,173 @@
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="83" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="D2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="G2" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="E3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="G3" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="1" t="s">
+      <c r="D4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="G4" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="3" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="G5" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="1" t="s">
+      <c r="E6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
+      <c r="G6" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1720,7 +1811,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED61EE79-1B75-41E6-BD8B-15990556690E}">
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
@@ -1729,1286 +1820,1551 @@
     <col min="4" max="4" width="17.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="196.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="D2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="G2" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="G3" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="D4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="G4" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="D5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="G5" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="1" t="s">
+      <c r="D6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="G6" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="E7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="G7" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="1" t="s">
+      <c r="E8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="G8" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="E9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+      <c r="G9" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="1" t="s">
+      <c r="D10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="G10" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E11" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="E11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="G11" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="G12" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="D13" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="D13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="3" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+      <c r="G13" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="1" t="s">
+      <c r="D14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="G14" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E15" t="s">
-        <v>11</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="E15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
+      <c r="G15" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F16" s="1" t="s">
+      <c r="E16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="G16" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D17" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="D17" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+      <c r="G17" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="F18" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="G18" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="D19" t="s">
-        <v>10</v>
-      </c>
-      <c r="E19" t="s">
-        <v>11</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="D19" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
+      <c r="G19" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F20" s="1" t="s">
+      <c r="D20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="G20" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="3" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
+      <c r="G21" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F22" s="1" t="s">
+      <c r="E22" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="G22" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="3" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
+      <c r="G23" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D24" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E24" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F24" s="1" t="s">
+      <c r="E24" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="G24" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="D25" t="s">
-        <v>10</v>
-      </c>
-      <c r="E25" t="s">
+      <c r="D25" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="3" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
+      <c r="G25" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F26" s="1" t="s">
+      <c r="D26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+      <c r="G26" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="3" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
+      <c r="G27" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D28" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F28" s="1" t="s">
+      <c r="E28" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+      <c r="G28" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="D29" t="s">
-        <v>10</v>
-      </c>
-      <c r="E29" t="s">
-        <v>11</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="D29" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" s="3" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
+      <c r="G29" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="D30" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F30" s="1" t="s">
+      <c r="D30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
+      <c r="G30" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="D31" t="s">
-        <v>10</v>
-      </c>
-      <c r="E31" t="s">
+      <c r="D31" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="3" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
+      <c r="G31" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C32" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="D32" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E32" s="1" t="s">
+      <c r="D32" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="F32" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="G32" s="1"/>
-      <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
+      <c r="G32" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A33" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="D33" t="s">
-        <v>10</v>
-      </c>
-      <c r="E33" t="s">
+      <c r="D33" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" s="3" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
+      <c r="G33" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="D34" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F34" s="1" t="s">
+      <c r="D34" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="G34" s="1"/>
-      <c r="H34" s="1"/>
-      <c r="I34" s="1"/>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
+      <c r="G34" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A35" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D35" t="s">
-        <v>10</v>
-      </c>
-      <c r="E35" t="s">
+      <c r="D35" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E35" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35" s="3" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
+      <c r="G35" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="D36" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="E36" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="F36" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
-      <c r="I36" s="1"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
+      <c r="G36" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A37" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E37" t="s">
-        <v>11</v>
-      </c>
-      <c r="F37" t="s">
+      <c r="E37" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F37" s="3" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A38" s="1" t="s">
+      <c r="G37" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C38" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D38" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="E38" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F38" s="1" t="s">
+      <c r="F38" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="G38" s="1"/>
-      <c r="H38" s="1"/>
-      <c r="I38" s="1"/>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
+      <c r="G38" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="2"/>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A39" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="D39" t="s">
-        <v>10</v>
-      </c>
-      <c r="E39" t="s">
-        <v>11</v>
-      </c>
-      <c r="F39" t="s">
+      <c r="D39" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" s="3" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" s="1" t="s">
+      <c r="G39" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H39" s="3"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="D40" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E40" s="1" t="s">
+      <c r="D40" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E40" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="F40" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="G40" s="1"/>
-      <c r="H40" s="1"/>
-      <c r="I40" s="1"/>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
+      <c r="G40" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+      <c r="J40" s="2"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A41" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="D41" t="s">
-        <v>10</v>
-      </c>
-      <c r="E41" t="s">
+      <c r="D41" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E41" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F41" s="3" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
+      <c r="G41" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H41" s="3"/>
+      <c r="I41" s="3"/>
+      <c r="J41" s="3"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="D42" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F42" s="1" t="s">
+      <c r="D42" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="G42" s="1"/>
-      <c r="H42" s="1"/>
-      <c r="I42" s="1"/>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
+      <c r="G42" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H42" s="2"/>
+      <c r="I42" s="2"/>
+      <c r="J42" s="2"/>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A43" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="D43" t="s">
-        <v>10</v>
-      </c>
-      <c r="E43" t="s">
+      <c r="D43" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E43" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F43" t="s">
+      <c r="F43" s="3" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A44" s="1" t="s">
+      <c r="G43" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B44" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C44" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="D44" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F44" s="1" t="s">
+      <c r="D44" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="G44" s="1"/>
-      <c r="H44" s="1"/>
-      <c r="I44" s="1"/>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
+      <c r="G44" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H44" s="2"/>
+      <c r="I44" s="2"/>
+      <c r="J44" s="2"/>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A45" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C45" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D45" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E45" t="s">
-        <v>11</v>
-      </c>
-      <c r="F45" t="s">
+      <c r="E45" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F45" s="3" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="1" t="s">
+      <c r="G45" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="C46" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="D46" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E46" s="1" t="s">
+      <c r="D46" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E46" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="F46" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="G46" s="1"/>
-      <c r="H46" s="1"/>
-      <c r="I46" s="1"/>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
+      <c r="G46" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H46" s="2"/>
+      <c r="I46" s="2"/>
+      <c r="J46" s="2"/>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A47" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C47" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D47" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="E47" t="s">
+      <c r="E47" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="F47" t="s">
+      <c r="F47" s="3" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A48" s="1" t="s">
+      <c r="G47" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="C48" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="D48" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E48" s="1" t="s">
+      <c r="D48" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E48" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="F48" s="1" t="s">
+      <c r="F48" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="G48" s="1"/>
-      <c r="H48" s="1"/>
-      <c r="I48" s="1"/>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
+      <c r="G48" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H48" s="2"/>
+      <c r="I48" s="2"/>
+      <c r="J48" s="2"/>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A49" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C49" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="D49" t="s">
-        <v>10</v>
-      </c>
-      <c r="E49" t="s">
+      <c r="D49" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E49" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F49" s="3" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A50" s="1" t="s">
+      <c r="G49" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3"/>
+      <c r="J49" s="3"/>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="C50" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="D50" s="1" t="s">
+      <c r="D50" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E50" s="1" t="s">
+      <c r="E50" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F50" s="1" t="s">
+      <c r="F50" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="G50" s="1"/>
-      <c r="H50" s="1"/>
-      <c r="I50" s="1"/>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
+      <c r="G50" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H50" s="2"/>
+      <c r="I50" s="2"/>
+      <c r="J50" s="2"/>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A51" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C51" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D51" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E51" t="s">
-        <v>11</v>
-      </c>
-      <c r="F51" t="s">
+      <c r="E51" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F51" s="3" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A52" s="1" t="s">
+      <c r="G51" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="3"/>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="C52" s="1" t="s">
+      <c r="C52" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="D52" s="1" t="s">
+      <c r="D52" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E52" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F52" s="1" t="s">
+      <c r="E52" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F52" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="G52" s="1"/>
-      <c r="H52" s="1"/>
-      <c r="I52" s="1"/>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
+      <c r="G52" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H52" s="2"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="2"/>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A53" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C53" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="D53" t="s">
-        <v>10</v>
-      </c>
-      <c r="E53" t="s">
+      <c r="D53" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E53" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F53" t="s">
+      <c r="F53" s="3" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A54" s="1" t="s">
+      <c r="G53" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H53" s="3"/>
+      <c r="I53" s="3"/>
+      <c r="J53" s="3"/>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A54" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B54" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="C54" s="1" t="s">
+      <c r="C54" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D54" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F54" s="1" t="s">
+      <c r="D54" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F54" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="G54" s="1"/>
-      <c r="H54" s="1"/>
-      <c r="I54" s="1"/>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
+      <c r="G54" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H54" s="2"/>
+      <c r="I54" s="2"/>
+      <c r="J54" s="2"/>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A55" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B55" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="C55" t="s">
+      <c r="C55" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="D55" t="s">
-        <v>10</v>
-      </c>
-      <c r="E55" t="s">
+      <c r="D55" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E55" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F55" t="s">
+      <c r="F55" s="3" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A56" s="1" t="s">
+      <c r="G55" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H55" s="3"/>
+      <c r="I55" s="3"/>
+      <c r="J55" s="3"/>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A56" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="C56" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="D56" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F56" s="1" t="s">
+      <c r="D56" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F56" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="G56" s="1"/>
-      <c r="H56" s="1"/>
-      <c r="I56" s="1"/>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
+      <c r="G56" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H56" s="2"/>
+      <c r="I56" s="2"/>
+      <c r="J56" s="2"/>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A57" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C57" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="D57" t="s">
-        <v>10</v>
-      </c>
-      <c r="E57" t="s">
-        <v>11</v>
-      </c>
-      <c r="F57" t="s">
+      <c r="D57" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F57" s="3" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A58" s="1" t="s">
+      <c r="G57" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H57" s="3"/>
+      <c r="I57" s="3"/>
+      <c r="J57" s="3"/>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A58" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="C58" s="1" t="s">
+      <c r="C58" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="D58" s="1" t="s">
+      <c r="D58" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E58" s="1" t="s">
+      <c r="E58" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F58" s="1" t="s">
+      <c r="F58" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="G58" s="1"/>
-      <c r="H58" s="1"/>
-      <c r="I58" s="1"/>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
+      <c r="G58" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H58" s="2"/>
+      <c r="I58" s="2"/>
+      <c r="J58" s="2"/>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A59" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="C59" t="s">
+      <c r="C59" s="3" t="s">
         <v>273</v>
       </c>
-      <c r="D59" t="s">
+      <c r="D59" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E59" t="s">
-        <v>11</v>
-      </c>
-      <c r="F59" t="s">
+      <c r="E59" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F59" s="3" t="s">
         <v>274</v>
       </c>
+      <c r="G59" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H59" s="3"/>
+      <c r="I59" s="3"/>
+      <c r="J59" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
qa_test: rename Validated columns to Validated (Source) and Validated (APAI)
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CEEC262-F0E9-4A0D-8979-7C5D3889DC0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DF9FA4C-1FBA-4936-9588-46D05B825D78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="279">
   <si>
     <t>ID</t>
   </si>
@@ -59,9 +59,6 @@
     <t>Difficulty</t>
   </si>
   <si>
-    <t>Validated</t>
-  </si>
-  <si>
     <t>Pass / Fail</t>
   </si>
   <si>
@@ -876,6 +873,12 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>Validated (Source)</t>
+  </si>
+  <si>
+    <t>Validated (APAI)</t>
   </si>
 </sst>
 </file>
@@ -950,7 +953,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1317,42 +1320,42 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G2" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
@@ -1360,25 +1363,25 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
@@ -1386,25 +1389,25 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="G4" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -1412,25 +1415,25 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -1438,25 +1441,25 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="G6" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -1501,42 +1504,42 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="G2" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
@@ -1544,25 +1547,25 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>35</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
@@ -1570,25 +1573,25 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>39</v>
-      </c>
       <c r="G4" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -1596,25 +1599,25 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>42</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -1659,42 +1662,42 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>46</v>
-      </c>
       <c r="G2" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
@@ -1702,25 +1705,25 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>49</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
@@ -1728,25 +1731,25 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="G4" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -1754,25 +1757,25 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>55</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -1780,25 +1783,25 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="G6" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -1843,42 +1846,42 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="G2" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
@@ -1886,25 +1889,25 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>67</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
@@ -1912,25 +1915,25 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="G4" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -1938,25 +1941,25 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>73</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -1964,25 +1967,25 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>76</v>
-      </c>
       <c r="G6" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -1990,25 +1993,25 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="G7" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -2016,25 +2019,25 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>84</v>
-      </c>
       <c r="G8" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -2042,25 +2045,25 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>87</v>
-      </c>
       <c r="G9" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
@@ -2068,25 +2071,25 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>91</v>
-      </c>
       <c r="G10" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
@@ -2094,25 +2097,25 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>94</v>
-      </c>
       <c r="G11" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -2120,25 +2123,25 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="G12" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -2146,25 +2149,25 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>100</v>
-      </c>
       <c r="G13" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
@@ -2172,25 +2175,25 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="G14" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
@@ -2198,25 +2201,25 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>107</v>
-      </c>
       <c r="G15" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
@@ -2224,25 +2227,25 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>110</v>
-      </c>
       <c r="G16" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
@@ -2250,25 +2253,25 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="C17" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>114</v>
-      </c>
       <c r="G17" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
@@ -2276,25 +2279,25 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>117</v>
-      </c>
       <c r="G18" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
@@ -2302,25 +2305,25 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="D19" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>121</v>
-      </c>
       <c r="G19" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
@@ -2328,25 +2331,25 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>125</v>
-      </c>
       <c r="G20" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
@@ -2354,25 +2357,25 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C21" s="3" t="s">
+      <c r="D21" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="E21" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F21" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E21" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>129</v>
-      </c>
       <c r="G21" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
@@ -2380,25 +2383,25 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>132</v>
-      </c>
       <c r="G22" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
@@ -2406,25 +2409,25 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="C23" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="D23" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="E23" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="E23" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>137</v>
-      </c>
       <c r="G23" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
@@ -2432,25 +2435,25 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>141</v>
-      </c>
       <c r="G24" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
@@ -2458,25 +2461,25 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="C25" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="D25" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>145</v>
-      </c>
       <c r="G25" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
@@ -2484,25 +2487,25 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>149</v>
-      </c>
       <c r="G26" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
@@ -2510,25 +2513,25 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="C27" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="D27" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F27" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>153</v>
-      </c>
       <c r="G27" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
@@ -2536,25 +2539,25 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="D28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>157</v>
-      </c>
       <c r="G28" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
@@ -2562,25 +2565,25 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="C29" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="D29" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F29" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>161</v>
-      </c>
       <c r="G29" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
@@ -2588,25 +2591,25 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="D30" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>165</v>
-      </c>
       <c r="G30" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
@@ -2614,25 +2617,25 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="B31" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="C31" s="3" t="s">
+      <c r="D31" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F31" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="D31" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>168</v>
-      </c>
       <c r="G31" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
@@ -2640,25 +2643,25 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="D32" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="D32" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>172</v>
-      </c>
       <c r="G32" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
@@ -2666,25 +2669,25 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="B33" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="C33" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="D33" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="D33" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E33" s="3" t="s">
+      <c r="F33" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="F33" s="3" t="s">
-        <v>177</v>
-      </c>
       <c r="G33" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
@@ -2692,25 +2695,25 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="D34" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="D34" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>181</v>
-      </c>
       <c r="G34" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
@@ -2718,25 +2721,25 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B35" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="C35" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="D35" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F35" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D35" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>185</v>
-      </c>
       <c r="G35" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
@@ -2744,25 +2747,25 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="C36" s="2" t="s">
+      <c r="D36" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F36" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>188</v>
-      </c>
       <c r="G36" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
@@ -2770,25 +2773,25 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="C37" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="D37" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F37" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="D37" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>192</v>
-      </c>
       <c r="G37" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
@@ -2796,25 +2799,25 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="C38" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="D38" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F38" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>196</v>
-      </c>
       <c r="G38" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
@@ -2822,25 +2825,25 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="B39" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="C39" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="D39" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F39" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="D39" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>200</v>
-      </c>
       <c r="G39" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
@@ -2848,25 +2851,25 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="C40" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="D40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>204</v>
-      </c>
       <c r="G40" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
@@ -2874,25 +2877,25 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B41" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="C41" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="D41" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F41" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="D41" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>208</v>
-      </c>
       <c r="G41" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H41" s="3"/>
       <c r="I41" s="3"/>
@@ -2900,25 +2903,25 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="C42" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="D42" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="D42" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>212</v>
-      </c>
       <c r="G42" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
@@ -2926,25 +2929,25 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="C43" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="B43" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="C43" s="3" t="s">
+      <c r="D43" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F43" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="D43" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F43" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="G43" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H43" s="3"/>
       <c r="I43" s="3"/>
@@ -2952,25 +2955,25 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="C44" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="D44" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>219</v>
-      </c>
       <c r="G44" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
@@ -2978,25 +2981,25 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B45" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="C45" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="D45" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F45" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="D45" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E45" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F45" s="3" t="s">
-        <v>223</v>
-      </c>
       <c r="G45" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H45" s="3"/>
       <c r="I45" s="3"/>
@@ -3004,25 +3007,25 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="C46" s="2" t="s">
+      <c r="D46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F46" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="D46" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>226</v>
-      </c>
       <c r="G46" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
@@ -3030,25 +3033,25 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="B47" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="C47" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="D47" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="F47" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="D47" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="E47" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="F47" s="3" t="s">
-        <v>230</v>
-      </c>
       <c r="G47" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H47" s="3"/>
       <c r="I47" s="3"/>
@@ -3056,25 +3059,25 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="C48" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="D48" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F48" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="D48" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>234</v>
-      </c>
       <c r="G48" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
@@ -3082,25 +3085,25 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="C49" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="B49" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="C49" s="3" t="s">
+      <c r="D49" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F49" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="D49" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E49" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F49" s="3" t="s">
-        <v>237</v>
-      </c>
       <c r="G49" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H49" s="3"/>
       <c r="I49" s="3"/>
@@ -3108,25 +3111,25 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="C50" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="C50" s="2" t="s">
+      <c r="D50" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F50" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="D50" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>241</v>
-      </c>
       <c r="G50" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H50" s="2"/>
       <c r="I50" s="2"/>
@@ -3134,25 +3137,25 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="B51" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="B51" s="3" t="s">
+      <c r="C51" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="C51" s="3" t="s">
+      <c r="D51" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F51" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="D51" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E51" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F51" s="3" t="s">
-        <v>245</v>
-      </c>
       <c r="G51" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H51" s="3"/>
       <c r="I51" s="3"/>
@@ -3160,25 +3163,25 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B52" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="C52" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="C52" s="2" t="s">
+      <c r="D52" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F52" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="D52" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>249</v>
-      </c>
       <c r="G52" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H52" s="2"/>
       <c r="I52" s="2"/>
@@ -3186,25 +3189,25 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="C53" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="B53" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="C53" s="3" t="s">
+      <c r="D53" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F53" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="D53" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E53" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F53" s="3" t="s">
-        <v>252</v>
-      </c>
       <c r="G53" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H53" s="3"/>
       <c r="I53" s="3"/>
@@ -3212,25 +3215,25 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B54" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="C54" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="D54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F54" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D54" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>256</v>
-      </c>
       <c r="G54" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
@@ -3238,25 +3241,25 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="B55" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="B55" s="3" t="s">
+      <c r="C55" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="C55" s="3" t="s">
+      <c r="D55" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F55" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="D55" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F55" s="3" t="s">
-        <v>260</v>
-      </c>
       <c r="G55" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H55" s="3"/>
       <c r="I55" s="3"/>
@@ -3264,25 +3267,25 @@
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="C56" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="C56" s="2" t="s">
+      <c r="D56" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F56" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="D56" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>264</v>
-      </c>
       <c r="G56" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>
@@ -3290,25 +3293,25 @@
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="C57" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="B57" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="C57" s="3" t="s">
+      <c r="D57" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F57" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="D57" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E57" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>267</v>
-      </c>
       <c r="G57" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H57" s="3"/>
       <c r="I57" s="3"/>
@@ -3316,25 +3319,25 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="B58" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="C58" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="C58" s="2" t="s">
+      <c r="D58" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F58" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="D58" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>271</v>
-      </c>
       <c r="G58" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>
@@ -3342,25 +3345,25 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="C59" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="B59" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="C59" s="3" t="s">
+      <c r="D59" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F59" s="3" t="s">
         <v>273</v>
       </c>
-      <c r="D59" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E59" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F59" s="3" t="s">
-        <v>274</v>
-      </c>
       <c r="G59" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H59" s="3"/>
       <c r="I59" s="3"/>

</xml_diff>

<commit_message>
qa_test: drop Validated (APAI), add Remarks column; update README accordingly
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DF9FA4C-1FBA-4936-9588-46D05B825D78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FC2F5C3-C9D9-452A-A1CA-9A58A014E010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
@@ -878,7 +878,7 @@
     <t>Validated (Source)</t>
   </si>
   <si>
-    <t>Validated (APAI)</t>
+    <t>Remarks</t>
   </si>
 </sst>
 </file>
@@ -949,11 +949,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1297,10 +1299,10 @@
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="164.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -1329,10 +1331,10 @@
         <v>275</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="4" t="s">
         <v>278</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -1359,7 +1361,7 @@
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="J2" s="5"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1385,7 +1387,6 @@
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -1411,7 +1412,7 @@
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
+      <c r="J4" s="5"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
@@ -1437,7 +1438,6 @@
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
+      <c r="J6" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1481,10 +1481,10 @@
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="108.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -1513,10 +1513,10 @@
         <v>275</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="4" t="s">
         <v>278</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="J2" s="5"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1569,7 +1569,6 @@
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -1595,7 +1594,7 @@
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
+      <c r="J4" s="5"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
@@ -1621,7 +1620,6 @@
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1639,10 +1637,10 @@
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="83" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -1671,10 +1669,10 @@
         <v>275</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="4" t="s">
         <v>278</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -1701,7 +1699,7 @@
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="J2" s="5"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1727,7 +1725,6 @@
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -1753,7 +1750,7 @@
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
+      <c r="J4" s="5"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
@@ -1779,7 +1776,6 @@
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
@@ -1805,7 +1801,7 @@
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
+      <c r="J6" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1823,10 +1819,10 @@
     <col min="4" max="4" width="17.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="196.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -1855,10 +1851,10 @@
         <v>275</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="4" t="s">
         <v>278</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -1885,7 +1881,7 @@
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="J2" s="5"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1911,7 +1907,6 @@
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -1937,7 +1932,7 @@
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
+      <c r="J4" s="5"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
@@ -1963,7 +1958,6 @@
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
@@ -1989,7 +1983,7 @@
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
+      <c r="J6" s="5"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
@@ -2015,7 +2009,6 @@
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -2041,7 +2034,7 @@
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
+      <c r="J8" s="5"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
@@ -2067,7 +2060,6 @@
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -2093,7 +2085,7 @@
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
+      <c r="J10" s="5"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
@@ -2119,7 +2111,6 @@
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
@@ -2145,7 +2136,7 @@
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
+      <c r="J12" s="5"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
@@ -2171,7 +2162,6 @@
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
@@ -2197,7 +2187,7 @@
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
+      <c r="J14" s="5"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
@@ -2223,7 +2213,6 @@
       </c>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
@@ -2249,7 +2238,7 @@
       </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
+      <c r="J16" s="5"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
@@ -2275,7 +2264,6 @@
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
@@ -2301,7 +2289,7 @@
       </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
+      <c r="J18" s="5"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
@@ -2327,7 +2315,6 @@
       </c>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
@@ -2353,7 +2340,7 @@
       </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
+      <c r="J20" s="5"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
@@ -2379,7 +2366,6 @@
       </c>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
@@ -2405,7 +2391,7 @@
       </c>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
+      <c r="J22" s="5"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
@@ -2431,7 +2417,6 @@
       </c>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
@@ -2457,7 +2442,7 @@
       </c>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
+      <c r="J24" s="5"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
@@ -2483,7 +2468,6 @@
       </c>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
@@ -2509,7 +2493,7 @@
       </c>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
+      <c r="J26" s="5"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
@@ -2535,7 +2519,6 @@
       </c>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
-      <c r="J27" s="3"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
@@ -2561,7 +2544,7 @@
       </c>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
+      <c r="J28" s="5"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
@@ -2587,7 +2570,6 @@
       </c>
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
-      <c r="J29" s="3"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
@@ -2613,7 +2595,7 @@
       </c>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
+      <c r="J30" s="5"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
@@ -2639,7 +2621,6 @@
       </c>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
-      <c r="J31" s="3"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
@@ -2665,7 +2646,7 @@
       </c>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
+      <c r="J32" s="5"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
@@ -2691,7 +2672,6 @@
       </c>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
-      <c r="J33" s="3"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
@@ -2717,7 +2697,7 @@
       </c>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
+      <c r="J34" s="5"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
@@ -2743,7 +2723,6 @@
       </c>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
-      <c r="J35" s="3"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
@@ -2769,7 +2748,7 @@
       </c>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
+      <c r="J36" s="5"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
@@ -2795,7 +2774,6 @@
       </c>
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
-      <c r="J37" s="3"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
@@ -2821,7 +2799,7 @@
       </c>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
-      <c r="J38" s="2"/>
+      <c r="J38" s="5"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
@@ -2847,7 +2825,6 @@
       </c>
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
-      <c r="J39" s="3"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
@@ -2873,7 +2850,7 @@
       </c>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
-      <c r="J40" s="2"/>
+      <c r="J40" s="5"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
@@ -2899,7 +2876,6 @@
       </c>
       <c r="H41" s="3"/>
       <c r="I41" s="3"/>
-      <c r="J41" s="3"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
@@ -2925,7 +2901,7 @@
       </c>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
-      <c r="J42" s="2"/>
+      <c r="J42" s="5"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
@@ -2951,7 +2927,6 @@
       </c>
       <c r="H43" s="3"/>
       <c r="I43" s="3"/>
-      <c r="J43" s="3"/>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
@@ -2977,7 +2952,7 @@
       </c>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
-      <c r="J44" s="2"/>
+      <c r="J44" s="5"/>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
@@ -3003,7 +2978,6 @@
       </c>
       <c r="H45" s="3"/>
       <c r="I45" s="3"/>
-      <c r="J45" s="3"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
@@ -3029,7 +3003,7 @@
       </c>
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
-      <c r="J46" s="2"/>
+      <c r="J46" s="5"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
@@ -3055,7 +3029,6 @@
       </c>
       <c r="H47" s="3"/>
       <c r="I47" s="3"/>
-      <c r="J47" s="3"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
@@ -3081,7 +3054,7 @@
       </c>
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
-      <c r="J48" s="2"/>
+      <c r="J48" s="5"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
@@ -3107,7 +3080,6 @@
       </c>
       <c r="H49" s="3"/>
       <c r="I49" s="3"/>
-      <c r="J49" s="3"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
@@ -3133,7 +3105,7 @@
       </c>
       <c r="H50" s="2"/>
       <c r="I50" s="2"/>
-      <c r="J50" s="2"/>
+      <c r="J50" s="5"/>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
@@ -3159,7 +3131,6 @@
       </c>
       <c r="H51" s="3"/>
       <c r="I51" s="3"/>
-      <c r="J51" s="3"/>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
@@ -3185,7 +3156,7 @@
       </c>
       <c r="H52" s="2"/>
       <c r="I52" s="2"/>
-      <c r="J52" s="2"/>
+      <c r="J52" s="5"/>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
@@ -3211,7 +3182,6 @@
       </c>
       <c r="H53" s="3"/>
       <c r="I53" s="3"/>
-      <c r="J53" s="3"/>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
@@ -3237,7 +3207,7 @@
       </c>
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
-      <c r="J54" s="2"/>
+      <c r="J54" s="5"/>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
@@ -3263,7 +3233,6 @@
       </c>
       <c r="H55" s="3"/>
       <c r="I55" s="3"/>
-      <c r="J55" s="3"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
@@ -3289,7 +3258,7 @@
       </c>
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>
-      <c r="J56" s="2"/>
+      <c r="J56" s="5"/>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
@@ -3315,7 +3284,6 @@
       </c>
       <c r="H57" s="3"/>
       <c r="I57" s="3"/>
-      <c r="J57" s="3"/>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
@@ -3341,7 +3309,7 @@
       </c>
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>
-      <c r="J58" s="2"/>
+      <c r="J58" s="5"/>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
@@ -3367,7 +3335,6 @@
       </c>
       <c r="H59" s="3"/>
       <c r="I59" s="3"/>
-      <c r="J59" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
qa_test: add Found Source File/Page cols; run Impose - Auto Page Numbering (2 Pass, 3 Fail)
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FC2F5C3-C9D9-452A-A1CA-9A58A014E010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{246007A2-E6B9-432B-A772-C7CFC7FFC3C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
   <sheets>
     <sheet name="Impose - Auto Page Numbering" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="294">
   <si>
     <t>ID</t>
   </si>
@@ -879,6 +879,51 @@
   </si>
   <si>
     <t>Remarks</t>
+  </si>
+  <si>
+    <t>Found Source File</t>
+  </si>
+  <si>
+    <t>Found Source Page</t>
+  </si>
+  <si>
+    <t>The variable used in Apogee Impose to automatically add page numbers to an imposition is $page.rlindex.</t>
+  </si>
+  <si>
+    <t>Apogee-Impose-Trick_Automatic-Page-Numbering.pdf</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Correct variable cited. Source matches reference document.</t>
+  </si>
+  <si>
+    <t>To add a Text Mark to a Press Sheet in Apogee Impose, select the Press Sheet, go to the 'Marks' tab, choose 'Text Mark' from the 'Add Mark' dropdown menu, and then configure the settings for the Text Mark.</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Answer describes wrong UI path ('Add Mark' dropdown). Reference says: choose 'Text Mark' under Page Section of Marks palette and drag to Press Sheet. No source returned by APAI.</t>
+  </si>
+  <si>
+    <t>To save a new mark as a named Mark Set in Apogee Impose, create the mark, go to the 'Mark Sets' tab, click on 'Save As', enter a name for the Mark Set, and then click 'OK'.</t>
+  </si>
+  <si>
+    <t>Answer describes wrong steps ('Save As' / 'Mark Sets' tab). Reference says: click gear wheel at bottom of Mark Inspector, choose Add to Mark Set, select New. No source returned by APAI.</t>
+  </si>
+  <si>
+    <t>To apply a saved mark to every page in your layout in Apogee Impose, select the layout, go to the 'Marks' tab, choose the saved mark from the 'Apply Mark Set' dropdown menu, and then click 'Apply'.</t>
+  </si>
+  <si>
+    <t>Answer describes wrong UI path ('Apply Mark Set' dropdown). Reference says: select the mark under 'Page' in the Marks Set Inspector. No source returned by APAI.</t>
+  </si>
+  <si>
+    <t>Automatic page numbering provides clear guidance for both the bindery and pressman, facilitating a better understanding of how the piece should be assembled.</t>
+  </si>
+  <si>
+    <t>Answer matches reference. Correct source document and page.</t>
   </si>
 </sst>
 </file>
@@ -1290,7 +1335,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2DD8A55-FC28-4FDC-803C-713C907C6695}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
@@ -1301,11 +1346,12 @@
     <col min="6" max="6" width="164.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1331,13 +1377,19 @@
         <v>275</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1359,11 +1411,23 @@
       <c r="G2" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="5"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H2" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="J2" s="2">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
@@ -1385,10 +1449,19 @@
       <c r="G3" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H3" s="3"/>
+      <c r="H3" s="3" t="s">
+        <v>285</v>
+      </c>
       <c r="I3" s="3"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J3" s="3"/>
+      <c r="K3" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="L3" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -1410,11 +1483,19 @@
       <c r="G4" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>288</v>
+      </c>
       <c r="I4" s="2"/>
-      <c r="J4" s="5"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J4" s="2"/>
+      <c r="K4" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>19</v>
       </c>
@@ -1436,10 +1517,19 @@
       <c r="G5" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H5" s="3"/>
+      <c r="H5" s="3" t="s">
+        <v>290</v>
+      </c>
       <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J5" s="3"/>
+      <c r="K5" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="L5" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>24</v>
       </c>
@@ -1461,9 +1551,21 @@
       <c r="G6" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="5"/>
+      <c r="H6" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="J6" s="2">
+        <v>2</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>293</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
qa_test: add final score row to Impose - Auto Page Numbering (2/5 Pass)
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{246007A2-E6B9-432B-A772-C7CFC7FFC3C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED2B93C-B7CF-4BE3-B664-B628D0F43F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
@@ -1345,10 +1345,11 @@
     <col min="5" max="5" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="164.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="15.88671875" customWidth="1"/>
+    <col min="8" max="8" width="174.6640625" customWidth="1"/>
+    <col min="9" max="9" width="29.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
     <col min="11" max="11" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="77.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
qa_test: color Pass/Fail cells green/red in Impose - Auto Page Numbering
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED2B93C-B7CF-4BE3-B664-B628D0F43F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B32E308-CECD-495B-B3C6-7B56128CDB88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
@@ -930,7 +930,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -946,8 +946,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -963,6 +970,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00C000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCC0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -994,13 +1013,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1421,7 +1442,7 @@
       <c r="J2" s="2">
         <v>1</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="6" t="s">
         <v>283</v>
       </c>
       <c r="L2" s="5" t="s">
@@ -1455,7 +1476,7 @@
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="7" t="s">
         <v>286</v>
       </c>
       <c r="L3" t="s">
@@ -1489,7 +1510,7 @@
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="7" t="s">
         <v>286</v>
       </c>
       <c r="L4" s="5" t="s">
@@ -1523,7 +1544,7 @@
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
-      <c r="K5" s="3" t="s">
+      <c r="K5" s="7" t="s">
         <v>286</v>
       </c>
       <c r="L5" t="s">
@@ -1561,7 +1582,7 @@
       <c r="J6" s="2">
         <v>2</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="K6" s="6" t="s">
         <v>283</v>
       </c>
       <c r="L6" s="5" t="s">

</xml_diff>

<commit_message>
qa_test: add analysis note to Impose - Auto Page Numbering sheet
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B32E308-CECD-495B-B3C6-7B56128CDB88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DC44806-2C73-4918-A8ED-397EA7A9C43C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="296">
   <si>
     <t>ID</t>
   </si>
@@ -924,13 +924,19 @@
   </si>
   <si>
     <t>Answer matches reference. Correct source document and page.</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Score: 2/5 Pass. The 3 HOW_TO questions (IMP-002-004) all failed with hallucinated UI steps and no source citations, indicating the RAG system is not retrieving the procedural details from this document reliably.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -949,6 +955,22 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF046485"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF046485"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1013,7 +1035,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1022,6 +1044,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1356,7 +1382,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2DD8A55-FC28-4FDC-803C-713C907C6695}">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
@@ -1589,7 +1615,28 @@
         <v>293</v>
       </c>
     </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B9:L9"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
qa_test: run Impose - Folding Arrow sheet (3/4 Pass 75%)
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DC44806-2C73-4918-A8ED-397EA7A9C43C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{460A2BC3-1081-444B-A3F5-EE6ECB0BFF92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="308">
   <si>
     <t>ID</t>
   </si>
@@ -930,13 +930,49 @@
   </si>
   <si>
     <t>Score: 2/5 Pass. The 3 HOW_TO questions (IMP-002-004) all failed with hallucinated UI steps and no source citations, indicating the RAG system is not retrieving the procedural details from this document reliably.</t>
+  </si>
+  <si>
+    <t>The folding direction arrow in Apogee Impose indicates the direction in which the sheet will be folded.</t>
+  </si>
+  <si>
+    <t>Apogee_Impose_RG_14.0.1_en-US.pdf</t>
+  </si>
+  <si>
+    <t>Answer says 'direction the sheet will be folded'; reference says 'direction of the printed sheet moving into the folder'. Reference document (Folding-Direction-Arrow.pdf) not cited as top source.</t>
+  </si>
+  <si>
+    <t>When the fold direction arrow is pointing left, it indicates that the folding scheme is feeding into the folder with the short edge first.</t>
+  </si>
+  <si>
+    <t>Apogee-Impose-Trick_Folding-Direction-Arrow.pdf</t>
+  </si>
+  <si>
+    <t>No, the fold direction arrow also applies to pagination schemes and web production schemes.</t>
+  </si>
+  <si>
+    <t>Understanding the fold direction arrow is important because it helps ensure that the custom folding scheme is valid and correctly aligned with the folder's operation, reducing frustration and errors during setup.</t>
+  </si>
+  <si>
+    <t>Answer captures key idea about saving frustration. Correct source document and page.</t>
+  </si>
+  <si>
+    <t>FINAL SCORE</t>
+  </si>
+  <si>
+    <t>3 / 4 Pass (75%)</t>
+  </si>
+  <si>
+    <t>3 Pass (AP-FDA-002, AP-FDA-003, AP-FDA-004) | 1 Fail (AP-FDA-001)</t>
+  </si>
+  <si>
+    <t>Score: 3/4 Pass (75%). AP-FDA-001 failed due to an imprecise description of the arrow's meaning — the APAI answer described the folding direction rather than the sheet feed direction into the folder. The reference source document was not cited. The remaining 3 questions were answered correctly with the correct source retrieved.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -971,6 +1007,14 @@
       <i/>
       <sz val="11"/>
       <color rgb="FF046485"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1035,7 +1079,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1045,6 +1089,9 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1619,19 +1666,19 @@
       <c r="A9" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="12" t="s">
         <v>295</v>
       </c>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1643,7 +1690,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07129D57-73FC-44EA-91A3-D051877B6598}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
@@ -1658,7 +1705,7 @@
     <col min="10" max="10" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1684,13 +1731,19 @@
         <v>275</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="L1" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>28</v>
       </c>
@@ -1712,11 +1765,23 @@
       <c r="G2" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="5"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H2" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="J2" s="5">
+        <v>43</v>
+      </c>
+      <c r="K2" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="L2" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>32</v>
       </c>
@@ -1738,10 +1803,23 @@
       <c r="G3" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H3" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="L3" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -1763,11 +1841,23 @@
       <c r="G4" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="5"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H4" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="J4" s="5">
+        <v>1</v>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="L4" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>39</v>
       </c>
@@ -1789,10 +1879,55 @@
       <c r="G5" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
+      <c r="H5" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="L5" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="12"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B8:L8"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
qa_test: add FINAL SCORE row to Impose - Auto Page Numbering sheet
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{460A2BC3-1081-444B-A3F5-EE6ECB0BFF92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C4DE14A-EB38-4451-849C-966058AEEF48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="310">
   <si>
     <t>ID</t>
   </si>
@@ -966,6 +966,12 @@
   </si>
   <si>
     <t>Score: 3/4 Pass (75%). AP-FDA-001 failed due to an imprecise description of the arrow's meaning — the APAI answer described the folding direction rather than the sheet feed direction into the folder. The reference source document was not cited. The remaining 3 questions were answered correctly with the correct source retrieved.</t>
+  </si>
+  <si>
+    <t>2 / 5 Pass (40%)</t>
+  </si>
+  <si>
+    <t>2 Pass (AP-IMP-001, AP-IMP-005) | 3 Fail (AP-IMP-002, AP-IMP-003, AP-IMP-004)</t>
   </si>
 </sst>
 </file>
@@ -1662,6 +1668,17 @@
         <v>293</v>
       </c>
     </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>308</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>309</v>
+      </c>
+    </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>294</v>

</xml_diff>

<commit_message>
qa_test: add InkDrive CIP3 and ProductionCenter UG results (Run 3+4)
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C4DE14A-EB38-4451-849C-966058AEEF48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C5DCD90-8CD9-4AEF-BBA0-1DCC3099698D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
   <sheets>
     <sheet name="Impose - Auto Page Numbering" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="403">
   <si>
     <t>ID</t>
   </si>
@@ -972,13 +972,292 @@
   </si>
   <si>
     <t>2 Pass (AP-IMP-001, AP-IMP-005) | 3 Fail (AP-IMP-002, AP-IMP-003, AP-IMP-004)</t>
+  </si>
+  <si>
+    <t>ProductionCenter is a module of the printerâs workflow solution that is used to create and manage companies and users for the WebApproval softproofing service and the PrintSphere file-sharing service.</t>
+  </si>
+  <si>
+    <t>ProductionCenter_UG_14.0_en-US.pdf</t>
+  </si>
+  <si>
+    <t>WebApproval is a ProductionCenter service that enables collaboration between the Printer Company and Print Buyers for uploading files and approving softproofs.</t>
+  </si>
+  <si>
+    <t>Apogee_Prepress_OLH_14.0.2_en-US.pdf</t>
+  </si>
+  <si>
+    <t>WebFlow is a ProductionCenter service that allows Printer Company users to monitor all Apogee Prepress jobs and perform certain actions on these jobs from within their web browser.</t>
+  </si>
+  <si>
+    <t>Working_with_WebFlow.pdf</t>
+  </si>
+  <si>
+    <t>PrintSphere is a file-sharing and syncing service that allows users to store files in a dedicated space on the printsphere.com server, share files with other users, and sync files with their local computer.</t>
+  </si>
+  <si>
+    <t>PrintSphere_OLH_en-US_draft01.pdf</t>
+  </si>
+  <si>
+    <t>Workflow Connectivity in PrintSphere refers to the integration of the PrintSphere service with the Apogee Prepress or Asanti workflow system, allowing for automatic syncing and management of files within the workflow.</t>
+  </si>
+  <si>
+    <t>Answer about PrintSphere workflow, not ApogeeJobs shared folder per UG</t>
+  </si>
+  <si>
+    <t>The intended audience for the ProductionCenter User's Guide includes users who need to manage connectivity with the PrintSphere or WebApproval services, such as creating companies, users, and monitoring storage usage.</t>
+  </si>
+  <si>
+    <t>Incomplete - misses WebApproval/WebFlow/PrintSphere end-users scope</t>
+  </si>
+  <si>
+    <t>A new user receives access to ProductionCenter by being added to a company in ProductionCenter by an administrator. The administrator assigns the user a role, which determines the user's level of access and permissions within ProductionCenter.</t>
+  </si>
+  <si>
+    <t>The first time a user logs on to ProductionCenter, they must change their password.</t>
+  </si>
+  <si>
+    <t>Unfortunately I could not find a verified answer for your question. Please try rephrasing it, or contact support for help.</t>
+  </si>
+  <si>
+    <t>AI could not find answer; link validity (7 days) not retrieved</t>
+  </si>
+  <si>
+    <t>The two fields required to log on with an existing account are the e-mail address or User Name, and the password.</t>
+  </si>
+  <si>
+    <t>To log on using a passkey instead of a password, enter your e-mail address or User Name in the first field, and then click the 'Use Passkey' button. You will then be prompted to enter your passkey.</t>
+  </si>
+  <si>
+    <t>The Printer Administrator must enable the 'Allow Passkeys' setting in the PrintCenter Preferences for the Passkeys logon option to be available.</t>
+  </si>
+  <si>
+    <t>After logging on as a WebApproval user, the Jobs window is displayed, showing the jobs that require action by the user as an approver or as an uploader.</t>
+  </si>
+  <si>
+    <t>To log out of ProductionCenter, click the 'Log Out' button in the top-right corner of the screen.</t>
+  </si>
+  <si>
+    <t>AI says top-right corner; correct is top-left menu</t>
+  </si>
+  <si>
+    <t>To reset a forgotten password, click the 'Forgot Password' link on the logon screen. You will be prompted to enter your e-mail address, and a password reset link will be sent to your e-mail.</t>
+  </si>
+  <si>
+    <t>Only users with the Administrator role can edit other users' profiles in ProductionCenter.</t>
+  </si>
+  <si>
+    <t>A user can visually distinguish themselves within a Print Buyer Company by setting a unique color for their user profile. This color will be displayed in various areas of ProductionCenter to indicate actions or jobs associated with that user.</t>
+  </si>
+  <si>
+    <t>A Printer Administrator or CSR can create at least one user with the Administrator role for a Print Buyer company.</t>
+  </si>
+  <si>
+    <t>Printer_Company_-_Managing_Companies_Users.pdf</t>
+  </si>
+  <si>
+    <t>Describes admin creating admin user; REF describes adding any user as Administrator</t>
+  </si>
+  <si>
+    <t>The Uploader role is required to upload Production Files.</t>
+  </si>
+  <si>
+    <t>Production Files are the main content files (usually PDFs) that are processed by Apogee Prepress. Supplementary Files are additional files, such as source files, assets, or other documents, that are not processed by Apogee Prepress but are linked to a production job.</t>
+  </si>
+  <si>
+    <t>Upload_and_assign_files.pdf</t>
+  </si>
+  <si>
+    <t>No, a file uploaded for one job cannot be used in a different job.</t>
+  </si>
+  <si>
+    <t>The file cannot be placed in the Run List as there are not enough empty placeholders to accommodate all the pages.</t>
+  </si>
+  <si>
+    <t>Creating_and_Editing_Job_Tickets.pdf</t>
+  </si>
+  <si>
+    <t>AI says file cannot be placed at all; REF says last pages are not placed (partial placement)</t>
+  </si>
+  <si>
+    <t>To undo the last page placement, click the 'Undo' button located at the top of the Run List.</t>
+  </si>
+  <si>
+    <t>Pages with the 'Ready to Inspect' status and rejected pages can be replaced.</t>
+  </si>
+  <si>
+    <t>Preflighting is the process of checking a PDF file to ensure it meets specific criteria and standards before it is used in production. This includes checking for issues such as color management, font embedding, and other potential problems that could affect the final output.</t>
+  </si>
+  <si>
+    <t>Generic Apogee preflight description; REF refers to WebApproval system check</t>
+  </si>
+  <si>
+    <t>A preflight error is a critical issue that must be resolved before the job can proceed, while a preflight warning is a non-critical issue that may not affect the job's processing but should be reviewed.</t>
+  </si>
+  <si>
+    <t>To save a preflight Problem Report, click the 'Save' button in the Preflight panel and choose a location to save the report.</t>
+  </si>
+  <si>
+    <t>AI says Save button; REF says Mail Problem Report (email)</t>
+  </si>
+  <si>
+    <t>The two types of approval jobs in ProductionCenter are Direct Approval Job and Multiple Approval Job.</t>
+  </si>
+  <si>
+    <t>A page is considered approved in a Direct Approval job when one approver assigned to that job has approved that page.</t>
+  </si>
+  <si>
+    <t>A special license is required for the Multi Approval option.</t>
+  </si>
+  <si>
+    <t>Printer Administrators and CSRs can Force Approve pages, and a reason must be specified for the Force Approval.</t>
+  </si>
+  <si>
+    <t>Reapproval of a Frozen Page is a feature that allows Printer Administrators and CSRs to override the frozen state of a page, requiring it to be reapproved by the Print Buyer.</t>
+  </si>
+  <si>
+    <t>The two ways to create a new job in ProductionCenter are by clicking the 'New Job' button in the toolbar or by selecting 'New Job' from the 'File' menu.</t>
+  </si>
+  <si>
+    <t>AI describes general New Job button; REF lists Start New Job wizard and Hot Tickets</t>
+  </si>
+  <si>
+    <t>The four publishing options are: Publish, Publish Internally, Publish for Upload, and Publish for Approval.</t>
+  </si>
+  <si>
+    <t>In a Direct Approval job, a page is approved when one approver assigned to that job has approved that page. In a Multi Approval job, a page is approved when all approvers assigned to that job have approved that page.</t>
+  </si>
+  <si>
+    <t>To view additional job information such as page size, paper stock, and deadlines, click the 'Job Information' button in the toolbar or select 'Job Information' from the 'View' menu.</t>
+  </si>
+  <si>
+    <t>AI says Job Information button in toolbar; REF says Information icon on tile / press I</t>
+  </si>
+  <si>
+    <t>To edit user roles for a specific job, go to the 'Job Information' window, click on the 'Roles' tab, and then select the user whose role you want to change. From the drop-down menu, choose the new role and click 'OK' to save the changes.</t>
+  </si>
+  <si>
+    <t>AI describes different navigation steps; REF: Information icon → cogwheel → Edit User Roles</t>
+  </si>
+  <si>
+    <t>The Quick Picker options available when setting job deadlines are Today, Tomorrow, End of week (always a Friday), and Beginning of next week (always a Monday).</t>
+  </si>
+  <si>
+    <t>The three modes for comparing page history revisions in the Flipbook are Compare, Highlight, and Difference.</t>
+  </si>
+  <si>
+    <t>White Point and Texture</t>
+  </si>
+  <si>
+    <t>The job status icon showing a clock/warning indicates that the job is waiting for After Hours processing.</t>
+  </si>
+  <si>
+    <t>AI says waiting for After Hours processing; correct is approaching deadline / overdue</t>
+  </si>
+  <si>
+    <t>The icon indicating that all pages of a job have been placed and approved is the 'Approved' icon.</t>
+  </si>
+  <si>
+    <t>Approve_and_reject_pages.pdf</t>
+  </si>
+  <si>
+    <t>AI says 'Approved icon'; REF describes all pages placed and approved (job completed state)</t>
+  </si>
+  <si>
+    <t>Users with access to the Jobs window, including operators and administrators, can use the Jobs Filter feature.</t>
+  </si>
+  <si>
+    <t>AI says operators and admins; REF says only Printer Company users can filter</t>
+  </si>
+  <si>
+    <t>All Jobs' displays all jobs in the system, while 'My Jobs' displays only the jobs assigned to the current user.</t>
+  </si>
+  <si>
+    <t>Selecting multiple page status filters in the Jobs Filter behaves as an OR operation, meaning it will display jobs that match any of the selected statuses.</t>
+  </si>
+  <si>
+    <t>Versioning_-_Basic.pdf</t>
+  </si>
+  <si>
+    <t>AI could not find answer; REF: PDF files with layers cannot be assigned in versioning jobs</t>
+  </si>
+  <si>
+    <t>The 'Reject all n versions' checkbox allows you to reject a page or spread for all versions when reviewing a particular version.</t>
+  </si>
+  <si>
+    <t>The three modes for comparing product versions are: Compare, Highlight, and Difference.</t>
+  </si>
+  <si>
+    <t>To access Security Settings for passkeys in the Users window, select a user, click the 'Security' tab, and then click the 'Passkeys' button.</t>
+  </si>
+  <si>
+    <t>AI describes Security tab navigation; REF: click Security Settings link (arrow icon) in Users window</t>
+  </si>
+  <si>
+    <t>To add a passkey in ProductionCenter, select a user, click the 'Security' tab, click the 'Passkeys' button, and then click the 'Add' button.</t>
+  </si>
+  <si>
+    <t>To delete a passkey, select the user, click the 'Security' tab, click the 'Passkeys' button, select the passkey, and then click the 'Delete' button.</t>
+  </si>
+  <si>
+    <t>AI could not find answer; REF: Session Timeout default 30 min, max 4 hours</t>
+  </si>
+  <si>
+    <t>The Compare tab allows you to compare your edited e-mail messages against their factory settings in original or all other supported languages by using the additional drop-down list.</t>
+  </si>
+  <si>
+    <t>The Quick Approve action approves the current page or spread without displaying a confirmation window and takes you to the next page in the document that is awaiting approval.</t>
+  </si>
+  <si>
+    <t>AI could not find answer; REF: reason required in comment field when rejecting</t>
+  </si>
+  <si>
+    <t>AI could not find answer; REF: Press L = Show/hide Job Log</t>
+  </si>
+  <si>
+    <t>ALT + F</t>
+  </si>
+  <si>
+    <t>AI says ALT+F; REF says press { to flip view horizontally</t>
+  </si>
+  <si>
+    <t>38 Pass / 20 Fail (66%)</t>
+  </si>
+  <si>
+    <t>ProductionCenter UG test run 2026-06-03. 38/58 questions passed. Common failures: wrong source document, incorrect navigation instructions, unanswered questions.</t>
+  </si>
+  <si>
+    <t>The purpose of modifying Apogee CIP3 (.ppf) data is to more accurately preset the ink keys on a CIP3 enabled press, optimizing the preset data for initial press inking.</t>
+  </si>
+  <si>
+    <t>Apogee-InkDrive-Trick_Accurate-CIP3-Presets.pdf</t>
+  </si>
+  <si>
+    <t>Initially, 0, 50 and 100 are recommended.</t>
+  </si>
+  <si>
+    <t>Boost the power of the CIP preset by adding a fulcrum at 50 and adjusting the curve to increase the slope.</t>
+  </si>
+  <si>
+    <t>AI describes adjusting curve slope; REF says increase Adjusted Values above Density Values</t>
+  </si>
+  <si>
+    <t>Remember to save the resource and then apply it to the CIP3 data.</t>
+  </si>
+  <si>
+    <t>AI says save resource and apply; REF says update Parameter Sets</t>
+  </si>
+  <si>
+    <t>3 Pass / 2 Fail (60%)</t>
+  </si>
+  <si>
+    <t>InkDrive CIP3 test run 2026-06-03. 3/5 questions passed. Failures on Q4 (boost method wording) and Q5 (missing Parameter Sets tip).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1025,8 +1304,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FFCC6600"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1054,6 +1341,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFCC0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF235637"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEECC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1085,7 +1390,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1098,9 +1403,14 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1683,19 +1993,19 @@
       <c r="A9" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="15" t="s">
         <v>295</v>
       </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1720,6 +2030,7 @@
     <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="35.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
@@ -1927,19 +2238,19 @@
       <c r="A8" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="15" t="s">
         <v>307</v>
       </c>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1951,7 +2262,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB492513-0CEA-4027-8146-2D0121182802}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -1962,11 +2273,12 @@
     <col min="6" max="6" width="83" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1992,13 +2304,19 @@
         <v>275</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>42</v>
       </c>
@@ -2020,11 +2338,21 @@
       <c r="G2" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="5"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H2" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="J2" s="2">
+        <v>1</v>
+      </c>
+      <c r="K2" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L2" s="5"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>46</v>
       </c>
@@ -2046,10 +2374,20 @@
       <c r="G3" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H3" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="J3" s="3">
+        <v>1</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>49</v>
       </c>
@@ -2071,11 +2409,21 @@
       <c r="G4" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="5"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H4" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="J4" s="2">
+        <v>1</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L4" s="5"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>52</v>
       </c>
@@ -2097,10 +2445,19 @@
       <c r="G5" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H5" s="3"/>
+      <c r="H5" s="3" t="s">
+        <v>397</v>
+      </c>
       <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J5" s="3"/>
+      <c r="K5" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L5" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>55</v>
       </c>
@@ -2122,18 +2479,52 @@
       <c r="G6" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H6" s="2"/>
+      <c r="H6" s="2" t="s">
+        <v>399</v>
+      </c>
       <c r="I6" s="2"/>
-      <c r="J6" s="5"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B9" s="16" t="s">
+        <v>402</v>
+      </c>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="17"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B9:L9"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED61EE79-1B75-41E6-BD8B-15990556690E}">
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
@@ -2144,11 +2535,12 @@
     <col min="6" max="6" width="196.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2174,13 +2566,19 @@
         <v>275</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>59</v>
       </c>
@@ -2202,11 +2600,21 @@
       <c r="G2" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="5"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H2" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J2" s="2">
+        <v>3</v>
+      </c>
+      <c r="K2" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L2" s="5"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>63</v>
       </c>
@@ -2228,10 +2636,20 @@
       <c r="G3" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H3" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="J3" s="3">
+        <v>43</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>67</v>
       </c>
@@ -2253,11 +2671,21 @@
       <c r="G4" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="5"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H4" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="J4" s="2">
+        <v>1</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L4" s="5"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>70</v>
       </c>
@@ -2279,10 +2707,20 @@
       <c r="G5" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H5" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="J5" s="3">
+        <v>7</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>73</v>
       </c>
@@ -2304,11 +2742,23 @@
       <c r="G6" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="5"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H6" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="J6" s="2">
+        <v>8</v>
+      </c>
+      <c r="K6" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>76</v>
       </c>
@@ -2330,10 +2780,23 @@
       <c r="G7" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H7" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="J7" s="3">
+        <v>8</v>
+      </c>
+      <c r="K7" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L7" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>80</v>
       </c>
@@ -2355,11 +2818,17 @@
       <c r="G8" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H8" s="2"/>
+      <c r="H8" s="2" t="s">
+        <v>322</v>
+      </c>
       <c r="I8" s="2"/>
-      <c r="J8" s="5"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J8" s="2"/>
+      <c r="K8" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L8" s="5"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>84</v>
       </c>
@@ -2381,10 +2850,16 @@
       <c r="G9" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H9" s="3"/>
+      <c r="H9" s="3" t="s">
+        <v>323</v>
+      </c>
       <c r="I9" s="3"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J9" s="3"/>
+      <c r="K9" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>87</v>
       </c>
@@ -2406,11 +2881,19 @@
       <c r="G10" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H10" s="2"/>
+      <c r="H10" s="2" t="s">
+        <v>324</v>
+      </c>
       <c r="I10" s="2"/>
-      <c r="J10" s="5"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J10" s="2"/>
+      <c r="K10" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>91</v>
       </c>
@@ -2432,10 +2915,20 @@
       <c r="G11" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H11" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="J11" s="3">
+        <v>12</v>
+      </c>
+      <c r="K11" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>94</v>
       </c>
@@ -2457,11 +2950,17 @@
       <c r="G12" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H12" s="2"/>
+      <c r="H12" s="2" t="s">
+        <v>327</v>
+      </c>
       <c r="I12" s="2"/>
-      <c r="J12" s="5"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J12" s="2"/>
+      <c r="K12" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L12" s="5"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>97</v>
       </c>
@@ -2483,10 +2982,20 @@
       <c r="G13" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H13" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="J13" s="3">
+        <v>12</v>
+      </c>
+      <c r="K13" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>100</v>
       </c>
@@ -2508,11 +3017,21 @@
       <c r="G14" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="5"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H14" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J14" s="2">
+        <v>67</v>
+      </c>
+      <c r="K14" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L14" s="5"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>104</v>
       </c>
@@ -2534,10 +3053,19 @@
       <c r="G15" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H15" s="3"/>
+      <c r="H15" s="3" t="s">
+        <v>330</v>
+      </c>
       <c r="I15" s="3"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J15" s="3"/>
+      <c r="K15" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L15" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>107</v>
       </c>
@@ -2559,11 +3087,17 @@
       <c r="G16" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H16" s="2"/>
+      <c r="H16" s="2" t="s">
+        <v>332</v>
+      </c>
       <c r="I16" s="2"/>
-      <c r="J16" s="5"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J16" s="2"/>
+      <c r="K16" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L16" s="5"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>110</v>
       </c>
@@ -2585,10 +3119,20 @@
       <c r="G17" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H17" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="J17" s="3">
+        <v>16</v>
+      </c>
+      <c r="K17" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>114</v>
       </c>
@@ -2610,11 +3154,17 @@
       <c r="G18" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H18" s="2"/>
+      <c r="H18" s="2" t="s">
+        <v>334</v>
+      </c>
       <c r="I18" s="2"/>
-      <c r="J18" s="5"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J18" s="2"/>
+      <c r="K18" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L18" s="5"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>117</v>
       </c>
@@ -2636,10 +3186,23 @@
       <c r="G19" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H19" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="J19" s="3">
+        <v>2</v>
+      </c>
+      <c r="K19" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L19" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>121</v>
       </c>
@@ -2661,11 +3224,21 @@
       <c r="G20" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="5"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H20" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J20" s="2">
+        <v>17</v>
+      </c>
+      <c r="K20" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L20" s="5"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>125</v>
       </c>
@@ -2687,10 +3260,20 @@
       <c r="G21" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H21" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="J21" s="3">
+        <v>1</v>
+      </c>
+      <c r="K21" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>129</v>
       </c>
@@ -2712,11 +3295,21 @@
       <c r="G22" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="5"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H22" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J22" s="2">
+        <v>17</v>
+      </c>
+      <c r="K22" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L22" s="5"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>132</v>
       </c>
@@ -2738,10 +3331,23 @@
       <c r="G23" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H23" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="J23" s="3">
+        <v>3</v>
+      </c>
+      <c r="K23" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L23" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>137</v>
       </c>
@@ -2763,11 +3369,17 @@
       <c r="G24" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H24" s="2"/>
+      <c r="H24" s="2" t="s">
+        <v>345</v>
+      </c>
       <c r="I24" s="2"/>
-      <c r="J24" s="5"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J24" s="2"/>
+      <c r="K24" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L24" s="5"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>141</v>
       </c>
@@ -2789,10 +3401,20 @@
       <c r="G25" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H25" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="J25" s="3">
+        <v>28</v>
+      </c>
+      <c r="K25" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>145</v>
       </c>
@@ -2814,11 +3436,23 @@
       <c r="G26" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="5"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H26" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="J26" s="2">
+        <v>758</v>
+      </c>
+      <c r="K26" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L26" s="5" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>149</v>
       </c>
@@ -2840,10 +3474,20 @@
       <c r="G27" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H27" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="J27" s="3">
+        <v>31</v>
+      </c>
+      <c r="K27" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>153</v>
       </c>
@@ -2865,11 +3509,19 @@
       <c r="G28" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H28" s="2"/>
+      <c r="H28" s="2" t="s">
+        <v>350</v>
+      </c>
       <c r="I28" s="2"/>
-      <c r="J28" s="5"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J28" s="2"/>
+      <c r="K28" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L28" s="5" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>157</v>
       </c>
@@ -2891,10 +3543,20 @@
       <c r="G29" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H29" s="3"/>
-      <c r="I29" s="3"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H29" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="J29" s="3">
+        <v>3</v>
+      </c>
+      <c r="K29" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>161</v>
       </c>
@@ -2916,11 +3578,21 @@
       <c r="G30" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="5"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H30" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J30" s="2">
+        <v>35</v>
+      </c>
+      <c r="K30" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L30" s="5"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>165</v>
       </c>
@@ -2942,10 +3614,20 @@
       <c r="G31" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H31" s="3"/>
-      <c r="I31" s="3"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H31" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="J31" s="3">
+        <v>36</v>
+      </c>
+      <c r="K31" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>168</v>
       </c>
@@ -2967,11 +3649,21 @@
       <c r="G32" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="5"/>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H32" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J32" s="2">
+        <v>35</v>
+      </c>
+      <c r="K32" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L32" s="5"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
         <v>172</v>
       </c>
@@ -2993,10 +3685,20 @@
       <c r="G33" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H33" s="3"/>
-      <c r="I33" s="3"/>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H33" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="J33" s="3">
+        <v>35</v>
+      </c>
+      <c r="K33" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>177</v>
       </c>
@@ -3018,11 +3720,19 @@
       <c r="G34" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H34" s="2"/>
+      <c r="H34" s="2" t="s">
+        <v>357</v>
+      </c>
       <c r="I34" s="2"/>
-      <c r="J34" s="5"/>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J34" s="2"/>
+      <c r="K34" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L34" s="5" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
         <v>181</v>
       </c>
@@ -3044,10 +3754,20 @@
       <c r="G35" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H35" s="3"/>
-      <c r="I35" s="3"/>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H35" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="J35" s="3">
+        <v>293</v>
+      </c>
+      <c r="K35" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>185</v>
       </c>
@@ -3069,11 +3789,21 @@
       <c r="G36" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
-      <c r="J36" s="5"/>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H36" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J36" s="2">
+        <v>35</v>
+      </c>
+      <c r="K36" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L36" s="5"/>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>188</v>
       </c>
@@ -3095,10 +3825,19 @@
       <c r="G37" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H37" s="3"/>
+      <c r="H37" s="3" t="s">
+        <v>361</v>
+      </c>
       <c r="I37" s="3"/>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J37" s="3"/>
+      <c r="K37" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L37" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>192</v>
       </c>
@@ -3120,11 +3859,19 @@
       <c r="G38" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H38" s="2"/>
+      <c r="H38" s="2" t="s">
+        <v>363</v>
+      </c>
       <c r="I38" s="2"/>
-      <c r="J38" s="5"/>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J38" s="2"/>
+      <c r="K38" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L38" s="5" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
         <v>196</v>
       </c>
@@ -3146,10 +3893,20 @@
       <c r="G39" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H39" s="3"/>
-      <c r="I39" s="3"/>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H39" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="J39" s="3">
+        <v>58</v>
+      </c>
+      <c r="K39" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>200</v>
       </c>
@@ -3171,11 +3928,21 @@
       <c r="G40" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H40" s="2"/>
-      <c r="I40" s="2"/>
-      <c r="J40" s="5"/>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H40" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J40" s="2">
+        <v>84</v>
+      </c>
+      <c r="K40" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L40" s="5"/>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
         <v>204</v>
       </c>
@@ -3197,10 +3964,20 @@
       <c r="G41" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H41" s="3"/>
-      <c r="I41" s="3"/>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H41" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="I41" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="J41" s="3">
+        <v>890</v>
+      </c>
+      <c r="K41" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>208</v>
       </c>
@@ -3222,11 +3999,23 @@
       <c r="G42" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H42" s="2"/>
-      <c r="I42" s="2"/>
-      <c r="J42" s="5"/>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H42" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="J42" s="2">
+        <v>145</v>
+      </c>
+      <c r="K42" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L42" s="5" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
         <v>212</v>
       </c>
@@ -3248,10 +4037,23 @@
       <c r="G43" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H43" s="3"/>
-      <c r="I43" s="3"/>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H43" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="I43" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="J43" s="3">
+        <v>2</v>
+      </c>
+      <c r="K43" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L43" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>215</v>
       </c>
@@ -3273,11 +4075,23 @@
       <c r="G44" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H44" s="2"/>
-      <c r="I44" s="2"/>
-      <c r="J44" s="5"/>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H44" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J44" s="2">
+        <v>74</v>
+      </c>
+      <c r="K44" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L44" s="5" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
         <v>219</v>
       </c>
@@ -3299,10 +4113,20 @@
       <c r="G45" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H45" s="3"/>
-      <c r="I45" s="3"/>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H45" s="14" t="s">
+        <v>375</v>
+      </c>
+      <c r="I45" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="J45" s="3">
+        <v>74</v>
+      </c>
+      <c r="K45" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>223</v>
       </c>
@@ -3324,11 +4148,21 @@
       <c r="G46" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H46" s="2"/>
-      <c r="I46" s="2"/>
-      <c r="J46" s="5"/>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H46" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J46" s="2">
+        <v>177</v>
+      </c>
+      <c r="K46" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L46" s="5"/>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>226</v>
       </c>
@@ -3350,10 +4184,23 @@
       <c r="G47" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H47" s="3"/>
-      <c r="I47" s="3"/>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H47" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="I47" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="J47" s="3">
+        <v>9</v>
+      </c>
+      <c r="K47" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L47" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>230</v>
       </c>
@@ -3375,11 +4222,21 @@
       <c r="G48" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H48" s="2"/>
-      <c r="I48" s="2"/>
-      <c r="J48" s="5"/>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H48" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="J48" s="2">
+        <v>10</v>
+      </c>
+      <c r="K48" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L48" s="5"/>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
         <v>234</v>
       </c>
@@ -3401,10 +4258,20 @@
       <c r="G49" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H49" s="3"/>
-      <c r="I49" s="3"/>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H49" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="I49" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="J49" s="3">
+        <v>94</v>
+      </c>
+      <c r="K49" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>237</v>
       </c>
@@ -3426,11 +4293,19 @@
       <c r="G50" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H50" s="2"/>
+      <c r="H50" s="2" t="s">
+        <v>381</v>
+      </c>
       <c r="I50" s="2"/>
-      <c r="J50" s="5"/>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J50" s="2"/>
+      <c r="K50" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L50" s="5" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
         <v>241</v>
       </c>
@@ -3452,10 +4327,16 @@
       <c r="G51" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H51" s="3"/>
+      <c r="H51" s="3" t="s">
+        <v>383</v>
+      </c>
       <c r="I51" s="3"/>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J51" s="3"/>
+      <c r="K51" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>245</v>
       </c>
@@ -3477,11 +4358,17 @@
       <c r="G52" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H52" s="2"/>
+      <c r="H52" s="2" t="s">
+        <v>384</v>
+      </c>
       <c r="I52" s="2"/>
-      <c r="J52" s="5"/>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J52" s="2"/>
+      <c r="K52" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L52" s="5"/>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
         <v>249</v>
       </c>
@@ -3503,10 +4390,20 @@
       <c r="G53" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H53" s="3"/>
-      <c r="I53" s="3"/>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H53" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="I53" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="J53" s="3">
+        <v>233</v>
+      </c>
+      <c r="K53" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>252</v>
       </c>
@@ -3528,11 +4425,19 @@
       <c r="G54" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H54" s="2"/>
+      <c r="H54" s="2" t="s">
+        <v>324</v>
+      </c>
       <c r="I54" s="2"/>
-      <c r="J54" s="5"/>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J54" s="2"/>
+      <c r="K54" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L54" s="5" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
         <v>256</v>
       </c>
@@ -3554,10 +4459,20 @@
       <c r="G55" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H55" s="3"/>
-      <c r="I55" s="3"/>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H55" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="I55" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="J55" s="3">
+        <v>248</v>
+      </c>
+      <c r="K55" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>260</v>
       </c>
@@ -3579,11 +4494,21 @@
       <c r="G56" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H56" s="2"/>
-      <c r="I56" s="2"/>
-      <c r="J56" s="5"/>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H56" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J56" s="2">
+        <v>47</v>
+      </c>
+      <c r="K56" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L56" s="5"/>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
         <v>264</v>
       </c>
@@ -3605,10 +4530,23 @@
       <c r="G57" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H57" s="3"/>
-      <c r="I57" s="3"/>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H57" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="I57" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="J57" s="3">
+        <v>5</v>
+      </c>
+      <c r="K57" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L57" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>267</v>
       </c>
@@ -3630,11 +4568,23 @@
       <c r="G58" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="H58" s="2"/>
-      <c r="I58" s="2"/>
-      <c r="J58" s="5"/>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H58" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J58" s="2">
+        <v>131</v>
+      </c>
+      <c r="K58" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L58" s="5" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
         <v>271</v>
       </c>
@@ -3656,10 +4606,49 @@
       <c r="G59" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H59" s="3"/>
-      <c r="I59" s="3"/>
+      <c r="H59" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="I59" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="J59" s="3">
+        <v>78</v>
+      </c>
+      <c r="K59" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="L59" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A60" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="K60" s="11" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B61" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="C61" s="17"/>
+      <c r="D61" s="17"/>
+      <c r="E61" s="17"/>
+      <c r="F61" s="17"/>
+      <c r="G61" s="17"/>
+      <c r="H61" s="17"/>
+      <c r="I61" s="17"/>
+      <c r="J61" s="17"/>
+      <c r="K61" s="17"/>
+      <c r="L61" s="17"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B61:L61"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
qa_test: fix Pass/Fail cell colors in sheets 3+4 to match sheets 1+2
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C5DCD90-8CD9-4AEF-BBA0-1DCC3099698D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A0FF4EF-89C6-4B43-A93B-FF16AE4596DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
@@ -1313,7 +1313,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1341,18 +1341,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFCC0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF235637"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC00000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1403,14 +1391,14 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1993,19 +1981,19 @@
       <c r="A9" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="13" t="s">
         <v>295</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="15"/>
-      <c r="L9" s="15"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="13"/>
+      <c r="L9" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2238,19 +2226,19 @@
       <c r="A8" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="13" t="s">
         <v>307</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="15"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13"/>
+      <c r="L8" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2347,7 +2335,7 @@
       <c r="J2" s="2">
         <v>1</v>
       </c>
-      <c r="K2" s="12" t="s">
+      <c r="K2" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L2" s="5"/>
@@ -2383,7 +2371,7 @@
       <c r="J3" s="3">
         <v>1</v>
       </c>
-      <c r="K3" s="12" t="s">
+      <c r="K3" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -2418,7 +2406,7 @@
       <c r="J4" s="2">
         <v>1</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="K4" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L4" s="5"/>
@@ -2450,7 +2438,7 @@
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
-      <c r="K5" s="13" t="s">
+      <c r="K5" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L5" t="s">
@@ -2484,7 +2472,7 @@
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="13" t="s">
+      <c r="K6" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L6" s="5" t="s">
@@ -2500,19 +2488,19 @@
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="14" t="s">
         <v>402</v>
       </c>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2609,7 +2597,7 @@
       <c r="J2" s="2">
         <v>3</v>
       </c>
-      <c r="K2" s="12" t="s">
+      <c r="K2" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L2" s="5"/>
@@ -2645,7 +2633,7 @@
       <c r="J3" s="3">
         <v>43</v>
       </c>
-      <c r="K3" s="12" t="s">
+      <c r="K3" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -2680,7 +2668,7 @@
       <c r="J4" s="2">
         <v>1</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="K4" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L4" s="5"/>
@@ -2716,7 +2704,7 @@
       <c r="J5" s="3">
         <v>7</v>
       </c>
-      <c r="K5" s="12" t="s">
+      <c r="K5" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -2751,7 +2739,7 @@
       <c r="J6" s="2">
         <v>8</v>
       </c>
-      <c r="K6" s="13" t="s">
+      <c r="K6" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L6" s="5" t="s">
@@ -2789,7 +2777,7 @@
       <c r="J7" s="3">
         <v>8</v>
       </c>
-      <c r="K7" s="13" t="s">
+      <c r="K7" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L7" t="s">
@@ -2823,7 +2811,7 @@
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
-      <c r="K8" s="12" t="s">
+      <c r="K8" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L8" s="5"/>
@@ -2855,7 +2843,7 @@
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
-      <c r="K9" s="12" t="s">
+      <c r="K9" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -2886,7 +2874,7 @@
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
-      <c r="K10" s="13" t="s">
+      <c r="K10" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L10" s="5" t="s">
@@ -2924,7 +2912,7 @@
       <c r="J11" s="3">
         <v>12</v>
       </c>
-      <c r="K11" s="12" t="s">
+      <c r="K11" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -2955,7 +2943,7 @@
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
-      <c r="K12" s="12" t="s">
+      <c r="K12" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L12" s="5"/>
@@ -2991,7 +2979,7 @@
       <c r="J13" s="3">
         <v>12</v>
       </c>
-      <c r="K13" s="12" t="s">
+      <c r="K13" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3026,7 +3014,7 @@
       <c r="J14" s="2">
         <v>67</v>
       </c>
-      <c r="K14" s="12" t="s">
+      <c r="K14" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L14" s="5"/>
@@ -3058,7 +3046,7 @@
       </c>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
-      <c r="K15" s="13" t="s">
+      <c r="K15" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L15" t="s">
@@ -3092,7 +3080,7 @@
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
-      <c r="K16" s="12" t="s">
+      <c r="K16" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L16" s="5"/>
@@ -3128,7 +3116,7 @@
       <c r="J17" s="3">
         <v>16</v>
       </c>
-      <c r="K17" s="12" t="s">
+      <c r="K17" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3159,7 +3147,7 @@
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
-      <c r="K18" s="12" t="s">
+      <c r="K18" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L18" s="5"/>
@@ -3195,7 +3183,7 @@
       <c r="J19" s="3">
         <v>2</v>
       </c>
-      <c r="K19" s="13" t="s">
+      <c r="K19" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L19" t="s">
@@ -3233,7 +3221,7 @@
       <c r="J20" s="2">
         <v>17</v>
       </c>
-      <c r="K20" s="12" t="s">
+      <c r="K20" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L20" s="5"/>
@@ -3269,7 +3257,7 @@
       <c r="J21" s="3">
         <v>1</v>
       </c>
-      <c r="K21" s="12" t="s">
+      <c r="K21" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3304,7 +3292,7 @@
       <c r="J22" s="2">
         <v>17</v>
       </c>
-      <c r="K22" s="12" t="s">
+      <c r="K22" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L22" s="5"/>
@@ -3340,7 +3328,7 @@
       <c r="J23" s="3">
         <v>3</v>
       </c>
-      <c r="K23" s="13" t="s">
+      <c r="K23" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L23" t="s">
@@ -3374,7 +3362,7 @@
       </c>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
-      <c r="K24" s="12" t="s">
+      <c r="K24" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L24" s="5"/>
@@ -3410,7 +3398,7 @@
       <c r="J25" s="3">
         <v>28</v>
       </c>
-      <c r="K25" s="12" t="s">
+      <c r="K25" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3445,7 +3433,7 @@
       <c r="J26" s="2">
         <v>758</v>
       </c>
-      <c r="K26" s="13" t="s">
+      <c r="K26" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L26" s="5" t="s">
@@ -3483,7 +3471,7 @@
       <c r="J27" s="3">
         <v>31</v>
       </c>
-      <c r="K27" s="12" t="s">
+      <c r="K27" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3514,7 +3502,7 @@
       </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
-      <c r="K28" s="13" t="s">
+      <c r="K28" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L28" s="5" t="s">
@@ -3552,7 +3540,7 @@
       <c r="J29" s="3">
         <v>3</v>
       </c>
-      <c r="K29" s="12" t="s">
+      <c r="K29" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3587,7 +3575,7 @@
       <c r="J30" s="2">
         <v>35</v>
       </c>
-      <c r="K30" s="12" t="s">
+      <c r="K30" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L30" s="5"/>
@@ -3623,7 +3611,7 @@
       <c r="J31" s="3">
         <v>36</v>
       </c>
-      <c r="K31" s="12" t="s">
+      <c r="K31" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3658,7 +3646,7 @@
       <c r="J32" s="2">
         <v>35</v>
       </c>
-      <c r="K32" s="12" t="s">
+      <c r="K32" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L32" s="5"/>
@@ -3694,7 +3682,7 @@
       <c r="J33" s="3">
         <v>35</v>
       </c>
-      <c r="K33" s="12" t="s">
+      <c r="K33" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3725,7 +3713,7 @@
       </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
-      <c r="K34" s="13" t="s">
+      <c r="K34" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L34" s="5" t="s">
@@ -3763,7 +3751,7 @@
       <c r="J35" s="3">
         <v>293</v>
       </c>
-      <c r="K35" s="12" t="s">
+      <c r="K35" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3798,7 +3786,7 @@
       <c r="J36" s="2">
         <v>35</v>
       </c>
-      <c r="K36" s="12" t="s">
+      <c r="K36" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L36" s="5"/>
@@ -3830,7 +3818,7 @@
       </c>
       <c r="I37" s="3"/>
       <c r="J37" s="3"/>
-      <c r="K37" s="13" t="s">
+      <c r="K37" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L37" t="s">
@@ -3864,7 +3852,7 @@
       </c>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
-      <c r="K38" s="13" t="s">
+      <c r="K38" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L38" s="5" t="s">
@@ -3902,7 +3890,7 @@
       <c r="J39" s="3">
         <v>58</v>
       </c>
-      <c r="K39" s="12" t="s">
+      <c r="K39" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3937,7 +3925,7 @@
       <c r="J40" s="2">
         <v>84</v>
       </c>
-      <c r="K40" s="12" t="s">
+      <c r="K40" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L40" s="5"/>
@@ -3973,7 +3961,7 @@
       <c r="J41" s="3">
         <v>890</v>
       </c>
-      <c r="K41" s="12" t="s">
+      <c r="K41" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -4008,7 +3996,7 @@
       <c r="J42" s="2">
         <v>145</v>
       </c>
-      <c r="K42" s="13" t="s">
+      <c r="K42" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L42" s="5" t="s">
@@ -4046,7 +4034,7 @@
       <c r="J43" s="3">
         <v>2</v>
       </c>
-      <c r="K43" s="13" t="s">
+      <c r="K43" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L43" t="s">
@@ -4084,7 +4072,7 @@
       <c r="J44" s="2">
         <v>74</v>
       </c>
-      <c r="K44" s="13" t="s">
+      <c r="K44" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L44" s="5" t="s">
@@ -4113,7 +4101,7 @@
       <c r="G45" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="H45" s="14" t="s">
+      <c r="H45" s="12" t="s">
         <v>375</v>
       </c>
       <c r="I45" s="3" t="s">
@@ -4122,7 +4110,7 @@
       <c r="J45" s="3">
         <v>74</v>
       </c>
-      <c r="K45" s="12" t="s">
+      <c r="K45" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -4157,7 +4145,7 @@
       <c r="J46" s="2">
         <v>177</v>
       </c>
-      <c r="K46" s="12" t="s">
+      <c r="K46" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L46" s="5"/>
@@ -4193,7 +4181,7 @@
       <c r="J47" s="3">
         <v>9</v>
       </c>
-      <c r="K47" s="13" t="s">
+      <c r="K47" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L47" t="s">
@@ -4231,7 +4219,7 @@
       <c r="J48" s="2">
         <v>10</v>
       </c>
-      <c r="K48" s="12" t="s">
+      <c r="K48" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L48" s="5"/>
@@ -4267,7 +4255,7 @@
       <c r="J49" s="3">
         <v>94</v>
       </c>
-      <c r="K49" s="12" t="s">
+      <c r="K49" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -4298,7 +4286,7 @@
       </c>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
-      <c r="K50" s="13" t="s">
+      <c r="K50" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L50" s="5" t="s">
@@ -4332,7 +4320,7 @@
       </c>
       <c r="I51" s="3"/>
       <c r="J51" s="3"/>
-      <c r="K51" s="12" t="s">
+      <c r="K51" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -4363,7 +4351,7 @@
       </c>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
-      <c r="K52" s="12" t="s">
+      <c r="K52" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L52" s="5"/>
@@ -4399,7 +4387,7 @@
       <c r="J53" s="3">
         <v>233</v>
       </c>
-      <c r="K53" s="12" t="s">
+      <c r="K53" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -4430,7 +4418,7 @@
       </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
-      <c r="K54" s="13" t="s">
+      <c r="K54" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L54" s="5" t="s">
@@ -4468,7 +4456,7 @@
       <c r="J55" s="3">
         <v>248</v>
       </c>
-      <c r="K55" s="12" t="s">
+      <c r="K55" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -4503,7 +4491,7 @@
       <c r="J56" s="2">
         <v>47</v>
       </c>
-      <c r="K56" s="12" t="s">
+      <c r="K56" s="16" t="s">
         <v>283</v>
       </c>
       <c r="L56" s="5"/>
@@ -4539,7 +4527,7 @@
       <c r="J57" s="3">
         <v>5</v>
       </c>
-      <c r="K57" s="13" t="s">
+      <c r="K57" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L57" t="s">
@@ -4577,7 +4565,7 @@
       <c r="J58" s="2">
         <v>131</v>
       </c>
-      <c r="K58" s="13" t="s">
+      <c r="K58" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L58" s="5" t="s">
@@ -4615,7 +4603,7 @@
       <c r="J59" s="3">
         <v>78</v>
       </c>
-      <c r="K59" s="13" t="s">
+      <c r="K59" s="17" t="s">
         <v>286</v>
       </c>
       <c r="L59" t="s">
@@ -4631,19 +4619,19 @@
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B61" s="16" t="s">
+      <c r="B61" s="14" t="s">
         <v>393</v>
       </c>
-      <c r="C61" s="17"/>
-      <c r="D61" s="17"/>
-      <c r="E61" s="17"/>
-      <c r="F61" s="17"/>
-      <c r="G61" s="17"/>
-      <c r="H61" s="17"/>
-      <c r="I61" s="17"/>
-      <c r="J61" s="17"/>
-      <c r="K61" s="17"/>
-      <c r="L61" s="17"/>
+      <c r="C61" s="15"/>
+      <c r="D61" s="15"/>
+      <c r="E61" s="15"/>
+      <c r="F61" s="15"/>
+      <c r="G61" s="15"/>
+      <c r="H61" s="15"/>
+      <c r="I61" s="15"/>
+      <c r="J61" s="15"/>
+      <c r="K61" s="15"/>
+      <c r="L61" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
qa_test: apply green/red colors to FINAL SCORE rows in all 4 sheets
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A0FF4EF-89C6-4B43-A93B-FF16AE4596DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF4EF53A-D5D2-4023-AB5A-CD10AA715C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="407">
   <si>
     <t>ID</t>
   </si>
@@ -956,24 +956,9 @@
     <t>Answer captures key idea about saving frustration. Correct source document and page.</t>
   </si>
   <si>
-    <t>FINAL SCORE</t>
-  </si>
-  <si>
-    <t>3 / 4 Pass (75%)</t>
-  </si>
-  <si>
-    <t>3 Pass (AP-FDA-002, AP-FDA-003, AP-FDA-004) | 1 Fail (AP-FDA-001)</t>
-  </si>
-  <si>
     <t>Score: 3/4 Pass (75%). AP-FDA-001 failed due to an imprecise description of the arrow's meaning — the APAI answer described the folding direction rather than the sheet feed direction into the folder. The reference source document was not cited. The remaining 3 questions were answered correctly with the correct source retrieved.</t>
   </si>
   <si>
-    <t>2 / 5 Pass (40%)</t>
-  </si>
-  <si>
-    <t>2 Pass (AP-IMP-001, AP-IMP-005) | 3 Fail (AP-IMP-002, AP-IMP-003, AP-IMP-004)</t>
-  </si>
-  <si>
     <t>ProductionCenter is a module of the printerâs workflow solution that is used to create and manage companies and users for the WebApproval softproofing service and the PrintSphere file-sharing service.</t>
   </si>
   <si>
@@ -1220,9 +1205,6 @@
     <t>AI says ALT+F; REF says press { to flip view horizontally</t>
   </si>
   <si>
-    <t>38 Pass / 20 Fail (66%)</t>
-  </si>
-  <si>
     <t>ProductionCenter UG test run 2026-06-03. 38/58 questions passed. Common failures: wrong source document, incorrect navigation instructions, unanswered questions.</t>
   </si>
   <si>
@@ -1247,10 +1229,40 @@
     <t>AI says save resource and apply; REF says update Parameter Sets</t>
   </si>
   <si>
-    <t>3 Pass / 2 Fail (60%)</t>
-  </si>
-  <si>
     <t>InkDrive CIP3 test run 2026-06-03. 3/5 questions passed. Failures on Q4 (boost method wording) and Q5 (missing Parameter Sets tip).</t>
+  </si>
+  <si>
+    <t>FINAL SCORE (40%)</t>
+  </si>
+  <si>
+    <t>2 Pass</t>
+  </si>
+  <si>
+    <t>3 Fail</t>
+  </si>
+  <si>
+    <t>FINAL SCORE (75%)</t>
+  </si>
+  <si>
+    <t>3 Pass</t>
+  </si>
+  <si>
+    <t>1 Fail</t>
+  </si>
+  <si>
+    <t>FINAL SCORE (60%)</t>
+  </si>
+  <si>
+    <t>2 Fail</t>
+  </si>
+  <si>
+    <t>FINAL SCORE (66%)</t>
+  </si>
+  <si>
+    <t>38 Pass</t>
+  </si>
+  <si>
+    <t>20 Fail</t>
   </si>
 </sst>
 </file>
@@ -1378,7 +1390,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1392,13 +1404,15 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1968,32 +1982,32 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>304</v>
-      </c>
-      <c r="K8" s="11" t="s">
-        <v>308</v>
-      </c>
-      <c r="L8" s="11" t="s">
-        <v>309</v>
+        <v>396</v>
+      </c>
+      <c r="K8" s="18" t="s">
+        <v>397</v>
+      </c>
+      <c r="L8" s="19" t="s">
+        <v>398</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="15" t="s">
         <v>295</v>
       </c>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="13"/>
-      <c r="L9" s="13"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2213,32 +2227,32 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>304</v>
-      </c>
-      <c r="K7" s="11" t="s">
-        <v>305</v>
-      </c>
-      <c r="L7" s="11" t="s">
-        <v>306</v>
+        <v>399</v>
+      </c>
+      <c r="K7" s="18" t="s">
+        <v>400</v>
+      </c>
+      <c r="L7" s="19" t="s">
+        <v>401</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B8" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
-      <c r="J8" s="13"/>
-      <c r="K8" s="13"/>
-      <c r="L8" s="13"/>
+      <c r="B8" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2327,15 +2341,15 @@
         <v>276</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="J2" s="2">
         <v>1</v>
       </c>
-      <c r="K2" s="16" t="s">
+      <c r="K2" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L2" s="5"/>
@@ -2366,12 +2380,12 @@
         <v>48</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="J3" s="3">
         <v>1</v>
       </c>
-      <c r="K3" s="16" t="s">
+      <c r="K3" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -2398,15 +2412,15 @@
         <v>276</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="J4" s="2">
         <v>1</v>
       </c>
-      <c r="K4" s="16" t="s">
+      <c r="K4" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L4" s="5"/>
@@ -2434,15 +2448,15 @@
         <v>276</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
-      <c r="K5" s="17" t="s">
+      <c r="K5" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L5" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -2468,39 +2482,42 @@
         <v>276</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="17" t="s">
+      <c r="K6" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>304</v>
-      </c>
-      <c r="K8" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
+      </c>
+      <c r="K8" s="18" t="s">
+        <v>400</v>
+      </c>
+      <c r="L8" s="19" t="s">
+        <v>403</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B9" s="14" t="s">
-        <v>402</v>
-      </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="15"/>
-      <c r="L9" s="15"/>
+      <c r="B9" s="16" t="s">
+        <v>395</v>
+      </c>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2589,15 +2606,15 @@
         <v>276</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J2" s="2">
         <v>3</v>
       </c>
-      <c r="K2" s="16" t="s">
+      <c r="K2" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L2" s="5"/>
@@ -2625,15 +2642,15 @@
         <v>276</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="J3" s="3">
         <v>43</v>
       </c>
-      <c r="K3" s="16" t="s">
+      <c r="K3" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -2660,15 +2677,15 @@
         <v>276</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="J4" s="2">
         <v>1</v>
       </c>
-      <c r="K4" s="16" t="s">
+      <c r="K4" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L4" s="5"/>
@@ -2696,15 +2713,15 @@
         <v>276</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="J5" s="3">
         <v>7</v>
       </c>
-      <c r="K5" s="16" t="s">
+      <c r="K5" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -2731,19 +2748,19 @@
         <v>276</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="J6" s="2">
         <v>8</v>
       </c>
-      <c r="K6" s="17" t="s">
+      <c r="K6" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -2769,19 +2786,19 @@
         <v>276</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="J7" s="3">
         <v>8</v>
       </c>
-      <c r="K7" s="17" t="s">
+      <c r="K7" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L7" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
@@ -2807,11 +2824,11 @@
         <v>276</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
-      <c r="K8" s="16" t="s">
+      <c r="K8" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L8" s="5"/>
@@ -2839,11 +2856,11 @@
         <v>276</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
-      <c r="K9" s="16" t="s">
+      <c r="K9" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -2870,15 +2887,15 @@
         <v>276</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
-      <c r="K10" s="17" t="s">
+      <c r="K10" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L10" s="5" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
@@ -2904,15 +2921,15 @@
         <v>276</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J11" s="3">
         <v>12</v>
       </c>
-      <c r="K11" s="16" t="s">
+      <c r="K11" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -2939,11 +2956,11 @@
         <v>276</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
-      <c r="K12" s="16" t="s">
+      <c r="K12" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L12" s="5"/>
@@ -2971,15 +2988,15 @@
         <v>276</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J13" s="3">
         <v>12</v>
       </c>
-      <c r="K13" s="16" t="s">
+      <c r="K13" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3006,15 +3023,15 @@
         <v>276</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J14" s="2">
         <v>67</v>
       </c>
-      <c r="K14" s="16" t="s">
+      <c r="K14" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L14" s="5"/>
@@ -3042,15 +3059,15 @@
         <v>276</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
-      <c r="K15" s="17" t="s">
+      <c r="K15" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L15" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
@@ -3076,11 +3093,11 @@
         <v>276</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
-      <c r="K16" s="16" t="s">
+      <c r="K16" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L16" s="5"/>
@@ -3108,15 +3125,15 @@
         <v>276</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J17" s="3">
         <v>16</v>
       </c>
-      <c r="K17" s="16" t="s">
+      <c r="K17" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3143,11 +3160,11 @@
         <v>276</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
-      <c r="K18" s="16" t="s">
+      <c r="K18" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L18" s="5"/>
@@ -3175,19 +3192,19 @@
         <v>276</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="J19" s="3">
         <v>2</v>
       </c>
-      <c r="K19" s="17" t="s">
+      <c r="K19" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L19" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
@@ -3213,15 +3230,15 @@
         <v>276</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J20" s="2">
         <v>17</v>
       </c>
-      <c r="K20" s="16" t="s">
+      <c r="K20" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L20" s="5"/>
@@ -3249,15 +3266,15 @@
         <v>276</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="J21" s="3">
         <v>1</v>
       </c>
-      <c r="K21" s="16" t="s">
+      <c r="K21" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3284,15 +3301,15 @@
         <v>276</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J22" s="2">
         <v>17</v>
       </c>
-      <c r="K22" s="16" t="s">
+      <c r="K22" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L22" s="5"/>
@@ -3320,19 +3337,19 @@
         <v>276</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="J23" s="3">
         <v>3</v>
       </c>
-      <c r="K23" s="17" t="s">
+      <c r="K23" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L23" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
@@ -3358,11 +3375,11 @@
         <v>276</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
-      <c r="K24" s="16" t="s">
+      <c r="K24" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L24" s="5"/>
@@ -3390,15 +3407,15 @@
         <v>276</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J25" s="3">
         <v>28</v>
       </c>
-      <c r="K25" s="16" t="s">
+      <c r="K25" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3425,19 +3442,19 @@
         <v>276</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="J26" s="2">
         <v>758</v>
       </c>
-      <c r="K26" s="17" t="s">
+      <c r="K26" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L26" s="5" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
@@ -3463,15 +3480,15 @@
         <v>276</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J27" s="3">
         <v>31</v>
       </c>
-      <c r="K27" s="16" t="s">
+      <c r="K27" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3498,15 +3515,15 @@
         <v>276</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
-      <c r="K28" s="17" t="s">
+      <c r="K28" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L28" s="5" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
@@ -3532,15 +3549,15 @@
         <v>276</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J29" s="3">
         <v>3</v>
       </c>
-      <c r="K29" s="16" t="s">
+      <c r="K29" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3567,15 +3584,15 @@
         <v>276</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J30" s="2">
         <v>35</v>
       </c>
-      <c r="K30" s="16" t="s">
+      <c r="K30" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L30" s="5"/>
@@ -3603,15 +3620,15 @@
         <v>276</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J31" s="3">
         <v>36</v>
       </c>
-      <c r="K31" s="16" t="s">
+      <c r="K31" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3638,15 +3655,15 @@
         <v>276</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J32" s="2">
         <v>35</v>
       </c>
-      <c r="K32" s="16" t="s">
+      <c r="K32" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L32" s="5"/>
@@ -3674,15 +3691,15 @@
         <v>276</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J33" s="3">
         <v>35</v>
       </c>
-      <c r="K33" s="16" t="s">
+      <c r="K33" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3709,15 +3726,15 @@
         <v>276</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
-      <c r="K34" s="17" t="s">
+      <c r="K34" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L34" s="5" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
@@ -3743,15 +3760,15 @@
         <v>276</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="J35" s="3">
         <v>293</v>
       </c>
-      <c r="K35" s="16" t="s">
+      <c r="K35" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3778,15 +3795,15 @@
         <v>276</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J36" s="2">
         <v>35</v>
       </c>
-      <c r="K36" s="16" t="s">
+      <c r="K36" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L36" s="5"/>
@@ -3814,15 +3831,15 @@
         <v>276</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="I37" s="3"/>
       <c r="J37" s="3"/>
-      <c r="K37" s="17" t="s">
+      <c r="K37" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L37" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
@@ -3848,15 +3865,15 @@
         <v>276</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
-      <c r="K38" s="17" t="s">
+      <c r="K38" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L38" s="5" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
@@ -3882,15 +3899,15 @@
         <v>276</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J39" s="3">
         <v>58</v>
       </c>
-      <c r="K39" s="16" t="s">
+      <c r="K39" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3917,15 +3934,15 @@
         <v>276</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J40" s="2">
         <v>84</v>
       </c>
-      <c r="K40" s="16" t="s">
+      <c r="K40" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L40" s="5"/>
@@ -3953,15 +3970,15 @@
         <v>276</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="J41" s="3">
         <v>890</v>
       </c>
-      <c r="K41" s="16" t="s">
+      <c r="K41" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -3988,19 +4005,19 @@
         <v>276</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="J42" s="2">
         <v>145</v>
       </c>
-      <c r="K42" s="17" t="s">
+      <c r="K42" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L42" s="5" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.3">
@@ -4026,19 +4043,19 @@
         <v>276</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="J43" s="3">
         <v>2</v>
       </c>
-      <c r="K43" s="17" t="s">
+      <c r="K43" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L43" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.3">
@@ -4064,19 +4081,19 @@
         <v>276</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J44" s="2">
         <v>74</v>
       </c>
-      <c r="K44" s="17" t="s">
+      <c r="K44" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L44" s="5" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.3">
@@ -4102,15 +4119,15 @@
         <v>276</v>
       </c>
       <c r="H45" s="12" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="I45" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J45" s="3">
         <v>74</v>
       </c>
-      <c r="K45" s="16" t="s">
+      <c r="K45" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -4137,15 +4154,15 @@
         <v>276</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J46" s="2">
         <v>177</v>
       </c>
-      <c r="K46" s="16" t="s">
+      <c r="K46" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L46" s="5"/>
@@ -4173,19 +4190,19 @@
         <v>276</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="J47" s="3">
         <v>9</v>
       </c>
-      <c r="K47" s="17" t="s">
+      <c r="K47" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L47" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
@@ -4211,15 +4228,15 @@
         <v>276</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="J48" s="2">
         <v>10</v>
       </c>
-      <c r="K48" s="16" t="s">
+      <c r="K48" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L48" s="5"/>
@@ -4247,15 +4264,15 @@
         <v>276</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J49" s="3">
         <v>94</v>
       </c>
-      <c r="K49" s="16" t="s">
+      <c r="K49" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -4282,15 +4299,15 @@
         <v>276</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
-      <c r="K50" s="17" t="s">
+      <c r="K50" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.3">
@@ -4316,11 +4333,11 @@
         <v>276</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="I51" s="3"/>
       <c r="J51" s="3"/>
-      <c r="K51" s="16" t="s">
+      <c r="K51" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -4347,11 +4364,11 @@
         <v>276</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
-      <c r="K52" s="16" t="s">
+      <c r="K52" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L52" s="5"/>
@@ -4382,12 +4399,12 @@
         <v>251</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J53" s="3">
         <v>233</v>
       </c>
-      <c r="K53" s="16" t="s">
+      <c r="K53" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -4414,15 +4431,15 @@
         <v>276</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
-      <c r="K54" s="17" t="s">
+      <c r="K54" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.3">
@@ -4448,15 +4465,15 @@
         <v>276</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="I55" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J55" s="3">
         <v>248</v>
       </c>
-      <c r="K55" s="16" t="s">
+      <c r="K55" s="13" t="s">
         <v>283</v>
       </c>
     </row>
@@ -4483,15 +4500,15 @@
         <v>276</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J56" s="2">
         <v>47</v>
       </c>
-      <c r="K56" s="16" t="s">
+      <c r="K56" s="13" t="s">
         <v>283</v>
       </c>
       <c r="L56" s="5"/>
@@ -4519,19 +4536,19 @@
         <v>276</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="J57" s="3">
         <v>5</v>
       </c>
-      <c r="K57" s="17" t="s">
+      <c r="K57" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L57" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.3">
@@ -4557,19 +4574,19 @@
         <v>276</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="J58" s="2">
         <v>131</v>
       </c>
-      <c r="K58" s="17" t="s">
+      <c r="K58" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L58" s="5" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.3">
@@ -4595,43 +4612,46 @@
         <v>276</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="J59" s="3">
         <v>78</v>
       </c>
-      <c r="K59" s="17" t="s">
+      <c r="K59" s="14" t="s">
         <v>286</v>
       </c>
       <c r="L59" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A60" s="11" t="s">
-        <v>304</v>
-      </c>
-      <c r="K60" s="11" t="s">
-        <v>392</v>
+        <v>404</v>
+      </c>
+      <c r="K60" s="18" t="s">
+        <v>405</v>
+      </c>
+      <c r="L60" s="19" t="s">
+        <v>406</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B61" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="C61" s="15"/>
-      <c r="D61" s="15"/>
-      <c r="E61" s="15"/>
-      <c r="F61" s="15"/>
-      <c r="G61" s="15"/>
-      <c r="H61" s="15"/>
-      <c r="I61" s="15"/>
-      <c r="J61" s="15"/>
-      <c r="K61" s="15"/>
-      <c r="L61" s="15"/>
+      <c r="B61" s="16" t="s">
+        <v>387</v>
+      </c>
+      <c r="C61" s="17"/>
+      <c r="D61" s="17"/>
+      <c r="E61" s="17"/>
+      <c r="F61" s="17"/>
+      <c r="G61" s="17"/>
+      <c r="H61" s="17"/>
+      <c r="I61" s="17"/>
+      <c r="J61" s="17"/>
+      <c r="K61" s="17"/>
+      <c r="L61" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
qa_test: FINAL SCORE rows with green/red pass/fail cells
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF4EF53A-D5D2-4023-AB5A-CD10AA715C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D107A2F-6E2D-4103-A9D0-998D71258CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
   <sheets>
     <sheet name="Impose - Auto Page Numbering" sheetId="1" r:id="rId1"/>
@@ -1390,7 +1390,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1406,13 +1406,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1984,10 +1985,10 @@
       <c r="A8" s="11" t="s">
         <v>396</v>
       </c>
-      <c r="K8" s="18" t="s">
+      <c r="K8" s="15" t="s">
         <v>397</v>
       </c>
-      <c r="L8" s="19" t="s">
+      <c r="L8" s="16" t="s">
         <v>398</v>
       </c>
     </row>
@@ -1995,19 +1996,19 @@
       <c r="A9" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="17" t="s">
         <v>295</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="15"/>
-      <c r="L9" s="15"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2229,10 +2230,10 @@
       <c r="A7" s="11" t="s">
         <v>399</v>
       </c>
-      <c r="K7" s="18" t="s">
+      <c r="K7" s="15" t="s">
         <v>400</v>
       </c>
-      <c r="L7" s="19" t="s">
+      <c r="L7" s="16" t="s">
         <v>401</v>
       </c>
     </row>
@@ -2240,19 +2241,19 @@
       <c r="A8" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="17" t="s">
         <v>304</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="15"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="17"/>
+      <c r="L8" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2497,27 +2498,27 @@
       <c r="A8" s="11" t="s">
         <v>402</v>
       </c>
-      <c r="K8" s="18" t="s">
+      <c r="K8" s="15" t="s">
         <v>400</v>
       </c>
-      <c r="L8" s="19" t="s">
+      <c r="L8" s="16" t="s">
         <v>403</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="18" t="s">
         <v>395</v>
       </c>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2529,7 +2530,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED61EE79-1B75-41E6-BD8B-15990556690E}">
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
@@ -4628,34 +4629,47 @@
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A60" s="11" t="s">
+      <c r="A60" s="20"/>
+      <c r="B60" s="20"/>
+      <c r="C60" s="20"/>
+      <c r="D60" s="20"/>
+      <c r="E60" s="20"/>
+      <c r="F60" s="20"/>
+      <c r="G60" s="20"/>
+      <c r="H60" s="20"/>
+      <c r="I60" s="20"/>
+      <c r="J60" s="20"/>
+      <c r="K60" s="20"/>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A61" s="11" t="s">
         <v>404</v>
       </c>
-      <c r="K60" s="18" t="s">
+      <c r="K61" s="15" t="s">
         <v>405</v>
       </c>
-      <c r="L60" s="19" t="s">
+      <c r="L61" s="16" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B61" s="16" t="s">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B62" s="18" t="s">
         <v>387</v>
       </c>
-      <c r="C61" s="17"/>
-      <c r="D61" s="17"/>
-      <c r="E61" s="17"/>
-      <c r="F61" s="17"/>
-      <c r="G61" s="17"/>
-      <c r="H61" s="17"/>
-      <c r="I61" s="17"/>
-      <c r="J61" s="17"/>
-      <c r="K61" s="17"/>
-      <c r="L61" s="17"/>
+      <c r="C62" s="19"/>
+      <c r="D62" s="19"/>
+      <c r="E62" s="19"/>
+      <c r="F62" s="19"/>
+      <c r="G62" s="19"/>
+      <c r="H62" s="19"/>
+      <c r="I62" s="19"/>
+      <c r="J62" s="19"/>
+      <c r="K62" s="19"/>
+      <c r="L62" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B61:L61"/>
+    <mergeCell ref="B62:L62"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Task 3: add 10 new Q&A sheets (68 questions, cols A-G) for batch 2 scored docs
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -1,22 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D107A2F-6E2D-4103-A9D0-998D71258CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB1069B3-BF96-4C42-89D0-9978812D5226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="10" activeTab="13" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
   <sheets>
     <sheet name="Impose - Auto Page Numbering" sheetId="1" r:id="rId1"/>
     <sheet name="Impose - Folding Arrow" sheetId="2" r:id="rId2"/>
     <sheet name="InkDrive - CIP3 Presets" sheetId="3" r:id="rId3"/>
     <sheet name="ProductionCenter UG" sheetId="4" r:id="rId4"/>
+    <sheet name="DQS - Digital QuickStrip" sheetId="5" r:id="rId5"/>
+    <sheet name="Lesson 26 - Number-Up C&amp;A" sheetId="6" r:id="rId6"/>
+    <sheet name="PC - Passkeys" sheetId="7" r:id="rId7"/>
+    <sheet name="PC - Approve Reject Pages" sheetId="8" r:id="rId8"/>
+    <sheet name="Proofing - GDI &amp; Split4Proof" sheetId="9" r:id="rId9"/>
+    <sheet name="Packaging - Packaging Pack" sheetId="10" r:id="rId10"/>
+    <sheet name="WebApproval - Softproof" sheetId="11" r:id="rId11"/>
+    <sheet name="Security - Virus Scanning" sheetId="12" r:id="rId12"/>
+    <sheet name="PC - Production Dashboard" sheetId="13" r:id="rId13"/>
+    <sheet name="PC - Enhanced Collaboration" sheetId="14" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1392" uniqueCount="655">
   <si>
     <t>ID</t>
   </si>
@@ -1263,6 +1273,750 @@
   </si>
   <si>
     <t>20 Fail</t>
+  </si>
+  <si>
+    <t>DQS-001</t>
+  </si>
+  <si>
+    <t>Intro, p.1</t>
+  </si>
+  <si>
+    <t>What is Digital QuickStrip (DQS) in Apogee Prepress?</t>
+  </si>
+  <si>
+    <t>DQS renders each page or element individually before combining them into a final composed layout within the Apogee Prepress system, allowing for greater control and efficiency.</t>
+  </si>
+  <si>
+    <t>DQS-002</t>
+  </si>
+  <si>
+    <t>Key Features, p.1</t>
+  </si>
+  <si>
+    <t>How does Digital QuickStrip differ from traditional workflow imposition in Apogee?</t>
+  </si>
+  <si>
+    <t>In traditional workflows, an entire imposed file is rendered at once. With DQS, imposition occurs after rendering—pages are processed separately and then assembled into the final layout, simplifying adjustments and reducing processing demands.</t>
+  </si>
+  <si>
+    <t>DQS-003</t>
+  </si>
+  <si>
+    <t>ROOM Principle, p.1</t>
+  </si>
+  <si>
+    <t>What is the ROOM principle in Apogee DQS?</t>
+  </si>
+  <si>
+    <t>ROOM stands for Render Once, Output Many. For step-and-repeat jobs, DQS renders the object just once and duplicates it across the layout, ensuring consistency and speeding up production by avoiding redundant rendering.</t>
+  </si>
+  <si>
+    <t>DQS-004</t>
+  </si>
+  <si>
+    <t>What are the key features of Digital QuickStrip in Apogee Prepress?</t>
+  </si>
+  <si>
+    <t>DQS provides: individual page rendering before compositing; post-rendering imposition (pages assembled after rendering); and the ROOM principle (Render Once, Output Many) for step-and-repeat jobs, ensuring consistency and faster production.</t>
+  </si>
+  <si>
+    <t>DQS-005</t>
+  </si>
+  <si>
+    <t>Is Digital QuickStrip included by default or is it a chargeable option in Apogee Prepress?</t>
+  </si>
+  <si>
+    <t>Digital QuickStrip (DQS) is a chargeable option in Apogee Prepress.</t>
+  </si>
+  <si>
+    <t>L26-001</t>
+  </si>
+  <si>
+    <t>What is the difference between Number-up Binding and Number-up Cut and Assemble in Apogee Impose?</t>
+  </si>
+  <si>
+    <t>Number-up Binding: multiple book signatures on a fold sheet are folded together, then assembled, then cut apart. Number-up Cut and Assemble: multiple book signatures are folded together, cut apart first, and then assembled in numerical order.</t>
+  </si>
+  <si>
+    <t>L26-002</t>
+  </si>
+  <si>
+    <t>Section 1, p.4</t>
+  </si>
+  <si>
+    <t>What Print &amp; Fold and Number Up settings are required in Auto Impose for a 2-up Cut &amp; Assemble job?</t>
+  </si>
+  <si>
+    <t>Print &amp; Fold tab: Press = Large Press; Sheet Size = 1000 x 650 mm; Folding scheme = Default Set. Number Up tab: Main Number Up Scheme = 2-up C&amp;A. The product is automatically assigned to this scheme.</t>
+  </si>
+  <si>
+    <t>L26-003</t>
+  </si>
+  <si>
+    <t>How do you create a 2-up Cut &amp; Assemble job from a template in Apogee Impose?</t>
+  </si>
+  <si>
+    <t>Select File &gt; New from Templates (Ctrl+N), select the Apogee Impose Template from the Tutorial Category, enter Order Number and Job Name, set copies to 50,000, set Product Type to Bound Stacked Coated A4 with 128 pages and A5 body size. Use Auto Impose with 2-up C&amp;A as the Number Up Scheme, then click Impose.</t>
+  </si>
+  <si>
+    <t>L26-004</t>
+  </si>
+  <si>
+    <t>Cut and Assemble reversed, p.6</t>
+  </si>
+  <si>
+    <t>How do you reverse the book signature positions in a 2-up Cut &amp; Assemble job?</t>
+  </si>
+  <si>
+    <t>Duplicate the existing job, change the Job Name, choose Auto Impose in the Products tab, select '2-up C&amp;A (reversed)' as the main Number Up Scheme in the Number Up tab, and click Impose.</t>
+  </si>
+  <si>
+    <t>L26-005</t>
+  </si>
+  <si>
+    <t>Cut Tumble and Assemble, p.7</t>
+  </si>
+  <si>
+    <t>What Number-Up Scheme should you use when one book signature needs a different orientation from the other?</t>
+  </si>
+  <si>
+    <t>Use the '2-up CT&amp;A' (Cut, Tumble &amp; Assemble) Number-Up Scheme. This tumbles one of the book signatures so it has a different orientation compared to the other. Choose '2-up CT&amp;A (reversed)' if you also need to switch the positions.</t>
+  </si>
+  <si>
+    <t>L26-006</t>
+  </si>
+  <si>
+    <t>Section 2, p.8</t>
+  </si>
+  <si>
+    <t>What is a Multi Product 2-up Cut job in Apogee Impose?</t>
+  </si>
+  <si>
+    <t>A Multi Product 2-up Cut job combines book signatures from multiple products on one fold sheet — for example, Product 1 BS 1 and Product 2 BS 1 together. Each pair is folded together and cut apart, then all book signatures for each product are assembled separately in numerical order.</t>
+  </si>
+  <si>
+    <t>L26-007</t>
+  </si>
+  <si>
+    <t>Section 2, p.9</t>
+  </si>
+  <si>
+    <t>How do you combine two products on the same fold sheet using Auto Impose?</t>
+  </si>
+  <si>
+    <t>In the Products tab, duplicate the first product and rename both. Use Auto Impose, select '2-up C' as the main Number Up Scheme, then select 'Combine products' in the Number Up tab. Product 1 and Product 2 are automatically assigned to Delivery A and B from the 2-up C scheme.</t>
+  </si>
+  <si>
+    <t>L26-008</t>
+  </si>
+  <si>
+    <t>What is the production trade-off when combining two products on the same fold sheet?</t>
+  </si>
+  <si>
+    <t>Combining products significantly reduces plates and press runs (in the example: from 128 to 64 plates, and from 16 to 8 press runs on an 8-color press). However, it may result in an overrun for one product — in the example Product 2 has an overrun of 5,000 copies.</t>
+  </si>
+  <si>
+    <t>L26-009</t>
+  </si>
+  <si>
+    <t>Section 1, p.5</t>
+  </si>
+  <si>
+    <t>How are the 8 book signatures of a 128-page job assigned to fold sheets in a 2-up C&amp;A job?</t>
+  </si>
+  <si>
+    <t>The 8 book signatures of 16 pages each are assigned to fold sheets in numerical order: BS 1 and BS 2 on the first fold sheet, BS 3 and BS 4 on the second, BS 5 and BS 6 on the third, and so on.</t>
+  </si>
+  <si>
+    <t>L26-010</t>
+  </si>
+  <si>
+    <t>Section 3, p.10-12</t>
+  </si>
+  <si>
+    <t>How do you create a job that combines 2-up and 1-up book signatures in the same imposition?</t>
+  </si>
+  <si>
+    <t>Create a new job from the Apogee Impose template with a cover enabled. In Edit Imposition, assign the cover (BS 1) to a 1-up fold scheme (F4-1) on a Small Press. Assign body book signatures to 2-up fold sheets (F16-6) on a Large Press, using Number-Up Schemes such as 2-up C or 2-up CT&amp;A for each fold sheet as needed.</t>
+  </si>
+  <si>
+    <t>PK-001</t>
+  </si>
+  <si>
+    <t>Section 1, p.1</t>
+  </si>
+  <si>
+    <t>What are Passkeys in the context of Apogee v14 WebApproval and WebFlow?</t>
+  </si>
+  <si>
+    <t>Passkeys are a modern, secure, and user-friendly authentication method introduced in Apogee v14 for WebApproval and WebFlow. They are based on public-key cryptography, offering a phishing-resistant and passwordless sign-in experience.</t>
+  </si>
+  <si>
+    <t>PK-002</t>
+  </si>
+  <si>
+    <t>Section 2, p.1</t>
+  </si>
+  <si>
+    <t>What technical requirements must be met to use Passkeys in WebApproval?</t>
+  </si>
+  <si>
+    <t>The system must serve content over HTTPS with a valid TLS certificate (secure context required). Passkeys are tied to the domain used in the SSL certificate, not the specific server IP or hostname.</t>
+  </si>
+  <si>
+    <t>PK-003</t>
+  </si>
+  <si>
+    <t>Section 2-3, p.2-3</t>
+  </si>
+  <si>
+    <t>How does the Passkey authentication process work when logging in to WebApproval?</t>
+  </si>
+  <si>
+    <t>The site sends a challenge to the user's device. The device uses the stored private key to sign the challenge and sends it back. The website verifies the response using the stored public key and the user is logged in. Identity is confirmed via Face ID, Touch ID, or a device PIN.</t>
+  </si>
+  <si>
+    <t>PK-004</t>
+  </si>
+  <si>
+    <t>Section 5, p.5</t>
+  </si>
+  <si>
+    <t>What steps must a user follow to set up Passkeys in WebApproval?</t>
+  </si>
+  <si>
+    <t>The user must first set a password and complete the initial login. Then log in with the password, go to My Profile and Security Settings, and create Passkeys from there. Passkeys are optional and not enforced.</t>
+  </si>
+  <si>
+    <t>PK-005</t>
+  </si>
+  <si>
+    <t>Section 4, p.5</t>
+  </si>
+  <si>
+    <t>What are the benefits of using Passkeys in WebApproval compared to traditional passwords?</t>
+  </si>
+  <si>
+    <t>No passwords to remember; resistant to phishing and data breaches; work across devices and platforms (Apple iOS/macOS, Google Android/Chrome, Microsoft Windows/Edge) via syncing with iCloud Keychain, Google Password Manager, etc.</t>
+  </si>
+  <si>
+    <t>PK-006</t>
+  </si>
+  <si>
+    <t>What happens to existing Passkeys if the WebApproval domain or subdomain is changed?</t>
+  </si>
+  <si>
+    <t>If the domain or subdomain is changed, existing Passkeys will break and must be re-created by each end-user, because Passkeys are tied to the domain used in the SSL certificate.</t>
+  </si>
+  <si>
+    <t>ARP-001</t>
+  </si>
+  <si>
+    <t>Section 1.1, p.1</t>
+  </si>
+  <si>
+    <t>What is the difference between Direct Approval and Multi Approval in ProductionCenter?</t>
+  </si>
+  <si>
+    <t>Direct Approval: as soon as 1 approver approves a page, it is approved. Multi Approval: all approvers must approve before the page is approved; if any approver rejects, the page is rejected for all users.</t>
+  </si>
+  <si>
+    <t>ARP-002</t>
+  </si>
+  <si>
+    <t>Section 1.2, p.1</t>
+  </si>
+  <si>
+    <t>What is Final Approval in ProductionCenter?</t>
+  </si>
+  <si>
+    <t>Final Approval is the last step in the approval process used to sign off pages for production. The printer company sets one or more final approvers; as soon as one of them approves a page, it becomes final approved and goes into production.</t>
+  </si>
+  <si>
+    <t>ARP-003</t>
+  </si>
+  <si>
+    <t>Section 2, p.3</t>
+  </si>
+  <si>
+    <t>How can you open a job for page inspection in ProductionCenter?</t>
+  </si>
+  <si>
+    <t>Click the link in the notification email to open the job in the flipbook, or log on to ProductionCenter, open the Jobs window in tile or list view, and click the job for which you need to approve pages.</t>
+  </si>
+  <si>
+    <t>ARP-004</t>
+  </si>
+  <si>
+    <t>Section 3.1, p.4-5</t>
+  </si>
+  <si>
+    <t>How do you approve or reject a page using the Actions panel in the flipbook?</t>
+  </si>
+  <si>
+    <t>Go to the page or spread, click the Approve or Reject button. A confirmation dialog appears. For rejection, enter a reason and click Reject. For approval, click Approve. Approved pages receive an Approved icon; rejected pages receive a Rejected icon and a red diagonal line.</t>
+  </si>
+  <si>
+    <t>ARP-005</t>
+  </si>
+  <si>
+    <t>Section 3.1, p.5</t>
+  </si>
+  <si>
+    <t>What does the Quick Approval button do, and when does it appear blue?</t>
+  </si>
+  <si>
+    <t>Quick Approval approves the current page or spread without a confirmation dialog and moves directly to the next page ready for inspection. It appears blue when on a page that cannot be approved because it was already approved or rejected.</t>
+  </si>
+  <si>
+    <t>ARP-006</t>
+  </si>
+  <si>
+    <t>Section 3.2, p.5</t>
+  </si>
+  <si>
+    <t>How do you approve or reject a page using the Actions menu in the flipbook?</t>
+  </si>
+  <si>
+    <t>Right-click on the page to display the Actions menu, then choose Approve/Reject Page or Approve/Reject Visible Pages. Note: approving via the Actions menu has no confirmation dialog; for rejection a reason must still be entered.</t>
+  </si>
+  <si>
+    <t>ARP-007</t>
+  </si>
+  <si>
+    <t>Section 3.3, p.6</t>
+  </si>
+  <si>
+    <t>How do you approve all remaining pages at once in the flipbook?</t>
+  </si>
+  <si>
+    <t>Click the cogwheel in the flipbook and select 'Approve All Remaining Pages', then click Approve to confirm.</t>
+  </si>
+  <si>
+    <t>ARP-008</t>
+  </si>
+  <si>
+    <t>Section 5.1, p.9</t>
+  </si>
+  <si>
+    <t>Can an approver approve a page that was previously rejected in ProductionCenter?</t>
+  </si>
+  <si>
+    <t>Only if the Job Rights setting 'Approvers can approve rejected pages' is enabled for their company. If disabled, a new file must be uploaded to replace the rejected page, or the Printer Company must be contacted.</t>
+  </si>
+  <si>
+    <t>ARP-009</t>
+  </si>
+  <si>
+    <t>Section 5.2, p.9</t>
+  </si>
+  <si>
+    <t>Can an approver reject a page that has already been approved?</t>
+  </si>
+  <si>
+    <t>No. An approver cannot reject an approved page — only users of the Printer Company can do this. If needed, contact the Printer Company to reject an approved page.</t>
+  </si>
+  <si>
+    <t>ARP-010</t>
+  </si>
+  <si>
+    <t>Section 6.2, p.12-13</t>
+  </si>
+  <si>
+    <t>How do you add a Page Remark with an annotation drawing in ProductionCenter?</t>
+  </si>
+  <si>
+    <t>In the Remarks panel of the Flipbook, click 'Add Remark', enter text, then draw an annotation on the page by selecting a tool (rectangle, circle, line, freehand, arrow), choosing a color from the color picker, and adjusting line thickness. The remark is added to the list.</t>
+  </si>
+  <si>
+    <t>ARP-011</t>
+  </si>
+  <si>
+    <t>Section 5.3, p.10-11</t>
+  </si>
+  <si>
+    <t>How do you approve pages in a versioning job in ProductionCenter?</t>
+  </si>
+  <si>
+    <t>Select the desired version using the Versions drop-down in the flipbook navigation, the Versions palette, or the job list. Then use the Approve/Reject buttons in the Actions panel or Actions menu. Depending on versioning setup, a checkbox allows approving/rejecting the same pages in all remaining versions as well.</t>
+  </si>
+  <si>
+    <t>ARP-012</t>
+  </si>
+  <si>
+    <t>How do you show or hide the Approval Progress bar in the flipbook?</t>
+  </si>
+  <si>
+    <t>Press the A key at the top of the flipbook to show or hide the Approval Progress bar.</t>
+  </si>
+  <si>
+    <t>GDI-001</t>
+  </si>
+  <si>
+    <t>What is the Apogee GDI Proofer?</t>
+  </si>
+  <si>
+    <t>The Apogee GDI Proofer uses Microsoft's GDI (Graphics Device Interface) to send layouts and page proofs to Windows-compatible printers, including everyday inkjets and high-end digital presses like HP or Epson models. It is a budget-friendly way to preview impositions or produce quick client proofs without dedicated proofing hardware.</t>
+  </si>
+  <si>
+    <t>GDI-002</t>
+  </si>
+  <si>
+    <t>What is Apogee Split4ProofApogee?</t>
+  </si>
+  <si>
+    <t>Split4ProofApogee is an option in ECO3's Apogee workflow that creates a finished, folded, and imposed proof. It takes the imposition of a print job and splits it into 1-up or 2-up press sheets, preserving all parameters like offsets, rotations, and marks. The result can be output as a rendered PDF for printing on a duplex-capable laser printer or digital press.</t>
+  </si>
+  <si>
+    <t>GDI-003</t>
+  </si>
+  <si>
+    <t>What is the difference between the GDI Proofer and Split4ProofApogee in Apogee Prepress?</t>
+  </si>
+  <si>
+    <t>The GDI Proofer sends layouts or page proofs directly to any Windows-compatible printer using GDI — it is for quick, budget-friendly previews without color calibration. Split4ProofApogee takes the full imposition and splits it into 1-up or 2-up press sheets to produce a physical folded-and-trimmed proof that simulates the final product.</t>
+  </si>
+  <si>
+    <t>GDI-004</t>
+  </si>
+  <si>
+    <t>What output devices does Split4ProofApogee support?</t>
+  </si>
+  <si>
+    <t>Split4ProofApogee supports duplex-capable laser printers and digital presses such as HP Indigo or Xerox iGen. Output can be a rendered PDF or file suitable for printing on these devices, which can then be folded, stapled, and trimmed to simulate the final product.</t>
+  </si>
+  <si>
+    <t>GDI-005</t>
+  </si>
+  <si>
+    <t>What imposition parameters are preserved when Split4ProofApogee splits a job?</t>
+  </si>
+  <si>
+    <t>Split4ProofApogee preserves all parameters from the main imposition flow, including offsets, rotations, and marks.</t>
+  </si>
+  <si>
+    <t>PKG-001</t>
+  </si>
+  <si>
+    <t>Can the existing Apogee Prepress system handle packaging and label production without additional software?</t>
+  </si>
+  <si>
+    <t>Yes. The same Apogee system with the same Task Processors and Client interface can handle packaging and label jobs. No extra tools, new workflows, or new software are required — the Packaging Pack activates this capability on the existing setup.</t>
+  </si>
+  <si>
+    <t>PKG-002</t>
+  </si>
+  <si>
+    <t>What types of output can be produced using the Folded Carton workflow in Apogee Prepress?</t>
+  </si>
+  <si>
+    <t>Folded carton jobs can be produced starting from CAD designs or manually created grids, with support for adding artwork, applying Mark Sets, generating Job Reports, managing spot colors, incorporating product embellishments, and exporting digital cut files for finishing and converting.</t>
+  </si>
+  <si>
+    <t>PKG-003</t>
+  </si>
+  <si>
+    <t>Section 1-2, p.1-2</t>
+  </si>
+  <si>
+    <t>What is the difference between Folded Carton and Labels production in Apogee Packaging Pack?</t>
+  </si>
+  <si>
+    <t>Folded Carton jobs start from CAD designs or manually created grids. Label jobs are created from grid-based layouts with automatic auto-filling based on copy count and other technical parameters. Both support artwork, Mark Sets, Job Reports, and digital cut file export, but labels add auto-fill functionality.</t>
+  </si>
+  <si>
+    <t>PKG-004</t>
+  </si>
+  <si>
+    <t>Section 5, p.3</t>
+  </si>
+  <si>
+    <t>How many Packaging tutorials are available on Apogee Network, and how are they organized?</t>
+  </si>
+  <si>
+    <t>There are 17 packaging tutorials on Apogee Network: 1 basic tutorial (Creating a Packaging Job), 7 basic feature tutorials (CAD files, multi-product jobs, snapping, overlaps, marks, double-sided, proofing), and 9 specific feature tutorials (exporting, grids, ink-free zones, templates, PDF processing steps, auto-fill, Amfortis Editor, hot tickets, approvals).</t>
+  </si>
+  <si>
+    <t>PKG-005</t>
+  </si>
+  <si>
+    <t>Section 3, p.2</t>
+  </si>
+  <si>
+    <t>What standard Apogee features also apply to Packaging and Label jobs?</t>
+  </si>
+  <si>
+    <t>All standard Apogee features apply: automation, scalability, processing capabilities, contract proofs, digital soft proofs, ABS or Spir@l screening, InkSaving, SolidTune, platemaking, and digital press output.</t>
+  </si>
+  <si>
+    <t>WA-001</t>
+  </si>
+  <si>
+    <t>Section 2, p.1-2</t>
+  </si>
+  <si>
+    <t>What is the purpose of the Product and Part definition in an Apogee Job Ticket?</t>
+  </si>
+  <si>
+    <t>The Product and Part definition contains information about how the finished product will look (page size, bleed, workstyle). It is entered once and used throughout the Apogee workflow by several Task Processors, including Apogee Impose and WebApproval, ensuring consistent handling across the entire workflow.</t>
+  </si>
+  <si>
+    <t>WA-002</t>
+  </si>
+  <si>
+    <t>Section 2, p.2</t>
+  </si>
+  <si>
+    <t>What setting in the Display TP ensures that WebApproval soft proofs use the correct page size?</t>
+  </si>
+  <si>
+    <t>In the Display TP, set the Output Size option to '&lt;Manual from part&gt;' (the default setting). This makes WebApproval pick up and use the page size values from the Product/Part tab when rendering soft proofs.</t>
+  </si>
+  <si>
+    <t>WA-003</t>
+  </si>
+  <si>
+    <t>Section 3, p.3-4</t>
+  </si>
+  <si>
+    <t>How is the bleed value shown in the WebApproval flipbook?</t>
+  </si>
+  <si>
+    <t>In the flipbook, at the bottom of each page, the bleed value from the Product tab is shown in green, and the PDF trim box value is shown in pink/pinkish color. If they match, no action is needed. If not, the mismatch is immediately visible to the print-buyer.</t>
+  </si>
+  <si>
+    <t>WA-004</t>
+  </si>
+  <si>
+    <t>Section 4, p.6</t>
+  </si>
+  <si>
+    <t>How does Apogee Preflight detect a page size mismatch between an incoming PDF and the intended product size?</t>
+  </si>
+  <si>
+    <t>In the Apogee Preflight parameter set for WebApproval, an Action list reads the intended page size from the Product tab and compares it to the actual PDF page size during preflighting. When values differ, a notification is automatically posted in the Apogee Client on PDF level.</t>
+  </si>
+  <si>
+    <t>WA-005</t>
+  </si>
+  <si>
+    <t>Section 5, p.7</t>
+  </si>
+  <si>
+    <t>How does WebApproval communicate page size mismatches to the print-buyer?</t>
+  </si>
+  <si>
+    <t>WebApproval displays yellow sticky notes on affected pages. Clicking the sticky note shows a remark explaining the issue. Clicking the red triangle opens an online help webpage. In the flipbook, a green solid line shows the intended page size and a pinkish dashed line shows the actual PDF trim box size.</t>
+  </si>
+  <si>
+    <t>WA-006</t>
+  </si>
+  <si>
+    <t>How can a print-buyer identify missing bleed in WebApproval?</t>
+  </si>
+  <si>
+    <t>In the flipbook, the bleed value from the Product tab is shown in green alongside the PDF trim box value in pink at the bottom of each page. If no bleed was foreseen by the designer, the mismatch between the two values is immediately visible, and the print-buyer can reject the affected pages.</t>
+  </si>
+  <si>
+    <t>WA-007</t>
+  </si>
+  <si>
+    <t>Measure section, p.9</t>
+  </si>
+  <si>
+    <t>How do you activate the Measure tool in the WebApproval flipbook?</t>
+  </si>
+  <si>
+    <t>Click the Cog wheel and select the Measure option, or use the shortcut 'V'. With the tool active, you can measure distances and the measured values are shown in the bottom area of the flipbook.</t>
+  </si>
+  <si>
+    <t>WA-008</t>
+  </si>
+  <si>
+    <t>Section 4-5, p.6-7</t>
+  </si>
+  <si>
+    <t>What control options does Apogee offer for handling Preflight errors in a WebApproval job?</t>
+  </si>
+  <si>
+    <t>Within each job, Apogee Preflight can report errors/warnings, refuse page placement, or automatically reject pages with errors. WebApproval then surfaces these issues to the print-buyer via yellow sticky notes at job and page level.</t>
+  </si>
+  <si>
+    <t>VS-001</t>
+  </si>
+  <si>
+    <t>Why is virus scanning important for Apogee and Amfortis production servers?</t>
+  </si>
+  <si>
+    <t>Virus scanning is critical for safeguarding production servers like Apogee/Amfortis and web portals such as WebApproval/WebFlow. It helps prevent production disruptions, malware infections, ransomware attacks, and spyware, protecting operations, customer trust, and business continuity.</t>
+  </si>
+  <si>
+    <t>VS-002</t>
+  </si>
+  <si>
+    <t>p.1</t>
+  </si>
+  <si>
+    <t>What are the risks of enabling a virus scanner without proper configuration on an Apogee system?</t>
+  </si>
+  <si>
+    <t>Badly configured virus scanning will negatively impact Apogee/Amfortis performance, slowing down processing, client interaction, and file handling. Uncontrolled scanning can also interrupt software updates or stop Apogee/Amfortis entirely. Scanning must be configured carefully with proper exclusions and tuning.</t>
+  </si>
+  <si>
+    <t>VS-003</t>
+  </si>
+  <si>
+    <t>What should you do before enabling virus scanning on an Apogee production server?</t>
+  </si>
+  <si>
+    <t>Always contact ECO3 Service before enabling any virus scanning. The ECO3 service team will provide all required guidance on how to properly set up and tune the virus protection software. Ensure your local IT team is aware they must not enable scanning without proper tuning.</t>
+  </si>
+  <si>
+    <t>VS-004</t>
+  </si>
+  <si>
+    <t>How do modern virus scanners minimize performance overhead on Apogee systems?</t>
+  </si>
+  <si>
+    <t>Modern scanners use optimized engines, caching, and real-time monitoring that focuses only on relevant changes. With proper configuration, performance impact remains low while significantly improving overall system security.</t>
+  </si>
+  <si>
+    <t>VS-005</t>
+  </si>
+  <si>
+    <t>What types of threats does virus scanning protect against on Apogee production servers?</t>
+  </si>
+  <si>
+    <t>Virus scanning protects against malware infections, ransomware attacks, spyware, and other harmful files that could cause production disruptions, downtime, data loss, or security breaches.</t>
+  </si>
+  <si>
+    <t>PD-001</t>
+  </si>
+  <si>
+    <t>What is the ECO3 Production Dashboard?</t>
+  </si>
+  <si>
+    <t>The ECO3 Production Dashboard is a browser-based tool providing a clear overview of production data. It tracks performance across PlateSetters, Proofers, and Digital Presses, monitors consumable usage and costs, analyzes trends with customizable time filters, and visualizes data with charts and graphs.</t>
+  </si>
+  <si>
+    <t>PD-002</t>
+  </si>
+  <si>
+    <t>Viewing section, p.1</t>
+  </si>
+  <si>
+    <t>What production data does the ECO3 Production Dashboard display for each output category?</t>
+  </si>
+  <si>
+    <t>For each category (PlateSetters, Proofers, Digital Presses), the dashboard displays: number of jobs processed, amount of consumables used (plates/proofs), and total imageable area in metric or imperial units.</t>
+  </si>
+  <si>
+    <t>PD-003</t>
+  </si>
+  <si>
+    <t>Export section, p.2</t>
+  </si>
+  <si>
+    <t>How do you export production data from the ECO3 Production Dashboard?</t>
+  </si>
+  <si>
+    <t>Click the three dots in the top-right corner of a data tile, then select Download CSV to save the data locally.</t>
+  </si>
+  <si>
+    <t>PD-004</t>
+  </si>
+  <si>
+    <t>Access section, p.3</t>
+  </si>
+  <si>
+    <t>How do you access the ECO3 Production Dashboard?</t>
+  </si>
+  <si>
+    <t>The dashboard is accessible via the secure link dashboard.eco3.net/. ECO3 handles all hosting, security, and maintenance, so no infrastructure management is required from the user side.</t>
+  </si>
+  <si>
+    <t>PD-005</t>
+  </si>
+  <si>
+    <t>What time filtering option is available in the ECO3 Production Dashboard?</t>
+  </si>
+  <si>
+    <t>The dashboard supports a fully customizable time filter, for example allowing you to view production data from the last 30 days.</t>
+  </si>
+  <si>
+    <t>EC-001</t>
+  </si>
+  <si>
+    <t>What enhancement was made to the Remarks feature in WebApproval with Apogee v14?</t>
+  </si>
+  <si>
+    <t>With Apogee v14, an 'Add Page Remark' icon was added to the side toolbar in WebApproval. This usability enhancement quickly opens the Remarks palette, making the annotation and remarking process more accessible and visible.</t>
+  </si>
+  <si>
+    <t>EC-002</t>
+  </si>
+  <si>
+    <t>What new annotation tools were added to WebApproval in Apogee v14?</t>
+  </si>
+  <si>
+    <t>New tools added: Oval/Circle (hold Shift for perfect circle), Line, Freehand, and Arrow. These are in addition to the existing Rectangle/Square tool. All tools are accessible via a floating panel.</t>
+  </si>
+  <si>
+    <t>EC-003</t>
+  </si>
+  <si>
+    <t>How can users customize the appearance of annotation tools in WebApproval?</t>
+  </si>
+  <si>
+    <t>Users can choose from 18 colors using the Color Picker, and adjust line thickness using a slider.</t>
+  </si>
+  <si>
+    <t>EC-004</t>
+  </si>
+  <si>
+    <t>Section 3, p.6</t>
+  </si>
+  <si>
+    <t>How does the notification and feedback loop work for page remarks in WebApproval?</t>
+  </si>
+  <si>
+    <t>Each page remark can trigger an email and/or notification (depending on configuration) directed to both the Print Buyer and the Customer Service Representative (CSR). When the Prepress operator replies in the Apogee Client, all parties are automatically informed again via email and/or notification.</t>
+  </si>
+  <si>
+    <t>EC-005</t>
+  </si>
+  <si>
+    <t>Section 4, p.7</t>
+  </si>
+  <si>
+    <t>How does the Remarks feature integrate with the Apogee Client in WebApproval?</t>
+  </si>
+  <si>
+    <t>In the Display flow of the Apogee Client, a remark icon is shown, allowing the operator to access the Remarks pane for quick review and interaction. From this pane, the operator can jump directly into Raster Preview by clicking the '1' in the blue circle.</t>
+  </si>
+  <si>
+    <t>EC-006</t>
+  </si>
+  <si>
+    <t>Section 6.1-6.2, p.12</t>
+  </si>
+  <si>
+    <t>What is the difference between a Job Remark and a Page Remark in WebApproval?</t>
+  </si>
+  <si>
+    <t>A Job Remark is a general remark attached to the whole job; it is not possible to reply to it. A Page Remark is attached to a specific page and supports reply functionality and annotation drawing.</t>
+  </si>
+  <si>
+    <t>EC-007</t>
+  </si>
+  <si>
+    <t>Section 2, p.3-5</t>
+  </si>
+  <si>
+    <t>How should different annotation shapes be used for different content types in WebApproval?</t>
+  </si>
+  <si>
+    <t>Rectangles are suited for highlighting images, oval/circle shapes for drawing attention to artwork needing extra work, and line shapes for annotating text areas. This allows stakeholders to communicate clearly about specific page elements.</t>
   </si>
 </sst>
 </file>
@@ -1390,7 +2144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1408,12 +2162,11 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1996,24 +2749,999 @@
       <c r="A9" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="19" t="s">
         <v>295</v>
       </c>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B9:L9"/>
   </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1E2E269-2DD0-4BCB-B449-CA0CF55313AB}">
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="97.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>547</v>
+      </c>
+      <c r="B2" t="s">
+        <v>408</v>
+      </c>
+      <c r="C2" t="s">
+        <v>548</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>549</v>
+      </c>
+      <c r="G2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>550</v>
+      </c>
+      <c r="B3" t="s">
+        <v>463</v>
+      </c>
+      <c r="C3" t="s">
+        <v>551</v>
+      </c>
+      <c r="D3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>552</v>
+      </c>
+      <c r="G3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>553</v>
+      </c>
+      <c r="B4" t="s">
+        <v>554</v>
+      </c>
+      <c r="C4" t="s">
+        <v>555</v>
+      </c>
+      <c r="D4" t="s">
+        <v>127</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>556</v>
+      </c>
+      <c r="G4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>557</v>
+      </c>
+      <c r="B5" t="s">
+        <v>558</v>
+      </c>
+      <c r="C5" t="s">
+        <v>559</v>
+      </c>
+      <c r="D5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>560</v>
+      </c>
+      <c r="G5" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>561</v>
+      </c>
+      <c r="B6" t="s">
+        <v>562</v>
+      </c>
+      <c r="C6" t="s">
+        <v>563</v>
+      </c>
+      <c r="D6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>564</v>
+      </c>
+      <c r="G6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E196AD85-A960-4564-B839-A1B724C18B70}">
+  <dimension ref="A1:L9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="99.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B2" t="s">
+        <v>566</v>
+      </c>
+      <c r="C2" t="s">
+        <v>567</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>568</v>
+      </c>
+      <c r="G2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>569</v>
+      </c>
+      <c r="B3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C3" t="s">
+        <v>571</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>572</v>
+      </c>
+      <c r="G3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>573</v>
+      </c>
+      <c r="B4" t="s">
+        <v>574</v>
+      </c>
+      <c r="C4" t="s">
+        <v>575</v>
+      </c>
+      <c r="D4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>576</v>
+      </c>
+      <c r="G4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>577</v>
+      </c>
+      <c r="B5" t="s">
+        <v>578</v>
+      </c>
+      <c r="C5" t="s">
+        <v>579</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" t="s">
+        <v>580</v>
+      </c>
+      <c r="G5" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>581</v>
+      </c>
+      <c r="B6" t="s">
+        <v>582</v>
+      </c>
+      <c r="C6" t="s">
+        <v>583</v>
+      </c>
+      <c r="D6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>584</v>
+      </c>
+      <c r="G6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>585</v>
+      </c>
+      <c r="B7" t="s">
+        <v>574</v>
+      </c>
+      <c r="C7" t="s">
+        <v>586</v>
+      </c>
+      <c r="D7" t="s">
+        <v>135</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s">
+        <v>587</v>
+      </c>
+      <c r="G7" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>588</v>
+      </c>
+      <c r="B8" t="s">
+        <v>589</v>
+      </c>
+      <c r="C8" t="s">
+        <v>590</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
+        <v>591</v>
+      </c>
+      <c r="G8" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>592</v>
+      </c>
+      <c r="B9" t="s">
+        <v>593</v>
+      </c>
+      <c r="C9" t="s">
+        <v>594</v>
+      </c>
+      <c r="D9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" t="s">
+        <v>595</v>
+      </c>
+      <c r="G9" t="s">
+        <v>276</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E7B2770-532B-410E-AFC3-F238AD862896}">
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="86.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B2" t="s">
+        <v>408</v>
+      </c>
+      <c r="C2" t="s">
+        <v>597</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>598</v>
+      </c>
+      <c r="G2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>599</v>
+      </c>
+      <c r="B3" t="s">
+        <v>600</v>
+      </c>
+      <c r="C3" t="s">
+        <v>601</v>
+      </c>
+      <c r="D3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>602</v>
+      </c>
+      <c r="G3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>603</v>
+      </c>
+      <c r="B4" t="s">
+        <v>600</v>
+      </c>
+      <c r="C4" t="s">
+        <v>604</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>605</v>
+      </c>
+      <c r="G4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>606</v>
+      </c>
+      <c r="B5" t="s">
+        <v>600</v>
+      </c>
+      <c r="C5" t="s">
+        <v>607</v>
+      </c>
+      <c r="D5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" t="s">
+        <v>608</v>
+      </c>
+      <c r="G5" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>609</v>
+      </c>
+      <c r="B6" t="s">
+        <v>600</v>
+      </c>
+      <c r="C6" t="s">
+        <v>610</v>
+      </c>
+      <c r="D6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>611</v>
+      </c>
+      <c r="G6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE2D4BFD-F916-42EB-B81E-4437686F0EBA}">
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="83" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>612</v>
+      </c>
+      <c r="B2" t="s">
+        <v>408</v>
+      </c>
+      <c r="C2" t="s">
+        <v>613</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>614</v>
+      </c>
+      <c r="G2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>615</v>
+      </c>
+      <c r="B3" t="s">
+        <v>616</v>
+      </c>
+      <c r="C3" t="s">
+        <v>617</v>
+      </c>
+      <c r="D3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>618</v>
+      </c>
+      <c r="G3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>619</v>
+      </c>
+      <c r="B4" t="s">
+        <v>620</v>
+      </c>
+      <c r="C4" t="s">
+        <v>621</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>622</v>
+      </c>
+      <c r="G4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>623</v>
+      </c>
+      <c r="B5" t="s">
+        <v>624</v>
+      </c>
+      <c r="C5" t="s">
+        <v>625</v>
+      </c>
+      <c r="D5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>626</v>
+      </c>
+      <c r="G5" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>627</v>
+      </c>
+      <c r="B6" t="s">
+        <v>408</v>
+      </c>
+      <c r="C6" t="s">
+        <v>628</v>
+      </c>
+      <c r="D6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>629</v>
+      </c>
+      <c r="G6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A9AAEA0-A39F-400A-A6E2-3B630AD3B8A5}">
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="81.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>630</v>
+      </c>
+      <c r="B2" t="s">
+        <v>463</v>
+      </c>
+      <c r="C2" t="s">
+        <v>631</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>632</v>
+      </c>
+      <c r="G2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>633</v>
+      </c>
+      <c r="B3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C3" t="s">
+        <v>634</v>
+      </c>
+      <c r="D3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>635</v>
+      </c>
+      <c r="G3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>636</v>
+      </c>
+      <c r="B4" t="s">
+        <v>570</v>
+      </c>
+      <c r="C4" t="s">
+        <v>637</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>638</v>
+      </c>
+      <c r="G4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>639</v>
+      </c>
+      <c r="B5" t="s">
+        <v>640</v>
+      </c>
+      <c r="C5" t="s">
+        <v>641</v>
+      </c>
+      <c r="D5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" t="s">
+        <v>642</v>
+      </c>
+      <c r="G5" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>643</v>
+      </c>
+      <c r="B6" t="s">
+        <v>644</v>
+      </c>
+      <c r="C6" t="s">
+        <v>645</v>
+      </c>
+      <c r="D6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>646</v>
+      </c>
+      <c r="G6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>647</v>
+      </c>
+      <c r="B7" t="s">
+        <v>648</v>
+      </c>
+      <c r="C7" t="s">
+        <v>649</v>
+      </c>
+      <c r="D7" t="s">
+        <v>127</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s">
+        <v>650</v>
+      </c>
+      <c r="G7" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>651</v>
+      </c>
+      <c r="B8" t="s">
+        <v>652</v>
+      </c>
+      <c r="C8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" t="s">
+        <v>654</v>
+      </c>
+      <c r="G8" t="s">
+        <v>276</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2241,19 +3969,19 @@
       <c r="A8" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="19" t="s">
         <v>304</v>
       </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2506,19 +4234,19 @@
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="17" t="s">
         <v>395</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="18"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="18"/>
+      <c r="L9" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4628,19 +6356,6 @@
         <v>386</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A60" s="20"/>
-      <c r="B60" s="20"/>
-      <c r="C60" s="20"/>
-      <c r="D60" s="20"/>
-      <c r="E60" s="20"/>
-      <c r="F60" s="20"/>
-      <c r="G60" s="20"/>
-      <c r="H60" s="20"/>
-      <c r="I60" s="20"/>
-      <c r="J60" s="20"/>
-      <c r="K60" s="20"/>
-    </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A61" s="11" t="s">
         <v>404</v>
@@ -4653,19 +6368,19 @@
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B62" s="18" t="s">
+      <c r="B62" s="17" t="s">
         <v>387</v>
       </c>
-      <c r="C62" s="19"/>
-      <c r="D62" s="19"/>
-      <c r="E62" s="19"/>
-      <c r="F62" s="19"/>
-      <c r="G62" s="19"/>
-      <c r="H62" s="19"/>
-      <c r="I62" s="19"/>
-      <c r="J62" s="19"/>
-      <c r="K62" s="19"/>
-      <c r="L62" s="19"/>
+      <c r="C62" s="18"/>
+      <c r="D62" s="18"/>
+      <c r="E62" s="18"/>
+      <c r="F62" s="18"/>
+      <c r="G62" s="18"/>
+      <c r="H62" s="18"/>
+      <c r="I62" s="18"/>
+      <c r="J62" s="18"/>
+      <c r="K62" s="18"/>
+      <c r="L62" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4673,4 +6388,1163 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECA949DB-6747-4609-92BE-8F7C116C6318}">
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="77.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="218.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>407</v>
+      </c>
+      <c r="B2" t="s">
+        <v>408</v>
+      </c>
+      <c r="C2" t="s">
+        <v>409</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>410</v>
+      </c>
+      <c r="G2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>411</v>
+      </c>
+      <c r="B3" t="s">
+        <v>412</v>
+      </c>
+      <c r="C3" t="s">
+        <v>413</v>
+      </c>
+      <c r="D3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>414</v>
+      </c>
+      <c r="G3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>415</v>
+      </c>
+      <c r="B4" t="s">
+        <v>416</v>
+      </c>
+      <c r="C4" t="s">
+        <v>417</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>418</v>
+      </c>
+      <c r="G4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>419</v>
+      </c>
+      <c r="B5" t="s">
+        <v>412</v>
+      </c>
+      <c r="C5" t="s">
+        <v>420</v>
+      </c>
+      <c r="D5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>421</v>
+      </c>
+      <c r="G5" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>422</v>
+      </c>
+      <c r="B6" t="s">
+        <v>408</v>
+      </c>
+      <c r="C6" t="s">
+        <v>423</v>
+      </c>
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>424</v>
+      </c>
+      <c r="G6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7732661-99F1-4627-B65D-A2763DB3309A}">
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="98.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>425</v>
+      </c>
+      <c r="B2" t="s">
+        <v>408</v>
+      </c>
+      <c r="C2" t="s">
+        <v>426</v>
+      </c>
+      <c r="D2" t="s">
+        <v>127</v>
+      </c>
+      <c r="E2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" t="s">
+        <v>427</v>
+      </c>
+      <c r="G2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>428</v>
+      </c>
+      <c r="B3" t="s">
+        <v>429</v>
+      </c>
+      <c r="C3" t="s">
+        <v>430</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>431</v>
+      </c>
+      <c r="G3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>432</v>
+      </c>
+      <c r="B4" t="s">
+        <v>429</v>
+      </c>
+      <c r="C4" t="s">
+        <v>433</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>434</v>
+      </c>
+      <c r="G4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>435</v>
+      </c>
+      <c r="B5" t="s">
+        <v>436</v>
+      </c>
+      <c r="C5" t="s">
+        <v>437</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" t="s">
+        <v>438</v>
+      </c>
+      <c r="G5" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>439</v>
+      </c>
+      <c r="B6" t="s">
+        <v>440</v>
+      </c>
+      <c r="C6" t="s">
+        <v>441</v>
+      </c>
+      <c r="D6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>442</v>
+      </c>
+      <c r="G6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>443</v>
+      </c>
+      <c r="B7" t="s">
+        <v>444</v>
+      </c>
+      <c r="C7" t="s">
+        <v>445</v>
+      </c>
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s">
+        <v>446</v>
+      </c>
+      <c r="G7" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>447</v>
+      </c>
+      <c r="B8" t="s">
+        <v>448</v>
+      </c>
+      <c r="C8" t="s">
+        <v>449</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>175</v>
+      </c>
+      <c r="F8" t="s">
+        <v>450</v>
+      </c>
+      <c r="G8" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>451</v>
+      </c>
+      <c r="B9" t="s">
+        <v>448</v>
+      </c>
+      <c r="C9" t="s">
+        <v>452</v>
+      </c>
+      <c r="D9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" t="s">
+        <v>175</v>
+      </c>
+      <c r="F9" t="s">
+        <v>453</v>
+      </c>
+      <c r="G9" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>454</v>
+      </c>
+      <c r="B10" t="s">
+        <v>455</v>
+      </c>
+      <c r="C10" t="s">
+        <v>456</v>
+      </c>
+      <c r="D10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" t="s">
+        <v>457</v>
+      </c>
+      <c r="G10" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>458</v>
+      </c>
+      <c r="B11" t="s">
+        <v>459</v>
+      </c>
+      <c r="C11" t="s">
+        <v>460</v>
+      </c>
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" t="s">
+        <v>175</v>
+      </c>
+      <c r="F11" t="s">
+        <v>461</v>
+      </c>
+      <c r="G11" t="s">
+        <v>276</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1703EDB3-442F-4F24-9877-BBF315546A3C}">
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="82.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="237.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>462</v>
+      </c>
+      <c r="B2" t="s">
+        <v>463</v>
+      </c>
+      <c r="C2" t="s">
+        <v>464</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>465</v>
+      </c>
+      <c r="G2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>466</v>
+      </c>
+      <c r="B3" t="s">
+        <v>467</v>
+      </c>
+      <c r="C3" t="s">
+        <v>468</v>
+      </c>
+      <c r="D3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>469</v>
+      </c>
+      <c r="G3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>470</v>
+      </c>
+      <c r="B4" t="s">
+        <v>471</v>
+      </c>
+      <c r="C4" t="s">
+        <v>472</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>473</v>
+      </c>
+      <c r="G4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>474</v>
+      </c>
+      <c r="B5" t="s">
+        <v>475</v>
+      </c>
+      <c r="C5" t="s">
+        <v>476</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" t="s">
+        <v>477</v>
+      </c>
+      <c r="G5" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>478</v>
+      </c>
+      <c r="B6" t="s">
+        <v>479</v>
+      </c>
+      <c r="C6" t="s">
+        <v>480</v>
+      </c>
+      <c r="D6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>481</v>
+      </c>
+      <c r="G6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>482</v>
+      </c>
+      <c r="B7" t="s">
+        <v>467</v>
+      </c>
+      <c r="C7" t="s">
+        <v>483</v>
+      </c>
+      <c r="D7" t="s">
+        <v>135</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s">
+        <v>484</v>
+      </c>
+      <c r="G7" t="s">
+        <v>276</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{528F97EE-0955-480B-AF6B-0088715AB229}">
+  <dimension ref="A1:L13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="77.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>485</v>
+      </c>
+      <c r="B2" t="s">
+        <v>486</v>
+      </c>
+      <c r="C2" t="s">
+        <v>487</v>
+      </c>
+      <c r="D2" t="s">
+        <v>127</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>488</v>
+      </c>
+      <c r="G2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>489</v>
+      </c>
+      <c r="B3" t="s">
+        <v>490</v>
+      </c>
+      <c r="C3" t="s">
+        <v>491</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>492</v>
+      </c>
+      <c r="G3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>493</v>
+      </c>
+      <c r="B4" t="s">
+        <v>494</v>
+      </c>
+      <c r="C4" t="s">
+        <v>495</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>496</v>
+      </c>
+      <c r="G4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B5" t="s">
+        <v>498</v>
+      </c>
+      <c r="C5" t="s">
+        <v>499</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>500</v>
+      </c>
+      <c r="G5" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>501</v>
+      </c>
+      <c r="B6" t="s">
+        <v>502</v>
+      </c>
+      <c r="C6" t="s">
+        <v>503</v>
+      </c>
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>504</v>
+      </c>
+      <c r="G6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>505</v>
+      </c>
+      <c r="B7" t="s">
+        <v>506</v>
+      </c>
+      <c r="C7" t="s">
+        <v>507</v>
+      </c>
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" t="s">
+        <v>508</v>
+      </c>
+      <c r="G7" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>509</v>
+      </c>
+      <c r="B8" t="s">
+        <v>510</v>
+      </c>
+      <c r="C8" t="s">
+        <v>511</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
+        <v>512</v>
+      </c>
+      <c r="G8" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>513</v>
+      </c>
+      <c r="B9" t="s">
+        <v>514</v>
+      </c>
+      <c r="C9" t="s">
+        <v>515</v>
+      </c>
+      <c r="D9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" t="s">
+        <v>516</v>
+      </c>
+      <c r="G9" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>517</v>
+      </c>
+      <c r="B10" t="s">
+        <v>518</v>
+      </c>
+      <c r="C10" t="s">
+        <v>519</v>
+      </c>
+      <c r="D10" t="s">
+        <v>135</v>
+      </c>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" t="s">
+        <v>520</v>
+      </c>
+      <c r="G10" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>521</v>
+      </c>
+      <c r="B11" t="s">
+        <v>522</v>
+      </c>
+      <c r="C11" t="s">
+        <v>523</v>
+      </c>
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" t="s">
+        <v>524</v>
+      </c>
+      <c r="G11" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>525</v>
+      </c>
+      <c r="B12" t="s">
+        <v>526</v>
+      </c>
+      <c r="C12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" t="s">
+        <v>175</v>
+      </c>
+      <c r="F12" t="s">
+        <v>528</v>
+      </c>
+      <c r="G12" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>529</v>
+      </c>
+      <c r="B13" t="s">
+        <v>502</v>
+      </c>
+      <c r="C13" t="s">
+        <v>530</v>
+      </c>
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" t="s">
+        <v>531</v>
+      </c>
+      <c r="G13" t="s">
+        <v>276</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{609488A8-6907-40DE-8767-67C21A25FFCF}">
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="79.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>532</v>
+      </c>
+      <c r="B2" t="s">
+        <v>408</v>
+      </c>
+      <c r="C2" t="s">
+        <v>533</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>534</v>
+      </c>
+      <c r="G2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>535</v>
+      </c>
+      <c r="B3" t="s">
+        <v>408</v>
+      </c>
+      <c r="C3" t="s">
+        <v>536</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>537</v>
+      </c>
+      <c r="G3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>538</v>
+      </c>
+      <c r="B4" t="s">
+        <v>408</v>
+      </c>
+      <c r="C4" t="s">
+        <v>539</v>
+      </c>
+      <c r="D4" t="s">
+        <v>127</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>540</v>
+      </c>
+      <c r="G4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>541</v>
+      </c>
+      <c r="B5" t="s">
+        <v>408</v>
+      </c>
+      <c r="C5" t="s">
+        <v>542</v>
+      </c>
+      <c r="D5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>543</v>
+      </c>
+      <c r="G5" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>544</v>
+      </c>
+      <c r="B6" t="s">
+        <v>408</v>
+      </c>
+      <c r="C6" t="s">
+        <v>545</v>
+      </c>
+      <c r="D6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>546</v>
+      </c>
+      <c r="G6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Task 3: apply header formatting to 10 new Q&A sheets
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB1069B3-BF96-4C42-89D0-9978812D5226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5545384-80C3-4616-B7F1-AC3AE5BDB8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="10" activeTab="13" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
@@ -2144,7 +2144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2162,11 +2162,12 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2749,19 +2750,19 @@
       <c r="A9" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="17" t="s">
         <v>295</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2776,50 +2777,55 @@
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="97.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="75.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="164.33203125" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="174.6640625" customWidth="1"/>
+    <col min="9" max="9" width="29.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="77.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="20" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="20" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="20" t="s">
         <v>278</v>
       </c>
     </row>
@@ -2948,50 +2954,55 @@
   <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="99.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="75.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="164.33203125" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="174.6640625" customWidth="1"/>
+    <col min="9" max="9" width="29.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="77.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="20" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="20" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="20" t="s">
         <v>278</v>
       </c>
     </row>
@@ -3189,50 +3200,55 @@
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="86.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="75.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="164.33203125" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="174.6640625" customWidth="1"/>
+    <col min="9" max="9" width="29.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="77.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="20" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="20" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="20" t="s">
         <v>278</v>
       </c>
     </row>
@@ -3361,50 +3377,55 @@
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="83" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="75.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="164.33203125" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="174.6640625" customWidth="1"/>
+    <col min="9" max="9" width="29.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="77.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="20" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="20" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="20" t="s">
         <v>278</v>
       </c>
     </row>
@@ -3533,50 +3554,55 @@
   <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="81.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="75.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="164.33203125" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="174.6640625" customWidth="1"/>
+    <col min="9" max="9" width="29.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="77.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="20" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="20" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="20" t="s">
         <v>278</v>
       </c>
     </row>
@@ -3969,19 +3995,19 @@
       <c r="A8" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="17" t="s">
         <v>304</v>
       </c>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="19"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="19"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="17"/>
+      <c r="L8" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4234,19 +4260,19 @@
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="18" t="s">
         <v>395</v>
       </c>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="18"/>
-      <c r="L9" s="18"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6368,19 +6394,19 @@
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B62" s="17" t="s">
+      <c r="B62" s="18" t="s">
         <v>387</v>
       </c>
-      <c r="C62" s="18"/>
-      <c r="D62" s="18"/>
-      <c r="E62" s="18"/>
-      <c r="F62" s="18"/>
-      <c r="G62" s="18"/>
-      <c r="H62" s="18"/>
-      <c r="I62" s="18"/>
-      <c r="J62" s="18"/>
-      <c r="K62" s="18"/>
-      <c r="L62" s="18"/>
+      <c r="C62" s="19"/>
+      <c r="D62" s="19"/>
+      <c r="E62" s="19"/>
+      <c r="F62" s="19"/>
+      <c r="G62" s="19"/>
+      <c r="H62" s="19"/>
+      <c r="I62" s="19"/>
+      <c r="J62" s="19"/>
+      <c r="K62" s="19"/>
+      <c r="L62" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6395,50 +6421,55 @@
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="77.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="218.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="75.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="164.33203125" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="174.6640625" customWidth="1"/>
+    <col min="9" max="9" width="29.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="77.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="20" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="20" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="20" t="s">
         <v>278</v>
       </c>
     </row>
@@ -6567,50 +6598,55 @@
   <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="98.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="75.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="164.33203125" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="174.6640625" customWidth="1"/>
+    <col min="9" max="9" width="29.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="77.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="20" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="20" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="20" t="s">
         <v>278</v>
       </c>
     </row>
@@ -6854,50 +6890,55 @@
   <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="82.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="237.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="75.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="164.33203125" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="174.6640625" customWidth="1"/>
+    <col min="9" max="9" width="29.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="77.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="20" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="20" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="20" t="s">
         <v>278</v>
       </c>
     </row>
@@ -7049,50 +7090,55 @@
   <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="77.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="75.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="164.33203125" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="174.6640625" customWidth="1"/>
+    <col min="9" max="9" width="29.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="77.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="20" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="20" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="20" t="s">
         <v>278</v>
       </c>
     </row>
@@ -7382,50 +7428,55 @@
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="79.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="255.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="75.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="164.33203125" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="174.6640625" customWidth="1"/>
+    <col min="9" max="9" width="29.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="77.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="20" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="20" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="20" t="s">
         <v>278</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Task 3: add PrintSphere OLH draft02 sheet — 50 questions (cols A-G)
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5545384-80C3-4616-B7F1-AC3AE5BDB8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FE225D3-3024-4B42-8C74-6971F2556D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="10" activeTab="13" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="11" activeTab="14" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
   <sheets>
     <sheet name="Impose - Auto Page Numbering" sheetId="1" r:id="rId1"/>
@@ -27,6 +27,7 @@
     <sheet name="Security - Virus Scanning" sheetId="12" r:id="rId12"/>
     <sheet name="PC - Production Dashboard" sheetId="13" r:id="rId13"/>
     <sheet name="PC - Enhanced Collaboration" sheetId="14" r:id="rId14"/>
+    <sheet name="PrintSphere OLH - draft02" sheetId="15" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1392" uniqueCount="655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1754" uniqueCount="848">
   <si>
     <t>ID</t>
   </si>
@@ -2017,6 +2018,585 @@
   </si>
   <si>
     <t>Rectangles are suited for highlighting images, oval/circle shapes for drawing attention to artwork needing extra work, and line shapes for annotating text areas. This allows stakeholders to communicate clearly about specific page elements.</t>
+  </si>
+  <si>
+    <t>PS2-001</t>
+  </si>
+  <si>
+    <t>About, p.8</t>
+  </si>
+  <si>
+    <t>PrintSphere is a file-sharing and file-syncing service that stores files in a dedicated space on the printsphere.com server. Files can be shared with registered users via local sharing or with unregistered users via a public link. Users can sync files with a computer and access the service via Webclient, desktop application, or mobile apps.</t>
+  </si>
+  <si>
+    <t>PS2-002</t>
+  </si>
+  <si>
+    <t>What is SphereCenter?</t>
+  </si>
+  <si>
+    <t>SphereCenter is a separate application where the PrintSphere subscription is started, users are created, and storage usage is monitored. It is not covered in the PrintSphere User's Guide — see the SphereCenter Help for instructions.</t>
+  </si>
+  <si>
+    <t>PS2-003</t>
+  </si>
+  <si>
+    <t>About, p.10</t>
+  </si>
+  <si>
+    <t>What browsers are recommended for PrintSphere?</t>
+  </si>
+  <si>
+    <t>Recommended browsers: Google Chrome (recommended), Microsoft Edge (Chromium-based), Mozilla Firefox, and Apple Safari (macOS only). PrintSphere works with all recent Windows, macOS, Android, and Apple iOS operating systems.</t>
+  </si>
+  <si>
+    <t>PS2-004</t>
+  </si>
+  <si>
+    <t>About, p.8-9</t>
+  </si>
+  <si>
+    <t>What is the difference between Manual PrintSphere users and Auto PrintSphere users?</t>
+  </si>
+  <si>
+    <t>Manual PrintSphere users have a full account with log-on credentials and can use the Webclient, desktop application, and mobile apps. Auto PrintSphere users have no account and access shared items via a public internet link without logging in; they cannot use the desktop app or mobile apps.</t>
+  </si>
+  <si>
+    <t>PS2-005</t>
+  </si>
+  <si>
+    <t>Ch.1, p.16</t>
+  </si>
+  <si>
+    <t>How do you sign in to the PrintSphere Webclient for the first time?</t>
+  </si>
+  <si>
+    <t>Open the invitation email and click the sign-up link. Set up your account by entering your details and creating a password. After completing sign-up you are redirected to the PrintSphere Webclient.</t>
+  </si>
+  <si>
+    <t>PS2-006</t>
+  </si>
+  <si>
+    <t>Ch.1, p.19</t>
+  </si>
+  <si>
+    <t>How do you change your PrintSphere password as a Printer Administrator?</t>
+  </si>
+  <si>
+    <t>Click your profile photo or initials in the top right corner, choose Settings. In the Password section on the Personal page, click Reset password. You are redirected to SphereCenter. Log in with your Printer Administrator credentials, click your name in the top right corner, open your Account, enter a new password and click Save.</t>
+  </si>
+  <si>
+    <t>PS2-007</t>
+  </si>
+  <si>
+    <t>Ch.1, p.20</t>
+  </si>
+  <si>
+    <t>How do you change your PrintSphere password as a Regular User?</t>
+  </si>
+  <si>
+    <t>Click your profile photo or initials in the top right corner, choose Settings. In the left panel select Password. Enter your current password, then your new password, and click Change password. The password must be at least 11 characters long.</t>
+  </si>
+  <si>
+    <t>PS2-008</t>
+  </si>
+  <si>
+    <t>Ch.1, p.22</t>
+  </si>
+  <si>
+    <t>How do you reset a forgotten PrintSphere password?</t>
+  </si>
+  <si>
+    <t>On the PrintSphere log-on page, click Forgot password. Enter your e-mail address and click Reset password. You will receive an email with a link to set a new password. If you are a Printer Administrator, you are redirected to SphereCenter to complete the reset.</t>
+  </si>
+  <si>
+    <t>PS2-009</t>
+  </si>
+  <si>
+    <t>Ch.1, p.19-20</t>
+  </si>
+  <si>
+    <t>What is the difference between changing a password as a Printer Administrator versus a Regular User in PrintSphere?</t>
+  </si>
+  <si>
+    <t>A Printer Administrator must go to SphereCenter to change their password — clicking Reset password in Settings redirects them there. A Regular User changes their password directly in PrintSphere Settings by selecting Password in the left panel and entering current and new passwords.</t>
+  </si>
+  <si>
+    <t>PS2-010</t>
+  </si>
+  <si>
+    <t>Ch.1, p.21</t>
+  </si>
+  <si>
+    <t>Can a user change their user name or e-mail address in PrintSphere?</t>
+  </si>
+  <si>
+    <t>No. The user name and e-mail address are part of the log-on credentials and cannot be changed by the user. The user must ask their administrator to make these changes.</t>
+  </si>
+  <si>
+    <t>PS2-011</t>
+  </si>
+  <si>
+    <t>Ch.1, p.24-26</t>
+  </si>
+  <si>
+    <t>What information can a user manage on the Personal page in PrintSphere?</t>
+  </si>
+  <si>
+    <t>Users can manage: profile picture, full name and its visibility, location and its visibility, language and locale preferences, password, and notification settings (email and/or online stream). Group memberships are shown but are read-only.</t>
+  </si>
+  <si>
+    <t>PS2-012</t>
+  </si>
+  <si>
+    <t>Ch.1, p.24</t>
+  </si>
+  <si>
+    <t>How do you access Profile and Preferences settings in PrintSphere?</t>
+  </si>
+  <si>
+    <t>Click your profile photo or initials in the top right corner on the menu bar and choose Settings. This opens the Personal page where you can view and edit your profile and preferences.</t>
+  </si>
+  <si>
+    <t>PS2-013</t>
+  </si>
+  <si>
+    <t>Ch.1, p.28</t>
+  </si>
+  <si>
+    <t>How do you download the PrintSphere desktop or mobile app from within the Webclient?</t>
+  </si>
+  <si>
+    <t>Click your profile photo or initials in the top right corner, choose Settings to go to the Personal page. Click Get the Desktop and Mobile Apps and click the download link for your operating system or app store.</t>
+  </si>
+  <si>
+    <t>PS2-014</t>
+  </si>
+  <si>
+    <t>Ch.2, p.35</t>
+  </si>
+  <si>
+    <t>How do you get more storage space when PrintSphere storage is full?</t>
+  </si>
+  <si>
+    <t>Contact your PrintSphere administrator. Storage allocation is managed by the administrator in SphereCenter. Users cannot increase their own storage quota.</t>
+  </si>
+  <si>
+    <t>PS2-015</t>
+  </si>
+  <si>
+    <t>Ch.2, p.37</t>
+  </si>
+  <si>
+    <t>How do you open the Inspector Panel in PrintSphere Webclient?</t>
+  </si>
+  <si>
+    <t>Open the Actions menu (...) for a file or folder and select Open details. Alternatively, click one of the status icons (e.g. Share) to open a specific tab directly. The Inspector Panel appears on the right side.</t>
+  </si>
+  <si>
+    <t>PS2-016</t>
+  </si>
+  <si>
+    <t>Ch.2, p.42</t>
+  </si>
+  <si>
+    <t>How do you add or remove a tag from a file or folder in PrintSphere?</t>
+  </si>
+  <si>
+    <t>To add: open the Inspector Panel, select the Tags tab, and select the tag to apply. Tagging a folder does not apply the tag to its files. To remove: open the Tags tab in the Inspector Panel and deselect the tag.</t>
+  </si>
+  <si>
+    <t>PS2-017</t>
+  </si>
+  <si>
+    <t>Ch.2, p.43</t>
+  </si>
+  <si>
+    <t>What is the Activity Page in PrintSphere?</t>
+  </si>
+  <si>
+    <t>The Activity Page is a log of activities in your PrintSphere space, showing actions by you and other users on assets you own or share. The printer administrator can see all activities across the entire space. Access it via Activity in the main menu.</t>
+  </si>
+  <si>
+    <t>PS2-018</t>
+  </si>
+  <si>
+    <t>Ch.2, p.43-44</t>
+  </si>
+  <si>
+    <t>What activity filters are available on the PrintSphere Activity Page?</t>
+  </si>
+  <si>
+    <t>Filters: All Activities, By you, By others, Favorites, File changes (created/deleted/changed files), Security (security and auditing events), File shares (share/remove share activities), Comments, and Antivirus (malware scanning activities).</t>
+  </si>
+  <si>
+    <t>PS2-019</t>
+  </si>
+  <si>
+    <t>Ch.2, p.45</t>
+  </si>
+  <si>
+    <t>How do you upload files to PrintSphere Webclient?</t>
+  </si>
+  <si>
+    <t>Click the + New button at the top of the Files page, select Upload file or Upload folders, select files or folders and click Open (files) or Upload (folders). Alternatively, drag and drop files or folders from your file manager directly onto the Files page.</t>
+  </si>
+  <si>
+    <t>PS2-020</t>
+  </si>
+  <si>
+    <t>Ch.2, p.60</t>
+  </si>
+  <si>
+    <t>How do you restore a previous version of a file in PrintSphere?</t>
+  </si>
+  <si>
+    <t>Open the Actions menu (...) for the file and select Open details. In the Inspector Panel select the Versions tab. Click the Actions menu (...) next to the desired version and select Restore version. To preview a version, click the label showing when the file was last modified.</t>
+  </si>
+  <si>
+    <t>PS2-021</t>
+  </si>
+  <si>
+    <t>Ch.2, p.61</t>
+  </si>
+  <si>
+    <t>How do you download multiple files at once from PrintSphere Webclient?</t>
+  </si>
+  <si>
+    <t>Select the check box for each item, click the Actions menu (...) at the top of the list, and choose Download. Multiple files are packaged into a single download.zip file. To download everything in the current folder, click Select All, then choose Download from the Actions menu.</t>
+  </si>
+  <si>
+    <t>PS2-022</t>
+  </si>
+  <si>
+    <t>Ch.2, p.62</t>
+  </si>
+  <si>
+    <t>What is the difference between local sharing and public sharing in PrintSphere?</t>
+  </si>
+  <si>
+    <t>Local sharing is with Manual PrintSphere users who have an account; they see the shared item in their space and must log in to access it. Public sharing is with Auto PrintSphere users via a public internet link; they access the item without logging in but cannot see other items in the space. A public link can be password protected.</t>
+  </si>
+  <si>
+    <t>PS2-023</t>
+  </si>
+  <si>
+    <t>Ch.2, p.63-65</t>
+  </si>
+  <si>
+    <t>How do you share a file or folder with another Manual PrintSphere user?</t>
+  </si>
+  <si>
+    <t>In the Files list view click the Shared status for the item (or in grid view, open Actions &gt; Show sharing options). In the Sharing tab of the Inspector Panel, type the user or group name, select from the results, set permissions as needed (View only, Allow editing, or Advanced options), and click Save share.</t>
+  </si>
+  <si>
+    <t>PS2-024</t>
+  </si>
+  <si>
+    <t>Ch.2, p.64</t>
+  </si>
+  <si>
+    <t>What sharing permissions are available when sharing with Manual PrintSphere users?</t>
+  </si>
+  <si>
+    <t>Permissions: View only, Allow editing, Set expiration date (Advanced), Allow download and sync (Advanced), Note to recipient (Advanced — for public sharing only), and Custom permissions: Create, Edit, Share, Delete (all in Advanced settings).</t>
+  </si>
+  <si>
+    <t>PS2-025</t>
+  </si>
+  <si>
+    <t>Ch.2, p.66</t>
+  </si>
+  <si>
+    <t>How do you share a file or folder with Auto PrintSphere users (public sharing)?</t>
+  </si>
+  <si>
+    <t>Click the Shared status for the item in list view, or in grid view open Actions &gt; Show sharing options. In the Sharing tab of the Inspector Panel, create a public share link. The Auto PrintSphere user can access the item via this link without logging in.</t>
+  </si>
+  <si>
+    <t>PS2-026</t>
+  </si>
+  <si>
+    <t>Ch.2, p.62-66</t>
+  </si>
+  <si>
+    <t>How is a local share recipient notified when a file is shared with them?</t>
+  </si>
+  <si>
+    <t>The shared item appears in the recipient's PrintSphere space showing the owner's name. Email notification is sent only if the recipient has enabled this in their profile notification settings. The owner can also click Copy link to send the link manually. The recipient must log in to access the item.</t>
+  </si>
+  <si>
+    <t>PS2-027</t>
+  </si>
+  <si>
+    <t>What tabs can appear in the Inspector Panel in PrintSphere Webclient?</t>
+  </si>
+  <si>
+    <t>Depending on the asset type, the Inspector Panel may show up to four tabs: Activity (all activity on the asset chronologically), Sharing (sharing options and permissions), Versions (version history for files), and Tags.</t>
+  </si>
+  <si>
+    <t>PS2-028</t>
+  </si>
+  <si>
+    <t>Ch.2, p.36-37</t>
+  </si>
+  <si>
+    <t>What does the Search function in PrintSphere Webclient search across?</t>
+  </si>
+  <si>
+    <t>The Search box searches across your entire PrintSphere space — files, folders, tags, and messages. It is not limited to the currently open folder. The search filters the current view as you type and can be cleared to return to the unfiltered view.</t>
+  </si>
+  <si>
+    <t>PS2-029</t>
+  </si>
+  <si>
+    <t>Ch.3, p.76-78</t>
+  </si>
+  <si>
+    <t>How do you install the PrintSphere desktop application?</t>
+  </si>
+  <si>
+    <t>Download the installer from the URL provided in the documentation for your OS. Run the wizard and click through Next and Install. On the Connect to PrintSphere screen enter your user name and password. Choose a sync option (sync everything, choose what to sync, or change local folder location). Click Connect to finish. The app runs in the background and a local PrintSphere folder is created.</t>
+  </si>
+  <si>
+    <t>PS2-030</t>
+  </si>
+  <si>
+    <t>Ch.3, p.79</t>
+  </si>
+  <si>
+    <t>How do you update the PrintSphere desktop application?</t>
+  </si>
+  <si>
+    <t>In the General tab of the desktop application, click Restart &amp; Update. This restarts the application (not your computer) and applies the available update.</t>
+  </si>
+  <si>
+    <t>PS2-031</t>
+  </si>
+  <si>
+    <t>How do you uninstall the PrintSphere desktop application?</t>
+  </si>
+  <si>
+    <t>Remove the application like any other program on your computer. The uninstall wizard gives you the option to delete or keep the local PrintSphere folder and its data. Uninstalling stops the syncing process.</t>
+  </si>
+  <si>
+    <t>PS2-032</t>
+  </si>
+  <si>
+    <t>Ch.3, p.87-88</t>
+  </si>
+  <si>
+    <t>How do you add a sync connection in the PrintSphere desktop application?</t>
+  </si>
+  <si>
+    <t>In the Account tab, click Add Sync Connection. Enter a connection name, choose the local folder or accept the default, select the remote folder on the PrintSphere server. Click Next, fine-tune sub-folder syncing as needed, then click Add Sync Connection to confirm. The connection is added to the list.</t>
+  </si>
+  <si>
+    <t>PS2-033</t>
+  </si>
+  <si>
+    <t>Ch.3, p.90-92</t>
+  </si>
+  <si>
+    <t>How do you configure ignored files in the PrintSphere desktop application?</t>
+  </si>
+  <si>
+    <t>In the General tab, click Edit ignored Files to open the Ignored Files Editor. To add a pattern: click Add, enter the pattern (wildcards * and ? supported), click OK. To modify default patterns: hover over the pattern to find the sync-exclude.lst file location and edit it in a text editor. Caution: custom entries are not validated — if syncing fails, check your syntax.</t>
+  </si>
+  <si>
+    <t>PS2-034</t>
+  </si>
+  <si>
+    <t>Ch.3, p.90</t>
+  </si>
+  <si>
+    <t>What is the difference between a checked and unchecked check box in the PrintSphere Ignored Files Editor?</t>
+  </si>
+  <si>
+    <t>Unchecked: files and folders matching the pattern are ignored (not synced). Checked: matching files are ignored AND treated as fleeting metadata, meaning the desktop application actively removes them.</t>
+  </si>
+  <si>
+    <t>PS2-035</t>
+  </si>
+  <si>
+    <t>Ch.3, p.92-93</t>
+  </si>
+  <si>
+    <t>How do you stop or start syncing a specific remote folder in the PrintSphere desktop application?</t>
+  </si>
+  <si>
+    <t>In the Account tab, click the sync connection to expand the folder tree. Check or uncheck the folders you want to include or exclude from syncing, then confirm the change.</t>
+  </si>
+  <si>
+    <t>PS2-036</t>
+  </si>
+  <si>
+    <t>What sync options are available during PrintSphere desktop application installation?</t>
+  </si>
+  <si>
+    <t>On the Setup local folder options screen: Sync everything from server (all files copied to local folder), Choose what to sync (browse and select specific folders), and Local Folder button (change the default local folder path). If the local folder already contains data: Keep local data (kept but may be overwritten) or Start a clean sync (all local data deleted before syncing).</t>
+  </si>
+  <si>
+    <t>PS2-037</t>
+  </si>
+  <si>
+    <t>Ch.3, p.99</t>
+  </si>
+  <si>
+    <t>What options are available in the PrintSphere System Tray context menu?</t>
+  </si>
+  <si>
+    <t>Right-clicking the System Tray icon shows: Open in browser, Open folder, Pause/Resume all folders, Log out / Log in, Pause/Resume all synchronization (all folders and accounts), and Quit PrintSphere. With multiple sync connections, select a connection first to see per-connection options.</t>
+  </si>
+  <si>
+    <t>PS2-038</t>
+  </si>
+  <si>
+    <t>Ch.3, p.83-85</t>
+  </si>
+  <si>
+    <t>What is the difference between a sync connection and an account in the PrintSphere desktop application?</t>
+  </si>
+  <si>
+    <t>An account represents your PrintSphere credentials and can contain multiple sync connections. A sync connection is a specific link between a local folder on your computer and a remote folder in your PrintSphere space. The Account tab shows all accounts and their sync connections in a folder tree structure.</t>
+  </si>
+  <si>
+    <t>PS2-039</t>
+  </si>
+  <si>
+    <t>Ch.3, p.92</t>
+  </si>
+  <si>
+    <t>What should you check if synchronization does not work as expected after editing ignored file patterns?</t>
+  </si>
+  <si>
+    <t>Check the syntax of your custom ignore patterns. The Ignored Files Editor does not validate custom entries and shows no warnings for incorrect syntax. Also note: patterns ending with a slash (/) apply only to directory components of the path being checked.</t>
+  </si>
+  <si>
+    <t>PS2-040</t>
+  </si>
+  <si>
+    <t>Ch.3, p.78</t>
+  </si>
+  <si>
+    <t>What options are offered when the local folder already contains data during PrintSphere desktop app installation?</t>
+  </si>
+  <si>
+    <t>Keep local data: existing data is kept but may be overwritten by the sync. Start a clean sync: all data in the selected local folder is deleted before syncing begins.</t>
+  </si>
+  <si>
+    <t>PS2-041</t>
+  </si>
+  <si>
+    <t>Ch.4, p.102</t>
+  </si>
+  <si>
+    <t>What are the prerequisites for installing the PrintSphere mobile app?</t>
+  </si>
+  <si>
+    <t>The device must run Android 10.0 or later or Apple iOS 17.0 or later. The app is free but requires PrintSphere user credentials (same as for the Webclient) to sign on and configure.</t>
+  </si>
+  <si>
+    <t>PS2-042</t>
+  </si>
+  <si>
+    <t>Ch.4, p.102-104</t>
+  </si>
+  <si>
+    <t>How do you install and configure the PrintSphere mobile app?</t>
+  </si>
+  <si>
+    <t>Search for 'printsphere' in the Google Play store or Apple App store and install the free app. Open the app — on first launch the configuration screen is shown. Verify the connection URL is https://www.printsphere.com/access. Tap Log in, enter your Username and password (same as Webclient credentials), tap Log in, then tap Grant access to connect to your PrintSphere space.</t>
+  </si>
+  <si>
+    <t>PS2-043</t>
+  </si>
+  <si>
+    <t>Ch.4, p.105</t>
+  </si>
+  <si>
+    <t>What gestures are used to interact with files and folders in the PrintSphere mobile app?</t>
+  </si>
+  <si>
+    <t>Tap a file to download and view it. Tap a folder to open it. Touch and hold (long press) a folder for a menu: Share link, Download, Rename, Move, Remove. Touch and hold a file for a menu: Share link, Download, Rename, Move, Remove, Send, Details.</t>
+  </si>
+  <si>
+    <t>PS2-044</t>
+  </si>
+  <si>
+    <t>Ch.4, p.107</t>
+  </si>
+  <si>
+    <t>How do you upload files from the PrintSphere mobile app?</t>
+  </si>
+  <si>
+    <t>Tap the + button at the bottom right corner. Choose Files to upload from your file system, or Content from other apps. A notification confirms when the upload is complete and synced to your space. Note: only files can be uploaded from the mobile app, not folders.</t>
+  </si>
+  <si>
+    <t>PS2-045</t>
+  </si>
+  <si>
+    <t>Ch.4, p.107-108</t>
+  </si>
+  <si>
+    <t>Does the PrintSphere mobile app support multiple accounts on Android and iOS?</t>
+  </si>
+  <si>
+    <t>Multiple accounts are fully supported on Apple iOS only. On Android, the option to add multiple accounts exists but is currently not functional. On iOS, manage accounts via Settings at the bottom of the screen.</t>
+  </si>
+  <si>
+    <t>PS2-046</t>
+  </si>
+  <si>
+    <t>Ch.4, p.101-105</t>
+  </si>
+  <si>
+    <t>What is the difference between the PrintSphere Webclient and the mobile app in terms of data syncing?</t>
+  </si>
+  <si>
+    <t>The Webclient provides browser-based file management with no local data sync. The mobile app shows your space contents but does not sync or download actual data unless you open or preview a specific file — it is designed for on-the-go access, not full synchronization like the desktop application.</t>
+  </si>
+  <si>
+    <t>PS2-047</t>
+  </si>
+  <si>
+    <t>Ch.5, p.111</t>
+  </si>
+  <si>
+    <t>Workflow Connectivity allows print service providers using Apogee Prepress or Asanti to configure their workflow to work with the PrintSphere service, enabling the creation of shared hot folders and automated system back-ups on printsphere.com.</t>
+  </si>
+  <si>
+    <t>PS2-048</t>
+  </si>
+  <si>
+    <t>How do you create a PrintSphere-enabled job in Apogee Prepress?</t>
+  </si>
+  <si>
+    <t>Enable Workflow Connectivity in the system configuration. In Apogee Prepress or Asanti, create a job and configure it to use PrintSphere as the destination for hot folder sharing. Refer to the Connectivity chapter (p.111) and the Apogee Prepress Help or Asanti Online Help for the full procedure.</t>
+  </si>
+  <si>
+    <t>PS2-049</t>
+  </si>
+  <si>
+    <t>Ch.5, p.112</t>
+  </si>
+  <si>
+    <t>What is the Database Back-Up to PrintSphere feature?</t>
+  </si>
+  <si>
+    <t>Database Back-Up to PrintSphere is a connectivity feature that allows the workflow system to automatically back up its database to the PrintSphere storage service on printsphere.com, providing integrated off-site backup and recovery.</t>
+  </si>
+  <si>
+    <t>PS2-050</t>
+  </si>
+  <si>
+    <t>Ch.5, p.112 and Glossary</t>
+  </si>
+  <si>
+    <t>What is the difference between Manual PrintSphere users, Auto PrintSphere users, and Guests?</t>
+  </si>
+  <si>
+    <t>Manual PrintSphere users have a full account and use the Webclient, desktop app, and mobile apps. Auto PrintSphere users are the default type in ProductionCenter — they access files via a public link without logging in and cannot use the desktop app or mobile apps. Guests are invited job-by-job in Apogee Prepress or Asanti to upload/download in a specific folder without logging in; they are not linked to a company and their email must be entered each time.</t>
   </si>
 </sst>
 </file>
@@ -2792,40 +3372,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="K1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="L1" s="4" t="s">
         <v>278</v>
       </c>
     </row>
@@ -2969,40 +3549,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="K1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="L1" s="4" t="s">
         <v>278</v>
       </c>
     </row>
@@ -3215,40 +3795,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="K1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="L1" s="4" t="s">
         <v>278</v>
       </c>
     </row>
@@ -3392,40 +3972,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="K1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="L1" s="4" t="s">
         <v>278</v>
       </c>
     </row>
@@ -3569,40 +4149,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="K1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="L1" s="4" t="s">
         <v>278</v>
       </c>
     </row>
@@ -3764,6 +4344,1218 @@
         <v>654</v>
       </c>
       <c r="G8" t="s">
+        <v>276</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A251F04E-0B0A-40FA-81B3-E61B64E9674E}">
+  <dimension ref="A1:L51"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.5546875" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="75.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="164.33203125" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="174.6640625" customWidth="1"/>
+    <col min="9" max="9" width="29.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="77.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="20" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1" s="20" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="20" t="s">
+        <v>275</v>
+      </c>
+      <c r="I1" s="20" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="20" t="s">
+        <v>280</v>
+      </c>
+      <c r="K1" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="20" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>655</v>
+      </c>
+      <c r="B2" t="s">
+        <v>656</v>
+      </c>
+      <c r="C2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>657</v>
+      </c>
+      <c r="G2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>658</v>
+      </c>
+      <c r="B3" t="s">
+        <v>656</v>
+      </c>
+      <c r="C3" t="s">
+        <v>659</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>660</v>
+      </c>
+      <c r="G3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>661</v>
+      </c>
+      <c r="B4" t="s">
+        <v>662</v>
+      </c>
+      <c r="C4" t="s">
+        <v>663</v>
+      </c>
+      <c r="D4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>664</v>
+      </c>
+      <c r="G4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>665</v>
+      </c>
+      <c r="B5" t="s">
+        <v>666</v>
+      </c>
+      <c r="C5" t="s">
+        <v>667</v>
+      </c>
+      <c r="D5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>668</v>
+      </c>
+      <c r="G5" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>669</v>
+      </c>
+      <c r="B6" t="s">
+        <v>670</v>
+      </c>
+      <c r="C6" t="s">
+        <v>671</v>
+      </c>
+      <c r="D6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>672</v>
+      </c>
+      <c r="G6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>673</v>
+      </c>
+      <c r="B7" t="s">
+        <v>674</v>
+      </c>
+      <c r="C7" t="s">
+        <v>675</v>
+      </c>
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s">
+        <v>676</v>
+      </c>
+      <c r="G7" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>677</v>
+      </c>
+      <c r="B8" t="s">
+        <v>678</v>
+      </c>
+      <c r="C8" t="s">
+        <v>679</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
+        <v>680</v>
+      </c>
+      <c r="G8" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>681</v>
+      </c>
+      <c r="B9" t="s">
+        <v>682</v>
+      </c>
+      <c r="C9" t="s">
+        <v>683</v>
+      </c>
+      <c r="D9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" t="s">
+        <v>684</v>
+      </c>
+      <c r="G9" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>685</v>
+      </c>
+      <c r="B10" t="s">
+        <v>686</v>
+      </c>
+      <c r="C10" t="s">
+        <v>687</v>
+      </c>
+      <c r="D10" t="s">
+        <v>127</v>
+      </c>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" t="s">
+        <v>688</v>
+      </c>
+      <c r="G10" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>689</v>
+      </c>
+      <c r="B11" t="s">
+        <v>690</v>
+      </c>
+      <c r="C11" t="s">
+        <v>691</v>
+      </c>
+      <c r="D11" t="s">
+        <v>135</v>
+      </c>
+      <c r="E11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" t="s">
+        <v>692</v>
+      </c>
+      <c r="G11" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>693</v>
+      </c>
+      <c r="B12" t="s">
+        <v>694</v>
+      </c>
+      <c r="C12" t="s">
+        <v>695</v>
+      </c>
+      <c r="D12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" t="s">
+        <v>696</v>
+      </c>
+      <c r="G12" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>697</v>
+      </c>
+      <c r="B13" t="s">
+        <v>698</v>
+      </c>
+      <c r="C13" t="s">
+        <v>699</v>
+      </c>
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" t="s">
+        <v>700</v>
+      </c>
+      <c r="G13" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>701</v>
+      </c>
+      <c r="B14" t="s">
+        <v>702</v>
+      </c>
+      <c r="C14" t="s">
+        <v>703</v>
+      </c>
+      <c r="D14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" t="s">
+        <v>704</v>
+      </c>
+      <c r="G14" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>705</v>
+      </c>
+      <c r="B15" t="s">
+        <v>706</v>
+      </c>
+      <c r="C15" t="s">
+        <v>707</v>
+      </c>
+      <c r="D15" t="s">
+        <v>135</v>
+      </c>
+      <c r="E15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" t="s">
+        <v>708</v>
+      </c>
+      <c r="G15" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>709</v>
+      </c>
+      <c r="B16" t="s">
+        <v>710</v>
+      </c>
+      <c r="C16" t="s">
+        <v>711</v>
+      </c>
+      <c r="D16" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" t="s">
+        <v>712</v>
+      </c>
+      <c r="G16" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>713</v>
+      </c>
+      <c r="B17" t="s">
+        <v>714</v>
+      </c>
+      <c r="C17" t="s">
+        <v>715</v>
+      </c>
+      <c r="D17" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" t="s">
+        <v>716</v>
+      </c>
+      <c r="G17" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>717</v>
+      </c>
+      <c r="B18" t="s">
+        <v>718</v>
+      </c>
+      <c r="C18" t="s">
+        <v>719</v>
+      </c>
+      <c r="D18" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" t="s">
+        <v>720</v>
+      </c>
+      <c r="G18" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>721</v>
+      </c>
+      <c r="B19" t="s">
+        <v>722</v>
+      </c>
+      <c r="C19" t="s">
+        <v>723</v>
+      </c>
+      <c r="D19" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" t="s">
+        <v>22</v>
+      </c>
+      <c r="F19" t="s">
+        <v>724</v>
+      </c>
+      <c r="G19" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>725</v>
+      </c>
+      <c r="B20" t="s">
+        <v>726</v>
+      </c>
+      <c r="C20" t="s">
+        <v>727</v>
+      </c>
+      <c r="D20" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" t="s">
+        <v>728</v>
+      </c>
+      <c r="G20" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>729</v>
+      </c>
+      <c r="B21" t="s">
+        <v>730</v>
+      </c>
+      <c r="C21" t="s">
+        <v>731</v>
+      </c>
+      <c r="D21" t="s">
+        <v>14</v>
+      </c>
+      <c r="E21" t="s">
+        <v>22</v>
+      </c>
+      <c r="F21" t="s">
+        <v>732</v>
+      </c>
+      <c r="G21" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>733</v>
+      </c>
+      <c r="B22" t="s">
+        <v>734</v>
+      </c>
+      <c r="C22" t="s">
+        <v>735</v>
+      </c>
+      <c r="D22" t="s">
+        <v>14</v>
+      </c>
+      <c r="E22" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" t="s">
+        <v>736</v>
+      </c>
+      <c r="G22" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>737</v>
+      </c>
+      <c r="B23" t="s">
+        <v>738</v>
+      </c>
+      <c r="C23" t="s">
+        <v>739</v>
+      </c>
+      <c r="D23" t="s">
+        <v>127</v>
+      </c>
+      <c r="E23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" t="s">
+        <v>740</v>
+      </c>
+      <c r="G23" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>741</v>
+      </c>
+      <c r="B24" t="s">
+        <v>742</v>
+      </c>
+      <c r="C24" t="s">
+        <v>743</v>
+      </c>
+      <c r="D24" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24" t="s">
+        <v>744</v>
+      </c>
+      <c r="G24" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>745</v>
+      </c>
+      <c r="B25" t="s">
+        <v>746</v>
+      </c>
+      <c r="C25" t="s">
+        <v>747</v>
+      </c>
+      <c r="D25" t="s">
+        <v>37</v>
+      </c>
+      <c r="E25" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" t="s">
+        <v>748</v>
+      </c>
+      <c r="G25" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>749</v>
+      </c>
+      <c r="B26" t="s">
+        <v>750</v>
+      </c>
+      <c r="C26" t="s">
+        <v>751</v>
+      </c>
+      <c r="D26" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" t="s">
+        <v>22</v>
+      </c>
+      <c r="F26" t="s">
+        <v>752</v>
+      </c>
+      <c r="G26" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>753</v>
+      </c>
+      <c r="B27" t="s">
+        <v>754</v>
+      </c>
+      <c r="C27" t="s">
+        <v>755</v>
+      </c>
+      <c r="D27" t="s">
+        <v>37</v>
+      </c>
+      <c r="E27" t="s">
+        <v>10</v>
+      </c>
+      <c r="F27" t="s">
+        <v>756</v>
+      </c>
+      <c r="G27" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>757</v>
+      </c>
+      <c r="B28" t="s">
+        <v>710</v>
+      </c>
+      <c r="C28" t="s">
+        <v>758</v>
+      </c>
+      <c r="D28" t="s">
+        <v>9</v>
+      </c>
+      <c r="E28" t="s">
+        <v>22</v>
+      </c>
+      <c r="F28" t="s">
+        <v>759</v>
+      </c>
+      <c r="G28" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>760</v>
+      </c>
+      <c r="B29" t="s">
+        <v>761</v>
+      </c>
+      <c r="C29" t="s">
+        <v>762</v>
+      </c>
+      <c r="D29" t="s">
+        <v>37</v>
+      </c>
+      <c r="E29" t="s">
+        <v>10</v>
+      </c>
+      <c r="F29" t="s">
+        <v>763</v>
+      </c>
+      <c r="G29" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>764</v>
+      </c>
+      <c r="B30" t="s">
+        <v>765</v>
+      </c>
+      <c r="C30" t="s">
+        <v>766</v>
+      </c>
+      <c r="D30" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30" t="s">
+        <v>22</v>
+      </c>
+      <c r="F30" t="s">
+        <v>767</v>
+      </c>
+      <c r="G30" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>768</v>
+      </c>
+      <c r="B31" t="s">
+        <v>769</v>
+      </c>
+      <c r="C31" t="s">
+        <v>770</v>
+      </c>
+      <c r="D31" t="s">
+        <v>14</v>
+      </c>
+      <c r="E31" t="s">
+        <v>10</v>
+      </c>
+      <c r="F31" t="s">
+        <v>771</v>
+      </c>
+      <c r="G31" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>772</v>
+      </c>
+      <c r="B32" t="s">
+        <v>769</v>
+      </c>
+      <c r="C32" t="s">
+        <v>773</v>
+      </c>
+      <c r="D32" t="s">
+        <v>14</v>
+      </c>
+      <c r="E32" t="s">
+        <v>10</v>
+      </c>
+      <c r="F32" t="s">
+        <v>774</v>
+      </c>
+      <c r="G32" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>775</v>
+      </c>
+      <c r="B33" t="s">
+        <v>776</v>
+      </c>
+      <c r="C33" t="s">
+        <v>777</v>
+      </c>
+      <c r="D33" t="s">
+        <v>14</v>
+      </c>
+      <c r="E33" t="s">
+        <v>22</v>
+      </c>
+      <c r="F33" t="s">
+        <v>778</v>
+      </c>
+      <c r="G33" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>779</v>
+      </c>
+      <c r="B34" t="s">
+        <v>780</v>
+      </c>
+      <c r="C34" t="s">
+        <v>781</v>
+      </c>
+      <c r="D34" t="s">
+        <v>14</v>
+      </c>
+      <c r="E34" t="s">
+        <v>175</v>
+      </c>
+      <c r="F34" t="s">
+        <v>782</v>
+      </c>
+      <c r="G34" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>783</v>
+      </c>
+      <c r="B35" t="s">
+        <v>784</v>
+      </c>
+      <c r="C35" t="s">
+        <v>785</v>
+      </c>
+      <c r="D35" t="s">
+        <v>9</v>
+      </c>
+      <c r="E35" t="s">
+        <v>175</v>
+      </c>
+      <c r="F35" t="s">
+        <v>786</v>
+      </c>
+      <c r="G35" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>787</v>
+      </c>
+      <c r="B36" t="s">
+        <v>788</v>
+      </c>
+      <c r="C36" t="s">
+        <v>789</v>
+      </c>
+      <c r="D36" t="s">
+        <v>14</v>
+      </c>
+      <c r="E36" t="s">
+        <v>22</v>
+      </c>
+      <c r="F36" t="s">
+        <v>790</v>
+      </c>
+      <c r="G36" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>791</v>
+      </c>
+      <c r="B37" t="s">
+        <v>776</v>
+      </c>
+      <c r="C37" t="s">
+        <v>792</v>
+      </c>
+      <c r="D37" t="s">
+        <v>37</v>
+      </c>
+      <c r="E37" t="s">
+        <v>22</v>
+      </c>
+      <c r="F37" t="s">
+        <v>793</v>
+      </c>
+      <c r="G37" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>794</v>
+      </c>
+      <c r="B38" t="s">
+        <v>795</v>
+      </c>
+      <c r="C38" t="s">
+        <v>796</v>
+      </c>
+      <c r="D38" t="s">
+        <v>37</v>
+      </c>
+      <c r="E38" t="s">
+        <v>22</v>
+      </c>
+      <c r="F38" t="s">
+        <v>797</v>
+      </c>
+      <c r="G38" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>798</v>
+      </c>
+      <c r="B39" t="s">
+        <v>799</v>
+      </c>
+      <c r="C39" t="s">
+        <v>800</v>
+      </c>
+      <c r="D39" t="s">
+        <v>127</v>
+      </c>
+      <c r="E39" t="s">
+        <v>175</v>
+      </c>
+      <c r="F39" t="s">
+        <v>801</v>
+      </c>
+      <c r="G39" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>802</v>
+      </c>
+      <c r="B40" t="s">
+        <v>803</v>
+      </c>
+      <c r="C40" t="s">
+        <v>804</v>
+      </c>
+      <c r="D40" t="s">
+        <v>135</v>
+      </c>
+      <c r="E40" t="s">
+        <v>22</v>
+      </c>
+      <c r="F40" t="s">
+        <v>805</v>
+      </c>
+      <c r="G40" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>806</v>
+      </c>
+      <c r="B41" t="s">
+        <v>807</v>
+      </c>
+      <c r="C41" t="s">
+        <v>808</v>
+      </c>
+      <c r="D41" t="s">
+        <v>135</v>
+      </c>
+      <c r="E41" t="s">
+        <v>22</v>
+      </c>
+      <c r="F41" t="s">
+        <v>809</v>
+      </c>
+      <c r="G41" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>810</v>
+      </c>
+      <c r="B42" t="s">
+        <v>811</v>
+      </c>
+      <c r="C42" t="s">
+        <v>812</v>
+      </c>
+      <c r="D42" t="s">
+        <v>9</v>
+      </c>
+      <c r="E42" t="s">
+        <v>10</v>
+      </c>
+      <c r="F42" t="s">
+        <v>813</v>
+      </c>
+      <c r="G42" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>814</v>
+      </c>
+      <c r="B43" t="s">
+        <v>815</v>
+      </c>
+      <c r="C43" t="s">
+        <v>816</v>
+      </c>
+      <c r="D43" t="s">
+        <v>14</v>
+      </c>
+      <c r="E43" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43" t="s">
+        <v>817</v>
+      </c>
+      <c r="G43" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>818</v>
+      </c>
+      <c r="B44" t="s">
+        <v>819</v>
+      </c>
+      <c r="C44" t="s">
+        <v>820</v>
+      </c>
+      <c r="D44" t="s">
+        <v>37</v>
+      </c>
+      <c r="E44" t="s">
+        <v>10</v>
+      </c>
+      <c r="F44" t="s">
+        <v>821</v>
+      </c>
+      <c r="G44" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>822</v>
+      </c>
+      <c r="B45" t="s">
+        <v>823</v>
+      </c>
+      <c r="C45" t="s">
+        <v>824</v>
+      </c>
+      <c r="D45" t="s">
+        <v>14</v>
+      </c>
+      <c r="E45" t="s">
+        <v>10</v>
+      </c>
+      <c r="F45" t="s">
+        <v>825</v>
+      </c>
+      <c r="G45" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>826</v>
+      </c>
+      <c r="B46" t="s">
+        <v>827</v>
+      </c>
+      <c r="C46" t="s">
+        <v>828</v>
+      </c>
+      <c r="D46" t="s">
+        <v>135</v>
+      </c>
+      <c r="E46" t="s">
+        <v>22</v>
+      </c>
+      <c r="F46" t="s">
+        <v>829</v>
+      </c>
+      <c r="G46" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>830</v>
+      </c>
+      <c r="B47" t="s">
+        <v>831</v>
+      </c>
+      <c r="C47" t="s">
+        <v>832</v>
+      </c>
+      <c r="D47" t="s">
+        <v>127</v>
+      </c>
+      <c r="E47" t="s">
+        <v>22</v>
+      </c>
+      <c r="F47" t="s">
+        <v>833</v>
+      </c>
+      <c r="G47" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>834</v>
+      </c>
+      <c r="B48" t="s">
+        <v>835</v>
+      </c>
+      <c r="C48" t="s">
+        <v>74</v>
+      </c>
+      <c r="D48" t="s">
+        <v>9</v>
+      </c>
+      <c r="E48" t="s">
+        <v>22</v>
+      </c>
+      <c r="F48" t="s">
+        <v>836</v>
+      </c>
+      <c r="G48" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>837</v>
+      </c>
+      <c r="B49" t="s">
+        <v>835</v>
+      </c>
+      <c r="C49" t="s">
+        <v>838</v>
+      </c>
+      <c r="D49" t="s">
+        <v>14</v>
+      </c>
+      <c r="E49" t="s">
+        <v>175</v>
+      </c>
+      <c r="F49" t="s">
+        <v>839</v>
+      </c>
+      <c r="G49" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>840</v>
+      </c>
+      <c r="B50" t="s">
+        <v>841</v>
+      </c>
+      <c r="C50" t="s">
+        <v>842</v>
+      </c>
+      <c r="D50" t="s">
+        <v>9</v>
+      </c>
+      <c r="E50" t="s">
+        <v>22</v>
+      </c>
+      <c r="F50" t="s">
+        <v>843</v>
+      </c>
+      <c r="G50" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>844</v>
+      </c>
+      <c r="B51" t="s">
+        <v>845</v>
+      </c>
+      <c r="C51" t="s">
+        <v>846</v>
+      </c>
+      <c r="D51" t="s">
+        <v>127</v>
+      </c>
+      <c r="E51" t="s">
+        <v>175</v>
+      </c>
+      <c r="F51" t="s">
+        <v>847</v>
+      </c>
+      <c r="G51" t="s">
         <v>276</v>
       </c>
     </row>
@@ -6436,40 +8228,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="K1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="L1" s="4" t="s">
         <v>278</v>
       </c>
     </row>
@@ -6613,40 +8405,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="K1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="L1" s="4" t="s">
         <v>278</v>
       </c>
     </row>
@@ -6905,40 +8697,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="K1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="L1" s="4" t="s">
         <v>278</v>
       </c>
     </row>
@@ -7105,40 +8897,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="K1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="L1" s="4" t="s">
         <v>278</v>
       </c>
     </row>
@@ -7443,40 +9235,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="K1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="L1" s="4" t="s">
         <v>278</v>
       </c>
     </row>

</xml_diff>

<commit_message>
qa_test: fix FINAL SCORE and Note row labels — replace 'pct' with '%'
</commit_message>
<xml_diff>
--- a/qa_test.xlsx
+++ b/qa_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DFB77A6-60A6-4E3F-85C1-07C3ED23ECC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29F62150-83C3-4DCA-8A26-83C22B0FAA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="11" activeTab="14" xr2:uid="{BAFA452A-E2F4-40F7-9E5A-F91737B52715}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2175" uniqueCount="1018">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2175" uniqueCount="1017">
   <si>
     <t>ID</t>
   </si>
@@ -2617,13 +2617,7 @@
     <t>Digital QuickStrip (DQS) in Apogee Prepress offers individual page rendering, post-rendering imposition, and the ROOM principle (Render Once, Output Many) for step-and-repeat jobs.</t>
   </si>
   <si>
-    <t>FINAL SCORE (80 pct)</t>
-  </si>
-  <si>
     <t>4 Pass</t>
-  </si>
-  <si>
-    <t>Auto-tested via APAI Chat API on 2026-06-12. 4 Pass / 1 Fail (80 pct). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
   </si>
   <si>
     <t>Number-up Binding combines two or more book signatures on a single bindery signature which is subsequently cut to produce multiple book signatures. Number-up Cut and Assemble involves folding together pairs of book signatures, cutting them apart, and then assembling them in numerical order.</t>
@@ -2700,13 +2694,7 @@
 18. Submit the job.</t>
   </si>
   <si>
-    <t>FINAL SCORE (90 pct)</t>
-  </si>
-  <si>
     <t>9 Pass</t>
-  </si>
-  <si>
-    <t>Auto-tested via APAI Chat API on 2026-06-12. 9 Pass / 1 Fail (90 pct). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
   </si>
   <si>
     <t>Passkeys in Apogee v14 WebApproval and WebFlow are a modern, secure, and user-friendly authentication method based on public-key cryptography. They provide a phishing-resistant and passwordless sign-in experience, enhancing security for webservers.</t>
@@ -2734,16 +2722,10 @@
     <t>If the WebApproval domain or subdomain is changed, existing Passkeys will no longer be compatible and will need to be re-created by the end-user.</t>
   </si>
   <si>
-    <t>FINAL SCORE (100 pct)</t>
-  </si>
-  <si>
     <t>6 Pass</t>
   </si>
   <si>
     <t>0 Fail</t>
-  </si>
-  <si>
-    <t>Auto-tested via APAI Chat API on 2026-06-12. 6 Pass / 0 Fail (100 pct). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
   </si>
   <si>
     <t>Direct Approval: A page is approved when one approver assigned to that job has approved that page. Multi Approval: A page is approved when all approvers assigned to that job have approved that page.</t>
@@ -2808,15 +2790,9 @@
     <t>Press the A key to show or hide the Approval Progress bar in the flipbook.</t>
   </si>
   <si>
-    <t>FINAL SCORE (92 pct)</t>
-  </si>
-  <si>
     <t>11 Pass</t>
   </si>
   <si>
-    <t>Auto-tested via APAI Chat API on 2026-06-12. 11 Pass / 1 Fail (92 pct). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
-  </si>
-  <si>
     <t>The Apogee GDI Proofer is an indirect generic device driver that allows almost any Windows-compatible printer to be used for proofing within the Apogee Prepress workflow. It uses Microsoft's GDI (Graphics Device Interface) to send layouts and page proofs to inkjets or high-end digital presses. It is a cost-effective solution for previewing impositions or producing quick client proofs without the need for dedicated proofing hardware.</t>
   </si>
   <si>
@@ -2868,12 +2844,6 @@
     <t>Partial match (24 pct) - review.</t>
   </si>
   <si>
-    <t>FINAL SCORE (40 pct)</t>
-  </si>
-  <si>
-    <t>Auto-tested via APAI Chat API on 2026-06-12. 2 Pass / 3 Fail (40 pct). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
-  </si>
-  <si>
     <t>The Product and Part definitions in an Apogee Job Ticket are used to specify the individual components of a print job, including their attributes such as name, page size, copy count, colors, stock, and binding options. This allows for detailed control over each element of the job, enabling complex multi-part and multi-product jobs to be accurately defined and managed.</t>
   </si>
   <si>
@@ -2913,13 +2883,7 @@
     <t>Apogee offers several control options for handling Preflight errors in a WebApproval job: 1. Report to WebApproval: Send a Preflight Report to the Customer via Remarks in the WebApproval application. 2. Refuse document placement when Preflight has errors: Select an option to refuse jobs with errors and/or warnings. 3. Automatically reject pages with Preflight errors: Choose to automatically reject pages that have Preflight errors.</t>
   </si>
   <si>
-    <t>FINAL SCORE (38 pct)</t>
-  </si>
-  <si>
     <t>5 Fail</t>
-  </si>
-  <si>
-    <t>Auto-tested via APAI Chat API on 2026-06-12. 3 Pass / 5 Fail (38 pct). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
   </si>
   <si>
     <t>Virus scanning is important for Apogee and Amfortis production servers to prevent production disruptions, malware infections, ransomware attacks, and spyware. It helps block harmful files before they can impact the systems, reducing the risk of downtime, data loss, and security breaches. Proper configuration of virus scanning is crucial to maintain system performance and security.</t>
@@ -2989,13 +2953,7 @@
     <t>Partial match (37 pct) - review.</t>
   </si>
   <si>
-    <t>FINAL SCORE (71 pct)</t>
-  </si>
-  <si>
     <t>5 Pass</t>
-  </si>
-  <si>
-    <t>Auto-tested via APAI Chat API on 2026-06-12. 5 Pass / 2 Fail (71 pct). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
   </si>
   <si>
     <t>PrintSphere is a service that allows users to store, share, and sync files via a dedicated space on the printsphere.com server. It can be accessed through the PrintSphere Webclient, desktop application, or mobile apps.</t>
@@ -3225,16 +3183,55 @@
     <t>Manual PrintSphere users have a PrintSphere account and can use the PrintSphere Webclient, mobile apps, and desktop application. Auto PrintSphere users can use certain features of the PrintSphere service without an account and without logging in, but cannot use the desktop application or mobile apps. Guests are invited on a job-by-job basis to upload/download files in a specified folder for a PrintSphere-enabled prepress job without logging in, and cannot use the desktop application or mobile apps.</t>
   </si>
   <si>
-    <t>FINAL SCORE (86 pct)</t>
-  </si>
-  <si>
     <t>43 Pass</t>
   </si>
   <si>
     <t>7 Fail</t>
   </si>
   <si>
-    <t>Auto-tested via APAI Chat API on 2026-06-12. 43 Pass / 7 Fail (86 pct). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
+    <t>FINAL SCORE (80%)</t>
+  </si>
+  <si>
+    <t>FINAL SCORE (90%)</t>
+  </si>
+  <si>
+    <t>FINAL SCORE (100%)</t>
+  </si>
+  <si>
+    <t>FINAL SCORE (92%)</t>
+  </si>
+  <si>
+    <t>FINAL SCORE (38%)</t>
+  </si>
+  <si>
+    <t>FINAL SCORE (71%)</t>
+  </si>
+  <si>
+    <t>FINAL SCORE (86%)</t>
+  </si>
+  <si>
+    <t>Auto-tested via APAI Chat API on 2026-06-12. 4 Pass / 1 Fail (80%). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
+  </si>
+  <si>
+    <t>Auto-tested via APAI Chat API on 2026-06-12. 9 Pass / 1 Fail (90%). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
+  </si>
+  <si>
+    <t>Auto-tested via APAI Chat API on 2026-06-12. 6 Pass / 0 Fail (100%). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
+  </si>
+  <si>
+    <t>Auto-tested via APAI Chat API on 2026-06-12. 11 Pass / 1 Fail (92%). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
+  </si>
+  <si>
+    <t>Auto-tested via APAI Chat API on 2026-06-12. 2 Pass / 3 Fail (40%). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
+  </si>
+  <si>
+    <t>Auto-tested via APAI Chat API on 2026-06-12. 3 Pass / 5 Fail (38%). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
+  </si>
+  <si>
+    <t>Auto-tested via APAI Chat API on 2026-06-12. 5 Pass / 2 Fail (71%). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
+  </si>
+  <si>
+    <t>Auto-tested via APAI Chat API on 2026-06-12. 43 Pass / 7 Fail (86%). Pass/Fail by keyword match - manual review recommended for borderline cases.</t>
   </si>
 </sst>
 </file>
@@ -3380,12 +3377,12 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3970,19 +3967,19 @@
       <c r="A9" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="20" t="s">
         <v>295</v>
       </c>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="20"/>
+      <c r="L9" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4072,10 +4069,10 @@
         <v>276</v>
       </c>
       <c r="H2" t="s">
-        <v>908</v>
+        <v>900</v>
       </c>
       <c r="I2" t="s">
-        <v>909</v>
+        <v>901</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -4107,10 +4104,10 @@
         <v>276</v>
       </c>
       <c r="H3" t="s">
-        <v>910</v>
+        <v>902</v>
       </c>
       <c r="I3" t="s">
-        <v>909</v>
+        <v>901</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -4119,7 +4116,7 @@
         <v>286</v>
       </c>
       <c r="L3" t="s">
-        <v>911</v>
+        <v>903</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -4145,10 +4142,10 @@
         <v>276</v>
       </c>
       <c r="H4" t="s">
-        <v>912</v>
+        <v>904</v>
       </c>
       <c r="I4" t="s">
-        <v>909</v>
+        <v>901</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -4180,10 +4177,10 @@
         <v>276</v>
       </c>
       <c r="H5" t="s">
-        <v>913</v>
+        <v>905</v>
       </c>
       <c r="I5" t="s">
-        <v>909</v>
+        <v>901</v>
       </c>
       <c r="J5">
         <v>3</v>
@@ -4192,7 +4189,7 @@
         <v>286</v>
       </c>
       <c r="L5" t="s">
-        <v>914</v>
+        <v>906</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -4218,10 +4215,10 @@
         <v>276</v>
       </c>
       <c r="H6" t="s">
-        <v>915</v>
+        <v>907</v>
       </c>
       <c r="I6" t="s">
-        <v>909</v>
+        <v>901</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -4230,12 +4227,12 @@
         <v>286</v>
       </c>
       <c r="L6" t="s">
-        <v>916</v>
+        <v>908</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>917</v>
+        <v>396</v>
       </c>
       <c r="K7" s="15" t="s">
         <v>397</v>
@@ -4246,7 +4243,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B8" s="18" t="s">
-        <v>918</v>
+        <v>1013</v>
       </c>
       <c r="C8" s="19"/>
       <c r="D8" s="19"/>
@@ -4347,7 +4344,7 @@
         <v>276</v>
       </c>
       <c r="H2" t="s">
-        <v>919</v>
+        <v>909</v>
       </c>
       <c r="I2" t="s">
         <v>297</v>
@@ -4359,7 +4356,7 @@
         <v>286</v>
       </c>
       <c r="L2" t="s">
-        <v>920</v>
+        <v>910</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
@@ -4385,10 +4382,10 @@
         <v>276</v>
       </c>
       <c r="H3" t="s">
-        <v>921</v>
+        <v>911</v>
       </c>
       <c r="I3" t="s">
-        <v>922</v>
+        <v>912</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -4397,7 +4394,7 @@
         <v>286</v>
       </c>
       <c r="L3" t="s">
-        <v>911</v>
+        <v>903</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -4423,10 +4420,10 @@
         <v>276</v>
       </c>
       <c r="H4" t="s">
-        <v>923</v>
+        <v>913</v>
       </c>
       <c r="I4" t="s">
-        <v>922</v>
+        <v>912</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -4435,7 +4432,7 @@
         <v>286</v>
       </c>
       <c r="L4" t="s">
-        <v>924</v>
+        <v>914</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -4461,10 +4458,10 @@
         <v>276</v>
       </c>
       <c r="H5" t="s">
-        <v>925</v>
+        <v>915</v>
       </c>
       <c r="I5" t="s">
-        <v>922</v>
+        <v>912</v>
       </c>
       <c r="J5">
         <v>6</v>
@@ -4496,10 +4493,10 @@
         <v>276</v>
       </c>
       <c r="H6" t="s">
-        <v>926</v>
+        <v>916</v>
       </c>
       <c r="I6" t="s">
-        <v>922</v>
+        <v>912</v>
       </c>
       <c r="J6">
         <v>2</v>
@@ -4508,7 +4505,7 @@
         <v>286</v>
       </c>
       <c r="L6" t="s">
-        <v>927</v>
+        <v>917</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -4534,10 +4531,10 @@
         <v>276</v>
       </c>
       <c r="H7" t="s">
-        <v>928</v>
+        <v>918</v>
       </c>
       <c r="I7" t="s">
-        <v>922</v>
+        <v>912</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -4569,10 +4566,10 @@
         <v>276</v>
       </c>
       <c r="H8" t="s">
-        <v>929</v>
+        <v>919</v>
       </c>
       <c r="I8" t="s">
-        <v>922</v>
+        <v>912</v>
       </c>
       <c r="J8">
         <v>1</v>
@@ -4581,7 +4578,7 @@
         <v>286</v>
       </c>
       <c r="L8" t="s">
-        <v>930</v>
+        <v>920</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
@@ -4607,7 +4604,7 @@
         <v>276</v>
       </c>
       <c r="H9" t="s">
-        <v>931</v>
+        <v>921</v>
       </c>
       <c r="I9" t="s">
         <v>308</v>
@@ -4621,18 +4618,18 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>932</v>
+        <v>1006</v>
       </c>
       <c r="K10" s="15" t="s">
         <v>400</v>
       </c>
       <c r="L10" s="16" t="s">
-        <v>933</v>
+        <v>922</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B11" s="18" t="s">
-        <v>934</v>
+        <v>1014</v>
       </c>
       <c r="C11" s="19"/>
       <c r="D11" s="19"/>
@@ -4733,10 +4730,10 @@
         <v>276</v>
       </c>
       <c r="H2" t="s">
-        <v>935</v>
+        <v>923</v>
       </c>
       <c r="I2" t="s">
-        <v>936</v>
+        <v>924</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -4768,10 +4765,10 @@
         <v>276</v>
       </c>
       <c r="H3" t="s">
-        <v>937</v>
+        <v>925</v>
       </c>
       <c r="I3" t="s">
-        <v>936</v>
+        <v>924</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -4780,7 +4777,7 @@
         <v>286</v>
       </c>
       <c r="L3" t="s">
-        <v>930</v>
+        <v>920</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -4806,10 +4803,10 @@
         <v>276</v>
       </c>
       <c r="H4" t="s">
-        <v>938</v>
+        <v>926</v>
       </c>
       <c r="I4" t="s">
-        <v>936</v>
+        <v>924</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -4841,10 +4838,10 @@
         <v>276</v>
       </c>
       <c r="H5" t="s">
-        <v>939</v>
+        <v>927</v>
       </c>
       <c r="I5" t="s">
-        <v>936</v>
+        <v>924</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -4876,10 +4873,10 @@
         <v>276</v>
       </c>
       <c r="H6" t="s">
-        <v>940</v>
+        <v>928</v>
       </c>
       <c r="I6" t="s">
-        <v>936</v>
+        <v>924</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -4890,10 +4887,10 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
+        <v>1002</v>
+      </c>
+      <c r="K7" s="15" t="s">
         <v>854</v>
-      </c>
-      <c r="K7" s="15" t="s">
-        <v>855</v>
       </c>
       <c r="L7" s="16" t="s">
         <v>401</v>
@@ -4901,7 +4898,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B8" s="18" t="s">
-        <v>856</v>
+        <v>1009</v>
       </c>
       <c r="C8" s="19"/>
       <c r="D8" s="19"/>
@@ -5002,7 +4999,7 @@
         <v>276</v>
       </c>
       <c r="H2" t="s">
-        <v>941</v>
+        <v>929</v>
       </c>
       <c r="I2" t="s">
         <v>308</v>
@@ -5037,10 +5034,10 @@
         <v>276</v>
       </c>
       <c r="H3" t="s">
-        <v>942</v>
+        <v>930</v>
       </c>
       <c r="I3" t="s">
-        <v>943</v>
+        <v>931</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -5072,10 +5069,10 @@
         <v>276</v>
       </c>
       <c r="H4" t="s">
-        <v>944</v>
+        <v>932</v>
       </c>
       <c r="I4" t="s">
-        <v>943</v>
+        <v>931</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -5107,10 +5104,10 @@
         <v>276</v>
       </c>
       <c r="H5" t="s">
-        <v>945</v>
+        <v>933</v>
       </c>
       <c r="I5" t="s">
-        <v>943</v>
+        <v>931</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -5119,7 +5116,7 @@
         <v>286</v>
       </c>
       <c r="L5" t="s">
-        <v>946</v>
+        <v>934</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -5145,10 +5142,10 @@
         <v>276</v>
       </c>
       <c r="H6" t="s">
-        <v>947</v>
+        <v>935</v>
       </c>
       <c r="I6" t="s">
-        <v>943</v>
+        <v>931</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -5159,10 +5156,10 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
+        <v>1002</v>
+      </c>
+      <c r="K7" s="15" t="s">
         <v>854</v>
-      </c>
-      <c r="K7" s="15" t="s">
-        <v>855</v>
       </c>
       <c r="L7" s="16" t="s">
         <v>401</v>
@@ -5170,7 +5167,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B8" s="18" t="s">
-        <v>856</v>
+        <v>1009</v>
       </c>
       <c r="C8" s="19"/>
       <c r="D8" s="19"/>
@@ -5271,10 +5268,10 @@
         <v>276</v>
       </c>
       <c r="H2" t="s">
-        <v>948</v>
+        <v>936</v>
       </c>
       <c r="I2" t="s">
-        <v>949</v>
+        <v>937</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -5306,10 +5303,10 @@
         <v>276</v>
       </c>
       <c r="H3" t="s">
-        <v>950</v>
+        <v>938</v>
       </c>
       <c r="I3" t="s">
-        <v>949</v>
+        <v>937</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -5341,10 +5338,10 @@
         <v>276</v>
       </c>
       <c r="H4" t="s">
-        <v>951</v>
+        <v>939</v>
       </c>
       <c r="I4" t="s">
-        <v>949</v>
+        <v>937</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -5376,7 +5373,7 @@
         <v>276</v>
       </c>
       <c r="H5" t="s">
-        <v>952</v>
+        <v>940</v>
       </c>
       <c r="I5" t="s">
         <v>366</v>
@@ -5388,7 +5385,7 @@
         <v>286</v>
       </c>
       <c r="L5" t="s">
-        <v>924</v>
+        <v>914</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -5414,7 +5411,7 @@
         <v>276</v>
       </c>
       <c r="H6" t="s">
-        <v>953</v>
+        <v>941</v>
       </c>
       <c r="I6" t="s">
         <v>308</v>
@@ -5448,8 +5445,8 @@
       <c r="G7" t="s">
         <v>276</v>
       </c>
-      <c r="H7" s="20" t="s">
-        <v>954</v>
+      <c r="H7" s="17" t="s">
+        <v>942</v>
       </c>
       <c r="I7" t="s">
         <v>306</v>
@@ -5484,7 +5481,7 @@
         <v>276</v>
       </c>
       <c r="H8" t="s">
-        <v>955</v>
+        <v>943</v>
       </c>
       <c r="I8" t="s">
         <v>308</v>
@@ -5496,15 +5493,15 @@
         <v>286</v>
       </c>
       <c r="L8" t="s">
-        <v>956</v>
+        <v>944</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
-        <v>957</v>
+        <v>1007</v>
       </c>
       <c r="K9" s="15" t="s">
-        <v>958</v>
+        <v>945</v>
       </c>
       <c r="L9" s="16" t="s">
         <v>403</v>
@@ -5512,7 +5509,7 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B10" s="18" t="s">
-        <v>959</v>
+        <v>1015</v>
       </c>
       <c r="C10" s="19"/>
       <c r="D10" s="19"/>
@@ -5613,10 +5610,10 @@
         <v>276</v>
       </c>
       <c r="H2" t="s">
-        <v>960</v>
+        <v>946</v>
       </c>
       <c r="I2" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J2">
         <v>8</v>
@@ -5648,7 +5645,7 @@
         <v>276</v>
       </c>
       <c r="H3" t="s">
-        <v>962</v>
+        <v>948</v>
       </c>
       <c r="I3" t="s">
         <v>306</v>
@@ -5683,10 +5680,10 @@
         <v>276</v>
       </c>
       <c r="H4" t="s">
-        <v>963</v>
+        <v>949</v>
       </c>
       <c r="I4" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -5718,10 +5715,10 @@
         <v>276</v>
       </c>
       <c r="H5" t="s">
-        <v>964</v>
+        <v>950</v>
       </c>
       <c r="I5" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J5">
         <v>8</v>
@@ -5753,10 +5750,10 @@
         <v>276</v>
       </c>
       <c r="H6" t="s">
-        <v>965</v>
+        <v>951</v>
       </c>
       <c r="I6" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -5791,10 +5788,10 @@
         <v>276</v>
       </c>
       <c r="H7" t="s">
-        <v>966</v>
+        <v>952</v>
       </c>
       <c r="I7" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J7">
         <v>17</v>
@@ -5825,11 +5822,11 @@
       <c r="G8" t="s">
         <v>276</v>
       </c>
-      <c r="H8" s="20" t="s">
-        <v>967</v>
+      <c r="H8" s="17" t="s">
+        <v>953</v>
       </c>
       <c r="I8" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J8">
         <v>14</v>
@@ -5861,10 +5858,10 @@
         <v>276</v>
       </c>
       <c r="H9" t="s">
-        <v>968</v>
+        <v>954</v>
       </c>
       <c r="I9" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J9">
         <v>14</v>
@@ -5895,11 +5892,11 @@
       <c r="G10" t="s">
         <v>276</v>
       </c>
-      <c r="H10" s="20" t="s">
-        <v>969</v>
+      <c r="H10" s="17" t="s">
+        <v>955</v>
       </c>
       <c r="I10" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J10">
         <v>16</v>
@@ -5931,10 +5928,10 @@
         <v>276</v>
       </c>
       <c r="H11" t="s">
-        <v>970</v>
+        <v>956</v>
       </c>
       <c r="I11" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J11">
         <v>13</v>
@@ -5966,10 +5963,10 @@
         <v>276</v>
       </c>
       <c r="H12" t="s">
-        <v>971</v>
+        <v>957</v>
       </c>
       <c r="I12" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J12">
         <v>3</v>
@@ -5978,7 +5975,7 @@
         <v>286</v>
       </c>
       <c r="L12" t="s">
-        <v>972</v>
+        <v>958</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
@@ -6004,10 +6001,10 @@
         <v>276</v>
       </c>
       <c r="H13" t="s">
-        <v>973</v>
+        <v>959</v>
       </c>
       <c r="I13" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J13">
         <v>13</v>
@@ -6039,10 +6036,10 @@
         <v>276</v>
       </c>
       <c r="H14" t="s">
-        <v>974</v>
+        <v>960</v>
       </c>
       <c r="I14" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J14">
         <v>7</v>
@@ -6074,10 +6071,10 @@
         <v>276</v>
       </c>
       <c r="H15" t="s">
-        <v>975</v>
+        <v>961</v>
       </c>
       <c r="I15" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J15">
         <v>32</v>
@@ -6109,10 +6106,10 @@
         <v>276</v>
       </c>
       <c r="H16" t="s">
-        <v>976</v>
+        <v>962</v>
       </c>
       <c r="I16" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J16">
         <v>27</v>
@@ -6144,10 +6141,10 @@
         <v>276</v>
       </c>
       <c r="H17" t="s">
-        <v>977</v>
+        <v>963</v>
       </c>
       <c r="I17" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J17">
         <v>2</v>
@@ -6179,10 +6176,10 @@
         <v>276</v>
       </c>
       <c r="H18" t="s">
-        <v>978</v>
+        <v>964</v>
       </c>
       <c r="I18" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J18">
         <v>26</v>
@@ -6214,10 +6211,10 @@
         <v>276</v>
       </c>
       <c r="H19" t="s">
-        <v>979</v>
+        <v>965</v>
       </c>
       <c r="I19" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J19">
         <v>26</v>
@@ -6249,7 +6246,7 @@
         <v>276</v>
       </c>
       <c r="H20" t="s">
-        <v>980</v>
+        <v>966</v>
       </c>
       <c r="I20" t="s">
         <v>308</v>
@@ -6283,11 +6280,11 @@
       <c r="G21" t="s">
         <v>276</v>
       </c>
-      <c r="H21" s="20" t="s">
-        <v>981</v>
+      <c r="H21" s="17" t="s">
+        <v>967</v>
       </c>
       <c r="I21" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J21">
         <v>2</v>
@@ -6319,10 +6316,10 @@
         <v>276</v>
       </c>
       <c r="H22" t="s">
-        <v>982</v>
+        <v>968</v>
       </c>
       <c r="I22" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J22">
         <v>27</v>
@@ -6354,10 +6351,10 @@
         <v>276</v>
       </c>
       <c r="H23" t="s">
-        <v>983</v>
+        <v>969</v>
       </c>
       <c r="I23" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J23">
         <v>8</v>
@@ -6388,11 +6385,11 @@
       <c r="G24" t="s">
         <v>276</v>
       </c>
-      <c r="H24" s="20" t="s">
-        <v>984</v>
+      <c r="H24" s="17" t="s">
+        <v>970</v>
       </c>
       <c r="I24" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J24">
         <v>46</v>
@@ -6427,7 +6424,7 @@
         <v>319</v>
       </c>
       <c r="I25" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J25">
         <v>8</v>
@@ -6436,7 +6433,7 @@
         <v>286</v>
       </c>
       <c r="L25" t="s">
-        <v>985</v>
+        <v>971</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="129.6" x14ac:dyDescent="0.3">
@@ -6461,11 +6458,11 @@
       <c r="G26" t="s">
         <v>276</v>
       </c>
-      <c r="H26" s="20" t="s">
-        <v>986</v>
+      <c r="H26" s="17" t="s">
+        <v>972</v>
       </c>
       <c r="I26" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J26">
         <v>2</v>
@@ -6497,10 +6494,10 @@
         <v>276</v>
       </c>
       <c r="H27" t="s">
-        <v>987</v>
+        <v>973</v>
       </c>
       <c r="I27" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J27">
         <v>26</v>
@@ -6532,10 +6529,10 @@
         <v>276</v>
       </c>
       <c r="H28" t="s">
-        <v>988</v>
+        <v>974</v>
       </c>
       <c r="I28" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J28">
         <v>29</v>
@@ -6544,7 +6541,7 @@
         <v>286</v>
       </c>
       <c r="L28" t="s">
-        <v>989</v>
+        <v>975</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
@@ -6570,10 +6567,10 @@
         <v>276</v>
       </c>
       <c r="H29" t="s">
-        <v>990</v>
+        <v>976</v>
       </c>
       <c r="I29" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J29">
         <v>3</v>
@@ -6582,7 +6579,7 @@
         <v>286</v>
       </c>
       <c r="L29" t="s">
-        <v>989</v>
+        <v>975</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
@@ -6608,10 +6605,10 @@
         <v>276</v>
       </c>
       <c r="H30" t="s">
-        <v>991</v>
+        <v>977</v>
       </c>
       <c r="I30" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J30">
         <v>7</v>
@@ -6643,10 +6640,10 @@
         <v>276</v>
       </c>
       <c r="H31" t="s">
-        <v>992</v>
+        <v>978</v>
       </c>
       <c r="I31" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J31">
         <v>73</v>
@@ -6678,10 +6675,10 @@
         <v>276</v>
       </c>
       <c r="H32" t="s">
-        <v>993</v>
+        <v>979</v>
       </c>
       <c r="I32" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J32">
         <v>26</v>
@@ -6712,11 +6709,11 @@
       <c r="G33" t="s">
         <v>276</v>
       </c>
-      <c r="H33" s="20" t="s">
-        <v>994</v>
+      <c r="H33" s="17" t="s">
+        <v>980</v>
       </c>
       <c r="I33" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J33">
         <v>73</v>
@@ -6747,11 +6744,11 @@
       <c r="G34" t="s">
         <v>276</v>
       </c>
-      <c r="H34" s="20" t="s">
-        <v>995</v>
+      <c r="H34" s="17" t="s">
+        <v>981</v>
       </c>
       <c r="I34" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J34">
         <v>78</v>
@@ -6783,10 +6780,10 @@
         <v>276</v>
       </c>
       <c r="H35" t="s">
-        <v>996</v>
+        <v>982</v>
       </c>
       <c r="I35" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J35">
         <v>34</v>
@@ -6818,10 +6815,10 @@
         <v>276</v>
       </c>
       <c r="H36" t="s">
-        <v>997</v>
+        <v>983</v>
       </c>
       <c r="I36" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J36">
         <v>73</v>
@@ -6853,10 +6850,10 @@
         <v>276</v>
       </c>
       <c r="H37" t="s">
-        <v>998</v>
+        <v>984</v>
       </c>
       <c r="I37" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J37">
         <v>75</v>
@@ -6865,7 +6862,7 @@
         <v>286</v>
       </c>
       <c r="L37" t="s">
-        <v>924</v>
+        <v>914</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
@@ -6891,10 +6888,10 @@
         <v>276</v>
       </c>
       <c r="H38" t="s">
-        <v>999</v>
+        <v>985</v>
       </c>
       <c r="I38" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J38">
         <v>80</v>
@@ -6926,10 +6923,10 @@
         <v>276</v>
       </c>
       <c r="H39" t="s">
-        <v>1000</v>
+        <v>986</v>
       </c>
       <c r="I39" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J39">
         <v>75</v>
@@ -6961,10 +6958,10 @@
         <v>276</v>
       </c>
       <c r="H40" t="s">
-        <v>1001</v>
+        <v>987</v>
       </c>
       <c r="I40" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J40">
         <v>88</v>
@@ -6996,10 +6993,10 @@
         <v>276</v>
       </c>
       <c r="H41" t="s">
-        <v>1002</v>
+        <v>988</v>
       </c>
       <c r="I41" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J41">
         <v>75</v>
@@ -7031,10 +7028,10 @@
         <v>276</v>
       </c>
       <c r="H42" t="s">
-        <v>1003</v>
+        <v>989</v>
       </c>
       <c r="I42" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J42">
         <v>5</v>
@@ -7065,11 +7062,11 @@
       <c r="G43" t="s">
         <v>276</v>
       </c>
-      <c r="H43" s="20" t="s">
-        <v>1004</v>
+      <c r="H43" s="17" t="s">
+        <v>990</v>
       </c>
       <c r="I43" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J43">
         <v>3</v>
@@ -7101,10 +7098,10 @@
         <v>276</v>
       </c>
       <c r="H44" t="s">
-        <v>1005</v>
+        <v>991</v>
       </c>
       <c r="I44" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J44">
         <v>2</v>
@@ -7136,7 +7133,7 @@
         <v>276</v>
       </c>
       <c r="H45" t="s">
-        <v>1006</v>
+        <v>992</v>
       </c>
       <c r="I45" t="s">
         <v>308</v>
@@ -7171,10 +7168,10 @@
         <v>276</v>
       </c>
       <c r="H46" t="s">
-        <v>1007</v>
+        <v>993</v>
       </c>
       <c r="I46" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J46">
         <v>28</v>
@@ -7206,10 +7203,10 @@
         <v>276</v>
       </c>
       <c r="H47" t="s">
-        <v>1008</v>
+        <v>994</v>
       </c>
       <c r="I47" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J47">
         <v>9</v>
@@ -7218,7 +7215,7 @@
         <v>286</v>
       </c>
       <c r="L47" t="s">
-        <v>1009</v>
+        <v>995</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
@@ -7244,10 +7241,10 @@
         <v>276</v>
       </c>
       <c r="H48" t="s">
-        <v>1010</v>
+        <v>996</v>
       </c>
       <c r="I48" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J48">
         <v>3</v>
@@ -7279,10 +7276,10 @@
         <v>276</v>
       </c>
       <c r="H49" t="s">
-        <v>1011</v>
+        <v>997</v>
       </c>
       <c r="I49" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J49">
         <v>107</v>
@@ -7314,10 +7311,10 @@
         <v>276</v>
       </c>
       <c r="H50" t="s">
-        <v>1012</v>
+        <v>998</v>
       </c>
       <c r="I50" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J50">
         <v>5</v>
@@ -7349,10 +7346,10 @@
         <v>276</v>
       </c>
       <c r="H51" t="s">
-        <v>1013</v>
+        <v>999</v>
       </c>
       <c r="I51" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
       <c r="J51">
         <v>8</v>
@@ -7363,18 +7360,18 @@
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52" s="11" t="s">
-        <v>1014</v>
+        <v>1008</v>
       </c>
       <c r="K52" s="15" t="s">
-        <v>1015</v>
+        <v>1000</v>
       </c>
       <c r="L52" s="16" t="s">
-        <v>1016</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B53" s="18" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="C53" s="19"/>
       <c r="D53" s="19"/>
@@ -7618,19 +7615,19 @@
       <c r="A8" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="20" t="s">
         <v>304</v>
       </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="20"/>
+      <c r="L8" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -10276,10 +10273,10 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
+        <v>1002</v>
+      </c>
+      <c r="K7" s="15" t="s">
         <v>854</v>
-      </c>
-      <c r="K7" s="15" t="s">
-        <v>855</v>
       </c>
       <c r="L7" s="16" t="s">
         <v>401</v>
@@ -10287,7 +10284,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B8" s="18" t="s">
-        <v>856</v>
+        <v>1009</v>
       </c>
       <c r="C8" s="19"/>
       <c r="D8" s="19"/>
@@ -10388,10 +10385,10 @@
         <v>276</v>
       </c>
       <c r="H2" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="I2" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="J2">
         <v>166</v>
@@ -10422,11 +10419,11 @@
       <c r="G3" t="s">
         <v>276</v>
       </c>
-      <c r="H3" s="20" t="s">
-        <v>859</v>
+      <c r="H3" s="17" t="s">
+        <v>857</v>
       </c>
       <c r="I3" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -10458,10 +10455,10 @@
         <v>276</v>
       </c>
       <c r="H4" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
       <c r="I4" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -10492,11 +10489,11 @@
       <c r="G5" t="s">
         <v>276</v>
       </c>
-      <c r="H5" s="20" t="s">
-        <v>862</v>
+      <c r="H5" s="17" t="s">
+        <v>860</v>
       </c>
       <c r="I5" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -10528,10 +10525,10 @@
         <v>276</v>
       </c>
       <c r="H6" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="I6" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="J6">
         <v>164</v>
@@ -10540,7 +10537,7 @@
         <v>286</v>
       </c>
       <c r="L6" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -10566,10 +10563,10 @@
         <v>276</v>
       </c>
       <c r="H7" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="I7" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="J7">
         <v>8</v>
@@ -10600,8 +10597,8 @@
       <c r="G8" t="s">
         <v>276</v>
       </c>
-      <c r="H8" s="20" t="s">
-        <v>866</v>
+      <c r="H8" s="17" t="s">
+        <v>864</v>
       </c>
       <c r="I8" t="s">
         <v>297</v>
@@ -10636,10 +10633,10 @@
         <v>276</v>
       </c>
       <c r="H9" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="I9" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="J9">
         <v>365</v>
@@ -10671,10 +10668,10 @@
         <v>276</v>
       </c>
       <c r="H10" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="I10" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="J10">
         <v>4</v>
@@ -10705,11 +10702,11 @@
       <c r="G11" t="s">
         <v>276</v>
       </c>
-      <c r="H11" s="20" t="s">
-        <v>869</v>
+      <c r="H11" s="17" t="s">
+        <v>867</v>
       </c>
       <c r="I11" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="J11">
         <v>66</v>
@@ -10720,10 +10717,10 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>870</v>
+        <v>1003</v>
       </c>
       <c r="K12" s="15" t="s">
-        <v>871</v>
+        <v>868</v>
       </c>
       <c r="L12" s="16" t="s">
         <v>401</v>
@@ -10731,7 +10728,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B13" s="18" t="s">
-        <v>872</v>
+        <v>1010</v>
       </c>
       <c r="C13" s="19"/>
       <c r="D13" s="19"/>
@@ -10832,10 +10829,10 @@
         <v>276</v>
       </c>
       <c r="H2" t="s">
-        <v>873</v>
+        <v>869</v>
       </c>
       <c r="I2" t="s">
-        <v>874</v>
+        <v>870</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -10867,10 +10864,10 @@
         <v>276</v>
       </c>
       <c r="H3" t="s">
-        <v>875</v>
+        <v>871</v>
       </c>
       <c r="I3" t="s">
-        <v>874</v>
+        <v>870</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -10902,10 +10899,10 @@
         <v>276</v>
       </c>
       <c r="H4" t="s">
-        <v>876</v>
+        <v>872</v>
       </c>
       <c r="I4" t="s">
-        <v>874</v>
+        <v>870</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -10936,11 +10933,11 @@
       <c r="G5" t="s">
         <v>276</v>
       </c>
-      <c r="H5" s="20" t="s">
-        <v>877</v>
+      <c r="H5" s="17" t="s">
+        <v>873</v>
       </c>
       <c r="I5" t="s">
-        <v>874</v>
+        <v>870</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -10972,10 +10969,10 @@
         <v>276</v>
       </c>
       <c r="H6" t="s">
-        <v>878</v>
+        <v>874</v>
       </c>
       <c r="I6" t="s">
-        <v>874</v>
+        <v>870</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -11007,10 +11004,10 @@
         <v>276</v>
       </c>
       <c r="H7" t="s">
-        <v>879</v>
+        <v>875</v>
       </c>
       <c r="I7" t="s">
-        <v>874</v>
+        <v>870</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -11021,18 +11018,18 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>880</v>
+        <v>1004</v>
       </c>
       <c r="K8" s="15" t="s">
-        <v>881</v>
+        <v>876</v>
       </c>
       <c r="L8" s="16" t="s">
-        <v>882</v>
+        <v>877</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B9" s="18" t="s">
-        <v>883</v>
+        <v>1011</v>
       </c>
       <c r="C9" s="19"/>
       <c r="D9" s="19"/>
@@ -11133,7 +11130,7 @@
         <v>276</v>
       </c>
       <c r="H2" t="s">
-        <v>884</v>
+        <v>878</v>
       </c>
       <c r="I2" t="s">
         <v>366</v>
@@ -11168,7 +11165,7 @@
         <v>276</v>
       </c>
       <c r="H3" t="s">
-        <v>885</v>
+        <v>879</v>
       </c>
       <c r="I3" t="s">
         <v>366</v>
@@ -11203,7 +11200,7 @@
         <v>276</v>
       </c>
       <c r="H4" t="s">
-        <v>886</v>
+        <v>880</v>
       </c>
       <c r="I4" t="s">
         <v>366</v>
@@ -11238,7 +11235,7 @@
         <v>276</v>
       </c>
       <c r="H5" t="s">
-        <v>887</v>
+        <v>881</v>
       </c>
       <c r="I5" t="s">
         <v>306</v>
@@ -11273,7 +11270,7 @@
         <v>276</v>
       </c>
       <c r="H6" t="s">
-        <v>888</v>
+        <v>882</v>
       </c>
       <c r="I6" t="s">
         <v>306</v>
@@ -11308,7 +11305,7 @@
         <v>276</v>
       </c>
       <c r="H7" t="s">
-        <v>889</v>
+        <v>883</v>
       </c>
       <c r="I7" t="s">
         <v>306</v>
@@ -11343,7 +11340,7 @@
         <v>276</v>
       </c>
       <c r="H8" t="s">
-        <v>890</v>
+        <v>884</v>
       </c>
       <c r="I8" t="s">
         <v>366</v>
@@ -11378,7 +11375,7 @@
         <v>276</v>
       </c>
       <c r="H9" t="s">
-        <v>891</v>
+        <v>885</v>
       </c>
       <c r="I9" t="s">
         <v>306</v>
@@ -11390,7 +11387,7 @@
         <v>286</v>
       </c>
       <c r="L9" t="s">
-        <v>892</v>
+        <v>886</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
@@ -11416,7 +11413,7 @@
         <v>276</v>
       </c>
       <c r="H10" t="s">
-        <v>893</v>
+        <v>887</v>
       </c>
       <c r="I10" t="s">
         <v>366</v>
@@ -11450,8 +11447,8 @@
       <c r="G11" t="s">
         <v>276</v>
       </c>
-      <c r="H11" s="20" t="s">
-        <v>894</v>
+      <c r="H11" s="17" t="s">
+        <v>888</v>
       </c>
       <c r="I11" t="s">
         <v>306</v>
@@ -11485,8 +11482,8 @@
       <c r="G12" t="s">
         <v>276</v>
       </c>
-      <c r="H12" s="20" t="s">
-        <v>895</v>
+      <c r="H12" s="17" t="s">
+        <v>889</v>
       </c>
       <c r="I12" t="s">
         <v>306</v>
@@ -11521,7 +11518,7 @@
         <v>276</v>
       </c>
       <c r="H13" t="s">
-        <v>896</v>
+        <v>890</v>
       </c>
       <c r="I13" t="s">
         <v>306</v>
@@ -11535,10 +11532,10 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
-        <v>897</v>
+        <v>1005</v>
       </c>
       <c r="K14" s="15" t="s">
-        <v>898</v>
+        <v>891</v>
       </c>
       <c r="L14" s="16" t="s">
         <v>401</v>
@@ -11546,7 +11543,7 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B15" s="18" t="s">
-        <v>899</v>
+        <v>1012</v>
       </c>
       <c r="C15" s="19"/>
       <c r="D15" s="19"/>
@@ -11647,7 +11644,7 @@
         <v>276</v>
       </c>
       <c r="H2" t="s">
-        <v>900</v>
+        <v>892</v>
       </c>
       <c r="I2" t="s">
         <v>308</v>
@@ -11682,10 +11679,10 @@
         <v>276</v>
       </c>
       <c r="H3" t="s">
-        <v>901</v>
+        <v>893</v>
       </c>
       <c r="I3" t="s">
-        <v>902</v>
+        <v>894</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -11717,10 +11714,10 @@
         <v>276</v>
       </c>
       <c r="H4" t="s">
-        <v>903</v>
+        <v>895</v>
       </c>
       <c r="I4" t="s">
-        <v>904</v>
+        <v>896</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -11752,7 +11749,7 @@
         <v>276</v>
       </c>
       <c r="H5" t="s">
-        <v>905</v>
+        <v>897</v>
       </c>
       <c r="I5" t="s">
         <v>308</v>
@@ -11787,10 +11784,10 @@
         <v>276</v>
       </c>
       <c r="H6" t="s">
-        <v>906</v>
+        <v>898</v>
       </c>
       <c r="I6" t="s">
-        <v>902</v>
+        <v>894</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -11799,15 +11796,15 @@
         <v>286</v>
       </c>
       <c r="L6" t="s">
-        <v>907</v>
+        <v>899</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
+        <v>1002</v>
+      </c>
+      <c r="K7" s="15" t="s">
         <v>854</v>
-      </c>
-      <c r="K7" s="15" t="s">
-        <v>855</v>
       </c>
       <c r="L7" s="16" t="s">
         <v>401</v>
@@ -11815,7 +11812,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B8" s="18" t="s">
-        <v>856</v>
+        <v>1009</v>
       </c>
       <c r="C8" s="19"/>
       <c r="D8" s="19"/>

</xml_diff>